<commit_message>
Format 70_94_109.xlsx with canonical 3-tier hierarchical headers
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/70_94_109.xlsx
+++ b/03_Coding_Sheets/70_94_109.xlsx
@@ -422,11 +422,6 @@
           <t>Coder Initials</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Article ID</t>
-        </is>
-      </c>
       <c r="C1" t="inlineStr">
         <is>
           <t>Sample ID</t>
@@ -453,456 +448,263 @@
           <t>Article Descriptors</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Unnamed: 7</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Unnamed: 8</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Unnamed: 9</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Unnamed: 10</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Unnamed: 11</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Unnamed: 12</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Unnamed: 13</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Unnamed: 14</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Unnamed: 15</t>
-        </is>
-      </c>
       <c r="Q1" t="inlineStr">
         <is>
           <t>Study/Sample Descriptors</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Unnamed: 17</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Unnamed: 18</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>Unnamed: 19</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Unnamed: 20</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>Unnamed: 21</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>Unnamed: 22</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>Unnamed: 23</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>Unnamed: 24</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>Unnamed: 25</t>
-        </is>
-      </c>
       <c r="AA1" t="inlineStr">
         <is>
           <t>Measure Descriptors</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>Unnamed: 27</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>Unnamed: 28</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>Unnamed: 29</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>Unnamed: 30</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>Unnamed: 31</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>Unnamed: 32</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>Unnamed: 33</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>Unnamed: 34</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>Unnamed: 35</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>Unnamed: 36</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>Unnamed: 37</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>Unnamed: 38</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>Unnamed: 39</t>
-        </is>
-      </c>
       <c r="AO1" t="inlineStr">
         <is>
           <t>Effect Size</t>
-        </is>
-      </c>
-      <c r="AP1" t="inlineStr">
-        <is>
-          <t>Unnamed: 41</t>
-        </is>
-      </c>
-      <c r="AQ1" t="inlineStr">
-        <is>
-          <t>Unnamed: 42</t>
-        </is>
-      </c>
-      <c r="AR1" t="inlineStr">
-        <is>
-          <t>Unnamed: 43</t>
-        </is>
-      </c>
-      <c r="AS1" t="inlineStr">
-        <is>
-          <t>Unnamed: 44</t>
-        </is>
-      </c>
-      <c r="AT1" t="inlineStr">
-        <is>
-          <t>Unnamed: 45</t>
-        </is>
-      </c>
-      <c r="AU1" t="inlineStr">
-        <is>
-          <t>Unnamed: 46</t>
-        </is>
-      </c>
-      <c r="AV1" t="inlineStr">
-        <is>
-          <t>Unnamed: 47</t>
-        </is>
-      </c>
-      <c r="AW1" t="inlineStr">
-        <is>
-          <t>Unnamed: 48</t>
-        </is>
-      </c>
-      <c r="AX1" t="inlineStr">
-        <is>
-          <t>Unnamed: 49</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" t="n">
-        <v>608</v>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Boundary spanning</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>Non-boundary-spanning variable</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>Boundary spanning-related variable</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>Non-boundary-spanning variable</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>Correlation r</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>BSMA0052</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level (team/firm/org analysis)</t>
-        </is>
-      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>This study examined how leaders’ internal and external activities mediate the relationship of functional heterogeneity and interteam goal interdependence to team effectiveness (in-role performance and innovation) in interdisciplinary teams. The results of the structural equation model from a sample of 92 interdisciplinary teams indicate that leaders’ internal activities fully mediate the relationship of team functional heterogeneity and interteam goal interdependence to team in-role performance. The leaders’ external activities were found to fully mediate the relationship of interteam goal interdependence to team innovation. We discuss the implications of these findings for both theory and practice.</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>The Role of Leader Boundary Activities in Enhancing Interdisciplinary Team Effectiveness</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Small Group Research</t>
+          <t>Publication Name</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Benoliel, Pascale; Somech, Anit</t>
+          <t>Authors</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Publication Type</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Other (specify)</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Full Citation (APA Style)</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Secondary Data? (If yes, provide reference to the original paper)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Quantitative. The study analyzes leader boundary spanning behavior aggregated at the team level (N=92 teams), violating the individual-level analysis requirement. Verbatim Evidence: "Data were collected from 92 management teams from 92 public educational organizations in Israel." AND "In the research hypotheses, the team is identified as the unit of analysis. ... Interteam goal interdependence and leader internal and external activities were represented by an aggregate of team member responses." AND "Prior to aggregating individual-level scores to the group level by mean, intraclass correlations (ICC) were calculated."</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Study Design</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Other (specify)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Country</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Country (specify)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>International Context</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Sample size (N)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Mean Age</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>% Female</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Org Tenure</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Occupation Type</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>Boundary spanning</t>
+          <t>Number of Items</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Min Score</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Max Score</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Report Type</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Report Type Note (if necessary)</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Specific Measure Used</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>Non-boundary-spanning variable</t>
+          <t>Number of Items</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Min Score</t>
         </is>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Max Score</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Report Type</t>
         </is>
       </c>
       <c r="AL3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Report Type Note (if necessary)</t>
         </is>
       </c>
       <c r="AM3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Specific Measure Used</t>
         </is>
       </c>
       <c r="AN3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="AO3" t="inlineStr">
         <is>
-          <t>Boundary spanning-related variable</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="AP3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Mean</t>
         </is>
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="AR3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Reliability (Alpha)</t>
         </is>
       </c>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>Non-boundary-spanning variable</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="AT3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>Mean</t>
         </is>
       </c>
       <c r="AU3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
-      <c r="AW3" t="inlineStr">
-        <is>
-          <t>Correlation r</t>
-        </is>
-      </c>
-      <c r="AX3" t="inlineStr">
-        <is>
-          <t>Notes</t>
+          <t>Reliability (Alpha)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Rule 14: Prune table layout numbering from variable names while preserving construct names
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/70_94_109.xlsx
+++ b/03_Coding_Sheets/70_94_109.xlsx
@@ -881,7 +881,7 @@
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>1. BSA</t>
+          <t>BSA</t>
         </is>
       </c>
       <c r="AP4" t="n">
@@ -895,7 +895,7 @@
       </c>
       <c r="AS4" t="inlineStr">
         <is>
-          <t>7. Status</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="AT4" t="n">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="AO5" t="inlineStr">
         <is>
-          <t>1. BSA</t>
+          <t>BSA</t>
         </is>
       </c>
       <c r="AP5" t="n">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="AS5" t="inlineStr">
         <is>
-          <t>8. Org. Size</t>
+          <t>Org. Size</t>
         </is>
       </c>
       <c r="AT5" t="n">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="AO6" t="inlineStr">
         <is>
-          <t>1. BSA</t>
+          <t>BSA</t>
         </is>
       </c>
       <c r="AP6" t="n">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="AS6" t="inlineStr">
         <is>
-          <t>9. Industry</t>
+          <t>Industry</t>
         </is>
       </c>
       <c r="AT6" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="AO7" t="inlineStr">
         <is>
-          <t>1. BSA</t>
+          <t>BSA</t>
         </is>
       </c>
       <c r="AP7" t="n">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="AS7" t="inlineStr">
         <is>
-          <t>10. Org. Comm.</t>
+          <t>Org. Comm.</t>
         </is>
       </c>
       <c r="AT7" t="n">
@@ -1713,7 +1713,7 @@
       </c>
       <c r="AO8" t="inlineStr">
         <is>
-          <t>1. BSA</t>
+          <t>BSA</t>
         </is>
       </c>
       <c r="AP8" t="n">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="AS8" t="inlineStr">
         <is>
-          <t>11. Prof. Comm.</t>
+          <t>Prof. Comm.</t>
         </is>
       </c>
       <c r="AT8" t="n">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="AO9" t="inlineStr">
         <is>
-          <t>1. BSA</t>
+          <t>BSA</t>
         </is>
       </c>
       <c r="AP9" t="n">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="AS9" t="inlineStr">
         <is>
-          <t>12. Dual Comm.</t>
+          <t>Dual Comm.</t>
         </is>
       </c>
       <c r="AT9" t="n">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="AO10" t="inlineStr">
         <is>
-          <t>1. BSA</t>
+          <t>BSA</t>
         </is>
       </c>
       <c r="AP10" t="n">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="AS10" t="inlineStr">
         <is>
-          <t>13. Complexity</t>
+          <t>Complexity</t>
         </is>
       </c>
       <c r="AT10" t="n">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="AO11" t="inlineStr">
         <is>
-          <t>1. BSA</t>
+          <t>BSA</t>
         </is>
       </c>
       <c r="AP11" t="n">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="AS11" t="inlineStr">
         <is>
-          <t>14. Uncertainty</t>
+          <t>Uncertainty</t>
         </is>
       </c>
       <c r="AT11" t="n">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="AO12" t="inlineStr">
         <is>
-          <t>1. BSA</t>
+          <t>BSA</t>
         </is>
       </c>
       <c r="AP12" t="n">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="AS12" t="inlineStr">
         <is>
-          <t>15. Interdepend.</t>
+          <t>Interdepend.</t>
         </is>
       </c>
       <c r="AT12" t="n">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="AO13" t="inlineStr">
         <is>
-          <t>1. BSA</t>
+          <t>BSA</t>
         </is>
       </c>
       <c r="AP13" t="n">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="AS13" t="inlineStr">
         <is>
-          <t>16. Degree</t>
+          <t>Degree</t>
         </is>
       </c>
       <c r="AT13" t="n">
@@ -2961,7 +2961,7 @@
       </c>
       <c r="AO14" t="inlineStr">
         <is>
-          <t>1. BSA</t>
+          <t>BSA</t>
         </is>
       </c>
       <c r="AP14" t="n">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="AS14" t="inlineStr">
         <is>
-          <t>17. Occupation</t>
+          <t>Occupation</t>
         </is>
       </c>
       <c r="AT14" t="n">
@@ -3169,7 +3169,7 @@
       </c>
       <c r="AO15" t="inlineStr">
         <is>
-          <t>1. BSA</t>
+          <t>BSA</t>
         </is>
       </c>
       <c r="AP15" t="n">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="AS15" t="inlineStr">
         <is>
-          <t>18. Prof. Control</t>
+          <t>Prof. Control</t>
         </is>
       </c>
       <c r="AT15" t="n">
@@ -3377,7 +3377,7 @@
       </c>
       <c r="AO16" t="inlineStr">
         <is>
-          <t>1. BSA</t>
+          <t>BSA</t>
         </is>
       </c>
       <c r="AP16" t="n">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="AS16" t="inlineStr">
         <is>
-          <t>19. Prof. Incent.</t>
+          <t>Prof. Incent.</t>
         </is>
       </c>
       <c r="AT16" t="n">
@@ -3585,7 +3585,7 @@
       </c>
       <c r="AO17" t="inlineStr">
         <is>
-          <t>3. External Com.</t>
+          <t>External Com.</t>
         </is>
       </c>
       <c r="AP17" t="n">
@@ -3599,7 +3599,7 @@
       </c>
       <c r="AS17" t="inlineStr">
         <is>
-          <t>2. Internal Com.</t>
+          <t>Internal Com.</t>
         </is>
       </c>
       <c r="AT17" t="n">
@@ -3793,7 +3793,7 @@
       </c>
       <c r="AO18" t="inlineStr">
         <is>
-          <t>3. External Com.</t>
+          <t>External Com.</t>
         </is>
       </c>
       <c r="AP18" t="n">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="AS18" t="inlineStr">
         <is>
-          <t>7. Status</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="AT18" t="n">
@@ -4001,7 +4001,7 @@
       </c>
       <c r="AO19" t="inlineStr">
         <is>
-          <t>3. External Com.</t>
+          <t>External Com.</t>
         </is>
       </c>
       <c r="AP19" t="n">
@@ -4015,7 +4015,7 @@
       </c>
       <c r="AS19" t="inlineStr">
         <is>
-          <t>8. Org. Size</t>
+          <t>Org. Size</t>
         </is>
       </c>
       <c r="AT19" t="n">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="AO20" t="inlineStr">
         <is>
-          <t>3. External Com.</t>
+          <t>External Com.</t>
         </is>
       </c>
       <c r="AP20" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="AS20" t="inlineStr">
         <is>
-          <t>9. Industry</t>
+          <t>Industry</t>
         </is>
       </c>
       <c r="AT20" t="n">
@@ -4417,7 +4417,7 @@
       </c>
       <c r="AO21" t="inlineStr">
         <is>
-          <t>3. External Com.</t>
+          <t>External Com.</t>
         </is>
       </c>
       <c r="AP21" t="n">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="AS21" t="inlineStr">
         <is>
-          <t>10. Org. Comm.</t>
+          <t>Org. Comm.</t>
         </is>
       </c>
       <c r="AT21" t="n">
@@ -4625,7 +4625,7 @@
       </c>
       <c r="AO22" t="inlineStr">
         <is>
-          <t>3. External Com.</t>
+          <t>External Com.</t>
         </is>
       </c>
       <c r="AP22" t="n">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="AS22" t="inlineStr">
         <is>
-          <t>11. Prof. Comm.</t>
+          <t>Prof. Comm.</t>
         </is>
       </c>
       <c r="AT22" t="n">
@@ -4833,7 +4833,7 @@
       </c>
       <c r="AO23" t="inlineStr">
         <is>
-          <t>3. External Com.</t>
+          <t>External Com.</t>
         </is>
       </c>
       <c r="AP23" t="n">
@@ -4847,7 +4847,7 @@
       </c>
       <c r="AS23" t="inlineStr">
         <is>
-          <t>12. Dual Comm.</t>
+          <t>Dual Comm.</t>
         </is>
       </c>
       <c r="AT23" t="n">
@@ -5041,7 +5041,7 @@
       </c>
       <c r="AO24" t="inlineStr">
         <is>
-          <t>3. External Com.</t>
+          <t>External Com.</t>
         </is>
       </c>
       <c r="AP24" t="n">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="AS24" t="inlineStr">
         <is>
-          <t>13. Complexity</t>
+          <t>Complexity</t>
         </is>
       </c>
       <c r="AT24" t="n">
@@ -5249,7 +5249,7 @@
       </c>
       <c r="AO25" t="inlineStr">
         <is>
-          <t>3. External Com.</t>
+          <t>External Com.</t>
         </is>
       </c>
       <c r="AP25" t="n">
@@ -5263,7 +5263,7 @@
       </c>
       <c r="AS25" t="inlineStr">
         <is>
-          <t>14. Uncertainty</t>
+          <t>Uncertainty</t>
         </is>
       </c>
       <c r="AT25" t="n">
@@ -5457,7 +5457,7 @@
       </c>
       <c r="AO26" t="inlineStr">
         <is>
-          <t>3. External Com.</t>
+          <t>External Com.</t>
         </is>
       </c>
       <c r="AP26" t="n">
@@ -5471,7 +5471,7 @@
       </c>
       <c r="AS26" t="inlineStr">
         <is>
-          <t>15. Interdepend.</t>
+          <t>Interdepend.</t>
         </is>
       </c>
       <c r="AT26" t="n">
@@ -5665,7 +5665,7 @@
       </c>
       <c r="AO27" t="inlineStr">
         <is>
-          <t>3. External Com.</t>
+          <t>External Com.</t>
         </is>
       </c>
       <c r="AP27" t="n">
@@ -5679,7 +5679,7 @@
       </c>
       <c r="AS27" t="inlineStr">
         <is>
-          <t>16. Degree</t>
+          <t>Degree</t>
         </is>
       </c>
       <c r="AT27" t="n">
@@ -5873,7 +5873,7 @@
       </c>
       <c r="AO28" t="inlineStr">
         <is>
-          <t>3. External Com.</t>
+          <t>External Com.</t>
         </is>
       </c>
       <c r="AP28" t="n">
@@ -5887,7 +5887,7 @@
       </c>
       <c r="AS28" t="inlineStr">
         <is>
-          <t>17. Occupation</t>
+          <t>Occupation</t>
         </is>
       </c>
       <c r="AT28" t="n">
@@ -6081,7 +6081,7 @@
       </c>
       <c r="AO29" t="inlineStr">
         <is>
-          <t>3. External Com.</t>
+          <t>External Com.</t>
         </is>
       </c>
       <c r="AP29" t="n">
@@ -6095,7 +6095,7 @@
       </c>
       <c r="AS29" t="inlineStr">
         <is>
-          <t>18. Prof. Control</t>
+          <t>Prof. Control</t>
         </is>
       </c>
       <c r="AT29" t="n">
@@ -6289,7 +6289,7 @@
       </c>
       <c r="AO30" t="inlineStr">
         <is>
-          <t>3. External Com.</t>
+          <t>External Com.</t>
         </is>
       </c>
       <c r="AP30" t="n">
@@ -6303,7 +6303,7 @@
       </c>
       <c r="AS30" t="inlineStr">
         <is>
-          <t>19. Prof. Incent.</t>
+          <t>Prof. Incent.</t>
         </is>
       </c>
       <c r="AT30" t="n">

</xml_diff>

<commit_message>
Standardize Rule 1 Clean Blank Cell Protocol across rules, skills, and 70_94_109.xlsx
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/70_94_109.xlsx
+++ b/03_Coding_Sheets/70_94_109.xlsx
@@ -728,9 +728,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>999</v>
-      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -759,11 +756,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N4" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -774,29 +766,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q4" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S4" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -807,22 +784,10 @@
       <c r="V4" t="n">
         <v>253</v>
       </c>
-      <c r="W4" t="n">
-        <v>999</v>
-      </c>
-      <c r="X4" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>999</v>
-      </c>
       <c r="Z4" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
-      </c>
-      <c r="AA4" t="n">
-        <v>999</v>
       </c>
       <c r="AB4" t="n">
         <v>7.5</v>
@@ -835,11 +800,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF4" t="inlineStr">
         <is>
           <t>boundary spanning score</t>
@@ -864,11 +824,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL4" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM4" t="inlineStr">
         <is>
           <t>job title</t>
@@ -884,28 +839,10 @@
           <t>BSA</t>
         </is>
       </c>
-      <c r="AP4" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ4" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR4" t="n">
-        <v>999</v>
-      </c>
       <c r="AS4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
-      </c>
-      <c r="AT4" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU4" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV4" t="n">
-        <v>999</v>
       </c>
       <c r="AW4" t="n">
         <v>0.05</v>
@@ -936,9 +873,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>999</v>
-      </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -967,11 +901,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N5" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -982,29 +911,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q5" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S5" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1015,22 +929,10 @@
       <c r="V5" t="n">
         <v>253</v>
       </c>
-      <c r="W5" t="n">
-        <v>999</v>
-      </c>
-      <c r="X5" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>999</v>
-      </c>
       <c r="Z5" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
-      </c>
-      <c r="AA5" t="n">
-        <v>999</v>
       </c>
       <c r="AB5" t="n">
         <v>7.5</v>
@@ -1043,11 +945,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF5" t="inlineStr">
         <is>
           <t>boundary spanning score</t>
@@ -1072,11 +969,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL5" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM5" t="inlineStr">
         <is>
           <t>Organizational size</t>
@@ -1092,28 +984,10 @@
           <t>BSA</t>
         </is>
       </c>
-      <c r="AP5" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ5" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR5" t="n">
-        <v>999</v>
-      </c>
       <c r="AS5" t="inlineStr">
         <is>
           <t>Org. Size</t>
         </is>
-      </c>
-      <c r="AT5" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU5" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV5" t="n">
-        <v>999</v>
       </c>
       <c r="AW5" t="n">
         <v>0.03</v>
@@ -1144,9 +1018,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>999</v>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -1175,11 +1046,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N6" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -1190,29 +1056,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q6" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S6" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1223,22 +1074,10 @@
       <c r="V6" t="n">
         <v>253</v>
       </c>
-      <c r="W6" t="n">
-        <v>999</v>
-      </c>
-      <c r="X6" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>999</v>
-      </c>
       <c r="Z6" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
-      </c>
-      <c r="AA6" t="n">
-        <v>999</v>
       </c>
       <c r="AB6" t="n">
         <v>7.5</v>
@@ -1251,11 +1090,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE6" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF6" t="inlineStr">
         <is>
           <t>boundary spanning score</t>
@@ -1280,11 +1114,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL6" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM6" t="inlineStr">
         <is>
           <t>dichotomous variable</t>
@@ -1300,28 +1129,10 @@
           <t>BSA</t>
         </is>
       </c>
-      <c r="AP6" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ6" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR6" t="n">
-        <v>999</v>
-      </c>
       <c r="AS6" t="inlineStr">
         <is>
           <t>Industry</t>
         </is>
-      </c>
-      <c r="AT6" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU6" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV6" t="n">
-        <v>999</v>
       </c>
       <c r="AW6" t="n">
         <v>0.02</v>
@@ -1352,9 +1163,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>999</v>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -1383,11 +1191,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N7" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -1398,29 +1201,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q7" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S7" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1431,22 +1219,10 @@
       <c r="V7" t="n">
         <v>253</v>
       </c>
-      <c r="W7" t="n">
-        <v>999</v>
-      </c>
-      <c r="X7" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>999</v>
-      </c>
       <c r="Z7" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
-      </c>
-      <c r="AA7" t="n">
-        <v>999</v>
       </c>
       <c r="AB7" t="n">
         <v>7.5</v>
@@ -1459,11 +1235,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE7" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF7" t="inlineStr">
         <is>
           <t>boundary spanning score</t>
@@ -1488,11 +1259,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL7" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM7" t="inlineStr">
         <is>
           <t>Organizational Commitment Questionnaire</t>
@@ -1508,25 +1274,10 @@
           <t>BSA</t>
         </is>
       </c>
-      <c r="AP7" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ7" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR7" t="n">
-        <v>999</v>
-      </c>
       <c r="AS7" t="inlineStr">
         <is>
           <t>Org. Comm.</t>
         </is>
-      </c>
-      <c r="AT7" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU7" t="n">
-        <v>999</v>
       </c>
       <c r="AV7" t="n">
         <v>0.92</v>
@@ -1560,9 +1311,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>999</v>
-      </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -1591,11 +1339,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N8" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -1606,29 +1349,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q8" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S8" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1639,22 +1367,10 @@
       <c r="V8" t="n">
         <v>253</v>
       </c>
-      <c r="W8" t="n">
-        <v>999</v>
-      </c>
-      <c r="X8" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>999</v>
-      </c>
       <c r="Z8" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
-      </c>
-      <c r="AA8" t="n">
-        <v>999</v>
       </c>
       <c r="AB8" t="n">
         <v>7.5</v>
@@ -1667,11 +1383,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE8" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF8" t="inlineStr">
         <is>
           <t>boundary spanning score</t>
@@ -1696,11 +1407,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL8" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM8" t="inlineStr">
         <is>
           <t>format similar to the OCQ</t>
@@ -1716,25 +1422,10 @@
           <t>BSA</t>
         </is>
       </c>
-      <c r="AP8" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR8" t="n">
-        <v>999</v>
-      </c>
       <c r="AS8" t="inlineStr">
         <is>
           <t>Prof. Comm.</t>
         </is>
-      </c>
-      <c r="AT8" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU8" t="n">
-        <v>999</v>
       </c>
       <c r="AV8" t="n">
         <v>0.9</v>
@@ -1768,9 +1459,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F9" t="n">
-        <v>999</v>
-      </c>
       <c r="G9" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -1799,11 +1487,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N9" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -1814,29 +1497,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q9" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S9" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1847,22 +1515,10 @@
       <c r="V9" t="n">
         <v>253</v>
       </c>
-      <c r="W9" t="n">
-        <v>999</v>
-      </c>
-      <c r="X9" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>999</v>
-      </c>
       <c r="Z9" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
-      </c>
-      <c r="AA9" t="n">
-        <v>999</v>
       </c>
       <c r="AB9" t="n">
         <v>7.5</v>
@@ -1875,11 +1531,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE9" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF9" t="inlineStr">
         <is>
           <t>boundary spanning score</t>
@@ -1890,25 +1541,11 @@
           <t>This was done by obtaining percentile ranking of subjects on intraunit and extraunit communication activity scores and using the mean of the two ranks as the boundary spanning score.</t>
         </is>
       </c>
-      <c r="AH9" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI9" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>999</v>
-      </c>
       <c r="AK9" t="inlineStr">
         <is>
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL9" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM9" t="inlineStr">
         <is>
           <t>interaction variable</t>
@@ -1924,28 +1561,10 @@
           <t>BSA</t>
         </is>
       </c>
-      <c r="AP9" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ9" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR9" t="n">
-        <v>999</v>
-      </c>
       <c r="AS9" t="inlineStr">
         <is>
           <t>Dual Comm.</t>
         </is>
-      </c>
-      <c r="AT9" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU9" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV9" t="n">
-        <v>999</v>
       </c>
       <c r="AW9" t="n">
         <v>-0.1</v>
@@ -1976,9 +1595,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>999</v>
-      </c>
       <c r="G10" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -2007,11 +1623,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N10" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -2022,29 +1633,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q10" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S10" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -2055,22 +1651,10 @@
       <c r="V10" t="n">
         <v>253</v>
       </c>
-      <c r="W10" t="n">
-        <v>999</v>
-      </c>
-      <c r="X10" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y10" t="n">
-        <v>999</v>
-      </c>
       <c r="Z10" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
-      </c>
-      <c r="AA10" t="n">
-        <v>999</v>
       </c>
       <c r="AB10" t="n">
         <v>7.5</v>
@@ -2083,11 +1667,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE10" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF10" t="inlineStr">
         <is>
           <t>boundary spanning score</t>
@@ -2112,11 +1691,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL10" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM10" t="inlineStr">
         <is>
           <t>weighted sum of the percentages</t>
@@ -2132,28 +1706,10 @@
           <t>BSA</t>
         </is>
       </c>
-      <c r="AP10" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ10" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR10" t="n">
-        <v>999</v>
-      </c>
       <c r="AS10" t="inlineStr">
         <is>
           <t>Complexity</t>
         </is>
-      </c>
-      <c r="AT10" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU10" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV10" t="n">
-        <v>999</v>
       </c>
       <c r="AW10" t="n">
         <v>-0.01</v>
@@ -2184,9 +1740,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F11" t="n">
-        <v>999</v>
-      </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -2215,11 +1768,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N11" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -2230,29 +1778,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q11" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S11" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -2263,22 +1796,10 @@
       <c r="V11" t="n">
         <v>253</v>
       </c>
-      <c r="W11" t="n">
-        <v>999</v>
-      </c>
-      <c r="X11" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y11" t="n">
-        <v>999</v>
-      </c>
       <c r="Z11" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
-      </c>
-      <c r="AA11" t="n">
-        <v>999</v>
       </c>
       <c r="AB11" t="n">
         <v>7.5</v>
@@ -2291,11 +1812,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE11" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF11" t="inlineStr">
         <is>
           <t>boundary spanning score</t>
@@ -2320,11 +1836,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL11" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM11" t="inlineStr">
         <is>
           <t>three-item scale</t>
@@ -2340,25 +1851,10 @@
           <t>BSA</t>
         </is>
       </c>
-      <c r="AP11" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ11" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR11" t="n">
-        <v>999</v>
-      </c>
       <c r="AS11" t="inlineStr">
         <is>
           <t>Uncertainty</t>
         </is>
-      </c>
-      <c r="AT11" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU11" t="n">
-        <v>999</v>
       </c>
       <c r="AV11" t="n">
         <v>0.76</v>
@@ -2392,9 +1888,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F12" t="n">
-        <v>999</v>
-      </c>
       <c r="G12" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -2423,11 +1916,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N12" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -2438,29 +1926,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q12" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S12" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -2471,22 +1944,10 @@
       <c r="V12" t="n">
         <v>253</v>
       </c>
-      <c r="W12" t="n">
-        <v>999</v>
-      </c>
-      <c r="X12" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y12" t="n">
-        <v>999</v>
-      </c>
       <c r="Z12" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
-      </c>
-      <c r="AA12" t="n">
-        <v>999</v>
       </c>
       <c r="AB12" t="n">
         <v>7.5</v>
@@ -2499,11 +1960,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE12" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF12" t="inlineStr">
         <is>
           <t>boundary spanning score</t>
@@ -2528,11 +1984,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL12" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM12" t="inlineStr">
         <is>
           <t>Extraproject Coordination scale</t>
@@ -2548,25 +1999,10 @@
           <t>BSA</t>
         </is>
       </c>
-      <c r="AP12" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ12" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR12" t="n">
-        <v>999</v>
-      </c>
       <c r="AS12" t="inlineStr">
         <is>
           <t>Interdepend.</t>
         </is>
-      </c>
-      <c r="AT12" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU12" t="n">
-        <v>999</v>
       </c>
       <c r="AV12" t="n">
         <v>0.63</v>
@@ -2600,9 +2036,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F13" t="n">
-        <v>999</v>
-      </c>
       <c r="G13" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -2631,11 +2064,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N13" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -2646,29 +2074,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q13" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S13" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -2679,22 +2092,10 @@
       <c r="V13" t="n">
         <v>253</v>
       </c>
-      <c r="W13" t="n">
-        <v>999</v>
-      </c>
-      <c r="X13" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y13" t="n">
-        <v>999</v>
-      </c>
       <c r="Z13" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
-      </c>
-      <c r="AA13" t="n">
-        <v>999</v>
       </c>
       <c r="AB13" t="n">
         <v>7.5</v>
@@ -2707,11 +2108,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE13" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF13" t="inlineStr">
         <is>
           <t>boundary spanning score</t>
@@ -2736,11 +2132,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL13" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM13" t="inlineStr">
         <is>
           <t>highest degree attained</t>
@@ -2756,28 +2147,10 @@
           <t>BSA</t>
         </is>
       </c>
-      <c r="AP13" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ13" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR13" t="n">
-        <v>999</v>
-      </c>
       <c r="AS13" t="inlineStr">
         <is>
           <t>Degree</t>
         </is>
-      </c>
-      <c r="AT13" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU13" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV13" t="n">
-        <v>999</v>
       </c>
       <c r="AW13" t="n">
         <v>-0.06</v>
@@ -2808,9 +2181,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>999</v>
-      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -2839,11 +2209,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N14" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -2854,29 +2219,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q14" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S14" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -2887,22 +2237,10 @@
       <c r="V14" t="n">
         <v>253</v>
       </c>
-      <c r="W14" t="n">
-        <v>999</v>
-      </c>
-      <c r="X14" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>999</v>
-      </c>
       <c r="Z14" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
-      </c>
-      <c r="AA14" t="n">
-        <v>999</v>
       </c>
       <c r="AB14" t="n">
         <v>7.5</v>
@@ -2915,11 +2253,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE14" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF14" t="inlineStr">
         <is>
           <t>boundary spanning score</t>
@@ -2944,11 +2277,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL14" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM14" t="inlineStr">
         <is>
           <t>profession</t>
@@ -2964,28 +2292,10 @@
           <t>BSA</t>
         </is>
       </c>
-      <c r="AP14" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ14" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR14" t="n">
-        <v>999</v>
-      </c>
       <c r="AS14" t="inlineStr">
         <is>
           <t>Occupation</t>
         </is>
-      </c>
-      <c r="AT14" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU14" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV14" t="n">
-        <v>999</v>
       </c>
       <c r="AW14" t="n">
         <v>0.12</v>
@@ -3016,9 +2326,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>999</v>
-      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -3047,11 +2354,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N15" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -3062,29 +2364,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q15" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S15" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -3095,22 +2382,10 @@
       <c r="V15" t="n">
         <v>253</v>
       </c>
-      <c r="W15" t="n">
-        <v>999</v>
-      </c>
-      <c r="X15" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y15" t="n">
-        <v>999</v>
-      </c>
       <c r="Z15" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
-      </c>
-      <c r="AA15" t="n">
-        <v>999</v>
       </c>
       <c r="AB15" t="n">
         <v>7.5</v>
@@ -3123,11 +2398,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE15" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF15" t="inlineStr">
         <is>
           <t>boundary spanning score</t>
@@ -3152,11 +2422,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL15" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM15" t="inlineStr">
         <is>
           <t>Professional Control</t>
@@ -3172,25 +2437,10 @@
           <t>BSA</t>
         </is>
       </c>
-      <c r="AP15" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ15" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR15" t="n">
-        <v>999</v>
-      </c>
       <c r="AS15" t="inlineStr">
         <is>
           <t>Prof. Control</t>
         </is>
-      </c>
-      <c r="AT15" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU15" t="n">
-        <v>999</v>
       </c>
       <c r="AV15" t="n">
         <v>0.61</v>
@@ -3224,9 +2474,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>999</v>
-      </c>
       <c r="G16" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -3255,11 +2502,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N16" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -3270,29 +2512,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q16" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S16" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -3303,22 +2530,10 @@
       <c r="V16" t="n">
         <v>253</v>
       </c>
-      <c r="W16" t="n">
-        <v>999</v>
-      </c>
-      <c r="X16" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>999</v>
-      </c>
       <c r="Z16" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
-      </c>
-      <c r="AA16" t="n">
-        <v>999</v>
       </c>
       <c r="AB16" t="n">
         <v>7.5</v>
@@ -3331,11 +2546,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE16" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF16" t="inlineStr">
         <is>
           <t>boundary spanning score</t>
@@ -3360,11 +2570,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL16" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM16" t="inlineStr">
         <is>
           <t>Professional Incentives</t>
@@ -3380,25 +2585,10 @@
           <t>BSA</t>
         </is>
       </c>
-      <c r="AP16" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ16" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR16" t="n">
-        <v>999</v>
-      </c>
       <c r="AS16" t="inlineStr">
         <is>
           <t>Prof. Incent.</t>
         </is>
-      </c>
-      <c r="AT16" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU16" t="n">
-        <v>999</v>
       </c>
       <c r="AV16" t="n">
         <v>0.72</v>
@@ -3432,9 +2622,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F17" t="n">
-        <v>999</v>
-      </c>
       <c r="G17" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -3463,11 +2650,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N17" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -3478,29 +2660,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q17" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S17" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -3511,15 +2678,6 @@
       <c r="V17" t="n">
         <v>253</v>
       </c>
-      <c r="W17" t="n">
-        <v>999</v>
-      </c>
-      <c r="X17" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y17" t="n">
-        <v>999</v>
-      </c>
       <c r="Z17" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -3539,11 +2697,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE17" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF17" t="inlineStr">
         <is>
           <t>Extraunit communication frequency</t>
@@ -3568,11 +2721,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL17" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM17" t="inlineStr">
         <is>
           <t>Intraunit communication frequency</t>
@@ -3588,28 +2736,10 @@
           <t>External Com.</t>
         </is>
       </c>
-      <c r="AP17" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ17" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR17" t="n">
-        <v>999</v>
-      </c>
       <c r="AS17" t="inlineStr">
         <is>
           <t>Internal Com.</t>
         </is>
-      </c>
-      <c r="AT17" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU17" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV17" t="n">
-        <v>999</v>
       </c>
       <c r="AW17" t="n">
         <v>0.1</v>
@@ -3640,9 +2770,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F18" t="n">
-        <v>999</v>
-      </c>
       <c r="G18" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -3671,11 +2798,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N18" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -3686,29 +2808,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q18" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S18" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -3719,15 +2826,6 @@
       <c r="V18" t="n">
         <v>253</v>
       </c>
-      <c r="W18" t="n">
-        <v>999</v>
-      </c>
-      <c r="X18" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y18" t="n">
-        <v>999</v>
-      </c>
       <c r="Z18" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -3747,11 +2845,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE18" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF18" t="inlineStr">
         <is>
           <t>Extraunit communication frequency</t>
@@ -3776,11 +2869,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL18" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM18" t="inlineStr">
         <is>
           <t>job title</t>
@@ -3796,28 +2884,10 @@
           <t>External Com.</t>
         </is>
       </c>
-      <c r="AP18" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ18" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR18" t="n">
-        <v>999</v>
-      </c>
       <c r="AS18" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
-      </c>
-      <c r="AT18" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU18" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV18" t="n">
-        <v>999</v>
       </c>
       <c r="AW18" t="n">
         <v>0.11</v>
@@ -3848,9 +2918,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F19" t="n">
-        <v>999</v>
-      </c>
       <c r="G19" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -3879,11 +2946,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N19" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -3894,29 +2956,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q19" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S19" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -3927,15 +2974,6 @@
       <c r="V19" t="n">
         <v>253</v>
       </c>
-      <c r="W19" t="n">
-        <v>999</v>
-      </c>
-      <c r="X19" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y19" t="n">
-        <v>999</v>
-      </c>
       <c r="Z19" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -3955,11 +2993,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE19" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF19" t="inlineStr">
         <is>
           <t>Extraunit communication frequency</t>
@@ -3984,11 +3017,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL19" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM19" t="inlineStr">
         <is>
           <t>Organizational size</t>
@@ -4004,28 +3032,10 @@
           <t>External Com.</t>
         </is>
       </c>
-      <c r="AP19" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ19" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR19" t="n">
-        <v>999</v>
-      </c>
       <c r="AS19" t="inlineStr">
         <is>
           <t>Org. Size</t>
         </is>
-      </c>
-      <c r="AT19" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU19" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV19" t="n">
-        <v>999</v>
       </c>
       <c r="AW19" t="n">
         <v>-0.05</v>
@@ -4056,9 +3066,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>999</v>
-      </c>
       <c r="G20" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -4087,11 +3094,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N20" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -4102,29 +3104,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q20" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S20" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -4135,15 +3122,6 @@
       <c r="V20" t="n">
         <v>253</v>
       </c>
-      <c r="W20" t="n">
-        <v>999</v>
-      </c>
-      <c r="X20" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y20" t="n">
-        <v>999</v>
-      </c>
       <c r="Z20" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -4163,11 +3141,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE20" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF20" t="inlineStr">
         <is>
           <t>Extraunit communication frequency</t>
@@ -4192,11 +3165,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL20" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM20" t="inlineStr">
         <is>
           <t>dichotomous variable</t>
@@ -4212,28 +3180,10 @@
           <t>External Com.</t>
         </is>
       </c>
-      <c r="AP20" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ20" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR20" t="n">
-        <v>999</v>
-      </c>
       <c r="AS20" t="inlineStr">
         <is>
           <t>Industry</t>
         </is>
-      </c>
-      <c r="AT20" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU20" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV20" t="n">
-        <v>999</v>
       </c>
       <c r="AW20" t="n">
         <v>-0.21</v>
@@ -4264,9 +3214,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>999</v>
-      </c>
       <c r="G21" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -4295,11 +3242,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N21" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -4310,29 +3252,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q21" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S21" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -4343,15 +3270,6 @@
       <c r="V21" t="n">
         <v>253</v>
       </c>
-      <c r="W21" t="n">
-        <v>999</v>
-      </c>
-      <c r="X21" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>999</v>
-      </c>
       <c r="Z21" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -4371,11 +3289,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE21" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF21" t="inlineStr">
         <is>
           <t>Extraunit communication frequency</t>
@@ -4400,11 +3313,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL21" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM21" t="inlineStr">
         <is>
           <t>Organizational Commitment Questionnaire</t>
@@ -4420,25 +3328,10 @@
           <t>External Com.</t>
         </is>
       </c>
-      <c r="AP21" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ21" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR21" t="n">
-        <v>999</v>
-      </c>
       <c r="AS21" t="inlineStr">
         <is>
           <t>Org. Comm.</t>
         </is>
-      </c>
-      <c r="AT21" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU21" t="n">
-        <v>999</v>
       </c>
       <c r="AV21" t="n">
         <v>0.92</v>
@@ -4472,9 +3365,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F22" t="n">
-        <v>999</v>
-      </c>
       <c r="G22" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -4503,11 +3393,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N22" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -4518,29 +3403,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q22" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S22" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -4551,15 +3421,6 @@
       <c r="V22" t="n">
         <v>253</v>
       </c>
-      <c r="W22" t="n">
-        <v>999</v>
-      </c>
-      <c r="X22" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>999</v>
-      </c>
       <c r="Z22" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -4579,11 +3440,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE22" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF22" t="inlineStr">
         <is>
           <t>Extraunit communication frequency</t>
@@ -4608,11 +3464,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL22" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM22" t="inlineStr">
         <is>
           <t>format similar to the OCQ</t>
@@ -4628,25 +3479,10 @@
           <t>External Com.</t>
         </is>
       </c>
-      <c r="AP22" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ22" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR22" t="n">
-        <v>999</v>
-      </c>
       <c r="AS22" t="inlineStr">
         <is>
           <t>Prof. Comm.</t>
         </is>
-      </c>
-      <c r="AT22" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU22" t="n">
-        <v>999</v>
       </c>
       <c r="AV22" t="n">
         <v>0.9</v>
@@ -4680,9 +3516,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>999</v>
-      </c>
       <c r="G23" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -4711,11 +3544,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N23" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -4726,29 +3554,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q23" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S23" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -4759,15 +3572,6 @@
       <c r="V23" t="n">
         <v>253</v>
       </c>
-      <c r="W23" t="n">
-        <v>999</v>
-      </c>
-      <c r="X23" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y23" t="n">
-        <v>999</v>
-      </c>
       <c r="Z23" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -4787,11 +3591,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE23" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF23" t="inlineStr">
         <is>
           <t>Extraunit communication frequency</t>
@@ -4802,25 +3601,11 @@
           <t>Extraunit communication frequency was measured by asking subjects to report frequency of work-related communication on a six-point scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day) with each of 12 categories of individuals over the past month.</t>
         </is>
       </c>
-      <c r="AH23" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI23" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ23" t="n">
-        <v>999</v>
-      </c>
       <c r="AK23" t="inlineStr">
         <is>
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL23" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM23" t="inlineStr">
         <is>
           <t>interaction variable</t>
@@ -4836,28 +3621,10 @@
           <t>External Com.</t>
         </is>
       </c>
-      <c r="AP23" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ23" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR23" t="n">
-        <v>999</v>
-      </c>
       <c r="AS23" t="inlineStr">
         <is>
           <t>Dual Comm.</t>
         </is>
-      </c>
-      <c r="AT23" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU23" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV23" t="n">
-        <v>999</v>
       </c>
       <c r="AW23" t="n">
         <v>-0.05</v>
@@ -4888,9 +3655,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F24" t="n">
-        <v>999</v>
-      </c>
       <c r="G24" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -4919,11 +3683,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N24" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -4934,29 +3693,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q24" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S24" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -4967,15 +3711,6 @@
       <c r="V24" t="n">
         <v>253</v>
       </c>
-      <c r="W24" t="n">
-        <v>999</v>
-      </c>
-      <c r="X24" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y24" t="n">
-        <v>999</v>
-      </c>
       <c r="Z24" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -4995,11 +3730,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE24" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF24" t="inlineStr">
         <is>
           <t>Extraunit communication frequency</t>
@@ -5024,11 +3754,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL24" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM24" t="inlineStr">
         <is>
           <t>weighted sum of the percentages</t>
@@ -5044,28 +3769,10 @@
           <t>External Com.</t>
         </is>
       </c>
-      <c r="AP24" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ24" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR24" t="n">
-        <v>999</v>
-      </c>
       <c r="AS24" t="inlineStr">
         <is>
           <t>Complexity</t>
         </is>
-      </c>
-      <c r="AT24" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU24" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV24" t="n">
-        <v>999</v>
       </c>
       <c r="AW24" t="n">
         <v>0.1</v>
@@ -5096,9 +3803,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F25" t="n">
-        <v>999</v>
-      </c>
       <c r="G25" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -5127,11 +3831,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N25" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -5142,29 +3841,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q25" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S25" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -5175,15 +3859,6 @@
       <c r="V25" t="n">
         <v>253</v>
       </c>
-      <c r="W25" t="n">
-        <v>999</v>
-      </c>
-      <c r="X25" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y25" t="n">
-        <v>999</v>
-      </c>
       <c r="Z25" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -5203,11 +3878,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE25" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF25" t="inlineStr">
         <is>
           <t>Extraunit communication frequency</t>
@@ -5232,11 +3902,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL25" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM25" t="inlineStr">
         <is>
           <t>three-item scale</t>
@@ -5252,25 +3917,10 @@
           <t>External Com.</t>
         </is>
       </c>
-      <c r="AP25" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ25" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR25" t="n">
-        <v>999</v>
-      </c>
       <c r="AS25" t="inlineStr">
         <is>
           <t>Uncertainty</t>
         </is>
-      </c>
-      <c r="AT25" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU25" t="n">
-        <v>999</v>
       </c>
       <c r="AV25" t="n">
         <v>0.76</v>
@@ -5304,9 +3954,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F26" t="n">
-        <v>999</v>
-      </c>
       <c r="G26" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -5335,11 +3982,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N26" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -5350,29 +3992,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q26" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S26" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -5383,15 +4010,6 @@
       <c r="V26" t="n">
         <v>253</v>
       </c>
-      <c r="W26" t="n">
-        <v>999</v>
-      </c>
-      <c r="X26" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y26" t="n">
-        <v>999</v>
-      </c>
       <c r="Z26" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -5411,11 +4029,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE26" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF26" t="inlineStr">
         <is>
           <t>Extraunit communication frequency</t>
@@ -5440,11 +4053,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL26" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM26" t="inlineStr">
         <is>
           <t>Extraproject Coordination scale</t>
@@ -5460,25 +4068,10 @@
           <t>External Com.</t>
         </is>
       </c>
-      <c r="AP26" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ26" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR26" t="n">
-        <v>999</v>
-      </c>
       <c r="AS26" t="inlineStr">
         <is>
           <t>Interdepend.</t>
         </is>
-      </c>
-      <c r="AT26" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU26" t="n">
-        <v>999</v>
       </c>
       <c r="AV26" t="n">
         <v>0.63</v>
@@ -5512,9 +4105,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F27" t="n">
-        <v>999</v>
-      </c>
       <c r="G27" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -5543,11 +4133,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N27" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -5558,29 +4143,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q27" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S27" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -5591,15 +4161,6 @@
       <c r="V27" t="n">
         <v>253</v>
       </c>
-      <c r="W27" t="n">
-        <v>999</v>
-      </c>
-      <c r="X27" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y27" t="n">
-        <v>999</v>
-      </c>
       <c r="Z27" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -5619,11 +4180,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE27" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF27" t="inlineStr">
         <is>
           <t>Extraunit communication frequency</t>
@@ -5648,11 +4204,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL27" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM27" t="inlineStr">
         <is>
           <t>highest degree attained</t>
@@ -5668,28 +4219,10 @@
           <t>External Com.</t>
         </is>
       </c>
-      <c r="AP27" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ27" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR27" t="n">
-        <v>999</v>
-      </c>
       <c r="AS27" t="inlineStr">
         <is>
           <t>Degree</t>
         </is>
-      </c>
-      <c r="AT27" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU27" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV27" t="n">
-        <v>999</v>
       </c>
       <c r="AW27" t="n">
         <v>0.17</v>
@@ -5720,9 +4253,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>999</v>
-      </c>
       <c r="G28" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -5751,11 +4281,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N28" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -5766,29 +4291,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q28" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S28" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -5799,15 +4309,6 @@
       <c r="V28" t="n">
         <v>253</v>
       </c>
-      <c r="W28" t="n">
-        <v>999</v>
-      </c>
-      <c r="X28" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y28" t="n">
-        <v>999</v>
-      </c>
       <c r="Z28" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -5827,11 +4328,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE28" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF28" t="inlineStr">
         <is>
           <t>Extraunit communication frequency</t>
@@ -5856,11 +4352,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL28" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM28" t="inlineStr">
         <is>
           <t>profession</t>
@@ -5876,28 +4367,10 @@
           <t>External Com.</t>
         </is>
       </c>
-      <c r="AP28" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ28" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR28" t="n">
-        <v>999</v>
-      </c>
       <c r="AS28" t="inlineStr">
         <is>
           <t>Occupation</t>
         </is>
-      </c>
-      <c r="AT28" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU28" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV28" t="n">
-        <v>999</v>
       </c>
       <c r="AW28" t="n">
         <v>-0.13</v>
@@ -5928,9 +4401,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F29" t="n">
-        <v>999</v>
-      </c>
       <c r="G29" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -5959,11 +4429,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N29" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -5974,29 +4439,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q29" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S29" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -6007,15 +4457,6 @@
       <c r="V29" t="n">
         <v>253</v>
       </c>
-      <c r="W29" t="n">
-        <v>999</v>
-      </c>
-      <c r="X29" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y29" t="n">
-        <v>999</v>
-      </c>
       <c r="Z29" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -6035,11 +4476,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE29" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF29" t="inlineStr">
         <is>
           <t>Extraunit communication frequency</t>
@@ -6064,11 +4500,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL29" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM29" t="inlineStr">
         <is>
           <t>Professional Control</t>
@@ -6084,25 +4515,10 @@
           <t>External Com.</t>
         </is>
       </c>
-      <c r="AP29" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ29" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR29" t="n">
-        <v>999</v>
-      </c>
       <c r="AS29" t="inlineStr">
         <is>
           <t>Prof. Control</t>
         </is>
-      </c>
-      <c r="AT29" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU29" t="n">
-        <v>999</v>
       </c>
       <c r="AV29" t="n">
         <v>0.61</v>
@@ -6136,9 +4552,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F30" t="n">
-        <v>999</v>
-      </c>
       <c r="G30" t="inlineStr">
         <is>
           <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
@@ -6167,11 +4580,6 @@
           <t>2 = Dissertation</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N30" t="inlineStr">
         <is>
           <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
@@ -6182,29 +4590,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q30" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S30" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -6215,15 +4608,6 @@
       <c r="V30" t="n">
         <v>253</v>
       </c>
-      <c r="W30" t="n">
-        <v>999</v>
-      </c>
-      <c r="X30" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y30" t="n">
-        <v>999</v>
-      </c>
       <c r="Z30" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -6243,11 +4627,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE30" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF30" t="inlineStr">
         <is>
           <t>Extraunit communication frequency</t>
@@ -6272,11 +4651,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL30" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM30" t="inlineStr">
         <is>
           <t>Professional Incentives</t>
@@ -6292,25 +4666,10 @@
           <t>External Com.</t>
         </is>
       </c>
-      <c r="AP30" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ30" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR30" t="n">
-        <v>999</v>
-      </c>
       <c r="AS30" t="inlineStr">
         <is>
           <t>Prof. Incent.</t>
         </is>
-      </c>
-      <c r="AT30" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU30" t="n">
-        <v>999</v>
       </c>
       <c r="AV30" t="n">
         <v>0.72</v>
@@ -6344,9 +4703,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F31" t="n">
-        <v>999</v>
-      </c>
       <c r="G31" t="inlineStr">
         <is>
           <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
@@ -6375,11 +4731,6 @@
           <t>1 = Journal article</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N31" t="inlineStr">
         <is>
           <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
@@ -6390,29 +4741,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q31" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S31" t="inlineStr">
         <is>
           <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -6423,15 +4759,9 @@
       <c r="V31" t="n">
         <v>382</v>
       </c>
-      <c r="W31" t="n">
-        <v>999</v>
-      </c>
       <c r="X31" t="n">
         <v>65.2</v>
       </c>
-      <c r="Y31" t="n">
-        <v>999</v>
-      </c>
       <c r="Z31" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -6451,11 +4781,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE31" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF31" t="inlineStr">
         <is>
           <t>Bettencourt et al. (2005)</t>
@@ -6480,11 +4805,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL31" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM31" t="inlineStr">
         <is>
           <t>Rizzo, House, and Lirtzman (1970)</t>
@@ -6499,12 +4819,6 @@
         <is>
           <t>External Representation</t>
         </is>
-      </c>
-      <c r="AP31" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ31" t="n">
-        <v>999</v>
       </c>
       <c r="AR31" t="n">
         <v>0.871</v>
@@ -6513,12 +4827,6 @@
         <is>
           <t>Role Conflict</t>
         </is>
-      </c>
-      <c r="AT31" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU31" t="n">
-        <v>999</v>
       </c>
       <c r="AV31" t="n">
         <v>0.619</v>
@@ -6552,9 +4860,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F32" t="n">
-        <v>999</v>
-      </c>
       <c r="G32" t="inlineStr">
         <is>
           <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
@@ -6583,11 +4888,6 @@
           <t>1 = Journal article</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N32" t="inlineStr">
         <is>
           <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
@@ -6598,29 +4898,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q32" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S32" t="inlineStr">
         <is>
           <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -6631,15 +4916,9 @@
       <c r="V32" t="n">
         <v>382</v>
       </c>
-      <c r="W32" t="n">
-        <v>999</v>
-      </c>
       <c r="X32" t="n">
         <v>65.2</v>
       </c>
-      <c r="Y32" t="n">
-        <v>999</v>
-      </c>
       <c r="Z32" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -6659,11 +4938,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE32" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF32" t="inlineStr">
         <is>
           <t>Bettencourt et al. (2005)</t>
@@ -6688,11 +4962,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL32" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM32" t="inlineStr">
         <is>
           <t>Rizzo, House, and Lirtzman (1970)</t>
@@ -6707,12 +4976,6 @@
         <is>
           <t>External Representation</t>
         </is>
-      </c>
-      <c r="AP32" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ32" t="n">
-        <v>999</v>
       </c>
       <c r="AR32" t="n">
         <v>0.871</v>
@@ -6721,12 +4984,6 @@
         <is>
           <t>Role Ambiguity</t>
         </is>
-      </c>
-      <c r="AT32" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU32" t="n">
-        <v>999</v>
       </c>
       <c r="AV32" t="n">
         <v>0.777</v>
@@ -6760,9 +5017,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F33" t="n">
-        <v>999</v>
-      </c>
       <c r="G33" t="inlineStr">
         <is>
           <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
@@ -6791,11 +5045,6 @@
           <t>1 = Journal article</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N33" t="inlineStr">
         <is>
           <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
@@ -6806,29 +5055,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q33" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S33" t="inlineStr">
         <is>
           <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -6839,15 +5073,9 @@
       <c r="V33" t="n">
         <v>382</v>
       </c>
-      <c r="W33" t="n">
-        <v>999</v>
-      </c>
       <c r="X33" t="n">
         <v>65.2</v>
       </c>
-      <c r="Y33" t="n">
-        <v>999</v>
-      </c>
       <c r="Z33" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -6867,11 +5095,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE33" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF33" t="inlineStr">
         <is>
           <t>Bettencourt et al. (2005)</t>
@@ -6896,11 +5119,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL33" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM33" t="inlineStr">
         <is>
           <t>Seibert, Kraimer, and Crant (2001)</t>
@@ -6915,12 +5133,6 @@
         <is>
           <t>External Representation</t>
         </is>
-      </c>
-      <c r="AP33" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ33" t="n">
-        <v>999</v>
       </c>
       <c r="AR33" t="n">
         <v>0.871</v>
@@ -6929,12 +5141,6 @@
         <is>
           <t>Proactive Personality</t>
         </is>
-      </c>
-      <c r="AT33" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU33" t="n">
-        <v>999</v>
       </c>
       <c r="AV33" t="n">
         <v>0.894</v>
@@ -6968,9 +5174,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F34" t="n">
-        <v>999</v>
-      </c>
       <c r="G34" t="inlineStr">
         <is>
           <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
@@ -6999,11 +5202,6 @@
           <t>1 = Journal article</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N34" t="inlineStr">
         <is>
           <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
@@ -7014,29 +5212,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q34" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S34" t="inlineStr">
         <is>
           <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="T34" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -7047,15 +5230,9 @@
       <c r="V34" t="n">
         <v>382</v>
       </c>
-      <c r="W34" t="n">
-        <v>999</v>
-      </c>
       <c r="X34" t="n">
         <v>65.2</v>
       </c>
-      <c r="Y34" t="n">
-        <v>999</v>
-      </c>
       <c r="Z34" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -7075,11 +5252,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE34" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF34" t="inlineStr">
         <is>
           <t>Bettencourt et al. (2005)</t>
@@ -7104,11 +5276,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL34" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM34" t="inlineStr">
         <is>
           <t>Zhou and George’s (2001) 4-item scale</t>
@@ -7123,12 +5290,6 @@
         <is>
           <t>External Representation</t>
         </is>
-      </c>
-      <c r="AP34" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ34" t="n">
-        <v>999</v>
       </c>
       <c r="AR34" t="n">
         <v>0.871</v>
@@ -7137,12 +5298,6 @@
         <is>
           <t>Employee Creativity</t>
         </is>
-      </c>
-      <c r="AT34" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU34" t="n">
-        <v>999</v>
       </c>
       <c r="AV34" t="n">
         <v>0.839</v>
@@ -7176,9 +5331,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F35" t="n">
-        <v>999</v>
-      </c>
       <c r="G35" t="inlineStr">
         <is>
           <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
@@ -7207,11 +5359,6 @@
           <t>1 = Journal article</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N35" t="inlineStr">
         <is>
           <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
@@ -7222,29 +5369,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q35" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S35" t="inlineStr">
         <is>
           <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="T35" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -7255,15 +5387,9 @@
       <c r="V35" t="n">
         <v>382</v>
       </c>
-      <c r="W35" t="n">
-        <v>999</v>
-      </c>
       <c r="X35" t="n">
         <v>65.2</v>
       </c>
-      <c r="Y35" t="n">
-        <v>999</v>
-      </c>
       <c r="Z35" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -7283,11 +5409,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE35" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF35" t="inlineStr">
         <is>
           <t>Bettencourt et al. (2005)</t>
@@ -7312,11 +5433,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL35" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM35" t="inlineStr">
         <is>
           <t>Rizzo, House, and Lirtzman (1970)</t>
@@ -7331,12 +5447,6 @@
         <is>
           <t>Internal Influence</t>
         </is>
-      </c>
-      <c r="AP35" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ35" t="n">
-        <v>999</v>
       </c>
       <c r="AR35" t="n">
         <v>0.872</v>
@@ -7345,12 +5455,6 @@
         <is>
           <t>Role Conflict</t>
         </is>
-      </c>
-      <c r="AT35" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU35" t="n">
-        <v>999</v>
       </c>
       <c r="AV35" t="n">
         <v>0.619</v>
@@ -7384,9 +5488,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F36" t="n">
-        <v>999</v>
-      </c>
       <c r="G36" t="inlineStr">
         <is>
           <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
@@ -7415,11 +5516,6 @@
           <t>1 = Journal article</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N36" t="inlineStr">
         <is>
           <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
@@ -7430,29 +5526,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q36" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S36" t="inlineStr">
         <is>
           <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="T36" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -7463,15 +5544,9 @@
       <c r="V36" t="n">
         <v>382</v>
       </c>
-      <c r="W36" t="n">
-        <v>999</v>
-      </c>
       <c r="X36" t="n">
         <v>65.2</v>
       </c>
-      <c r="Y36" t="n">
-        <v>999</v>
-      </c>
       <c r="Z36" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -7491,11 +5566,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE36" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF36" t="inlineStr">
         <is>
           <t>Bettencourt et al. (2005)</t>
@@ -7520,11 +5590,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL36" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM36" t="inlineStr">
         <is>
           <t>Rizzo, House, and Lirtzman (1970)</t>
@@ -7539,12 +5604,6 @@
         <is>
           <t>Internal Influence</t>
         </is>
-      </c>
-      <c r="AP36" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ36" t="n">
-        <v>999</v>
       </c>
       <c r="AR36" t="n">
         <v>0.872</v>
@@ -7553,12 +5612,6 @@
         <is>
           <t>Role Ambiguity</t>
         </is>
-      </c>
-      <c r="AT36" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU36" t="n">
-        <v>999</v>
       </c>
       <c r="AV36" t="n">
         <v>0.777</v>
@@ -7592,9 +5645,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F37" t="n">
-        <v>999</v>
-      </c>
       <c r="G37" t="inlineStr">
         <is>
           <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
@@ -7623,11 +5673,6 @@
           <t>1 = Journal article</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N37" t="inlineStr">
         <is>
           <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
@@ -7638,29 +5683,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q37" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S37" t="inlineStr">
         <is>
           <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="T37" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -7671,15 +5701,9 @@
       <c r="V37" t="n">
         <v>382</v>
       </c>
-      <c r="W37" t="n">
-        <v>999</v>
-      </c>
       <c r="X37" t="n">
         <v>65.2</v>
       </c>
-      <c r="Y37" t="n">
-        <v>999</v>
-      </c>
       <c r="Z37" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -7699,11 +5723,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE37" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF37" t="inlineStr">
         <is>
           <t>Bettencourt et al. (2005)</t>
@@ -7728,11 +5747,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL37" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM37" t="inlineStr">
         <is>
           <t>Seibert, Kraimer, and Crant (2001)</t>
@@ -7747,12 +5761,6 @@
         <is>
           <t>Internal Influence</t>
         </is>
-      </c>
-      <c r="AP37" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ37" t="n">
-        <v>999</v>
       </c>
       <c r="AR37" t="n">
         <v>0.872</v>
@@ -7761,12 +5769,6 @@
         <is>
           <t>Proactive Personality</t>
         </is>
-      </c>
-      <c r="AT37" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU37" t="n">
-        <v>999</v>
       </c>
       <c r="AV37" t="n">
         <v>0.894</v>
@@ -7800,9 +5802,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F38" t="n">
-        <v>999</v>
-      </c>
       <c r="G38" t="inlineStr">
         <is>
           <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
@@ -7831,11 +5830,6 @@
           <t>1 = Journal article</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N38" t="inlineStr">
         <is>
           <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
@@ -7846,29 +5840,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q38" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S38" t="inlineStr">
         <is>
           <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="T38" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -7879,15 +5858,9 @@
       <c r="V38" t="n">
         <v>382</v>
       </c>
-      <c r="W38" t="n">
-        <v>999</v>
-      </c>
       <c r="X38" t="n">
         <v>65.2</v>
       </c>
-      <c r="Y38" t="n">
-        <v>999</v>
-      </c>
       <c r="Z38" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -7907,11 +5880,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE38" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF38" t="inlineStr">
         <is>
           <t>Bettencourt et al. (2005)</t>
@@ -7936,11 +5904,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL38" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM38" t="inlineStr">
         <is>
           <t>Zhou and George’s (2001) 4-item scale</t>
@@ -7955,12 +5918,6 @@
         <is>
           <t>Internal Influence</t>
         </is>
-      </c>
-      <c r="AP38" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ38" t="n">
-        <v>999</v>
       </c>
       <c r="AR38" t="n">
         <v>0.872</v>
@@ -7969,12 +5926,6 @@
         <is>
           <t>Employee Creativity</t>
         </is>
-      </c>
-      <c r="AT38" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU38" t="n">
-        <v>999</v>
       </c>
       <c r="AV38" t="n">
         <v>0.839</v>
@@ -8008,9 +5959,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F39" t="n">
-        <v>999</v>
-      </c>
       <c r="G39" t="inlineStr">
         <is>
           <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
@@ -8039,11 +5987,6 @@
           <t>1 = Journal article</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N39" t="inlineStr">
         <is>
           <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
@@ -8054,29 +5997,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q39" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S39" t="inlineStr">
         <is>
           <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="T39" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -8087,15 +6015,9 @@
       <c r="V39" t="n">
         <v>382</v>
       </c>
-      <c r="W39" t="n">
-        <v>999</v>
-      </c>
       <c r="X39" t="n">
         <v>65.2</v>
       </c>
-      <c r="Y39" t="n">
-        <v>999</v>
-      </c>
       <c r="Z39" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -8115,11 +6037,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE39" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF39" t="inlineStr">
         <is>
           <t>Bettencourt et al. (2005)</t>
@@ -8144,11 +6061,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL39" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM39" t="inlineStr">
         <is>
           <t>Rizzo, House, and Lirtzman (1970)</t>
@@ -8163,12 +6075,6 @@
         <is>
           <t>Service Delivery</t>
         </is>
-      </c>
-      <c r="AP39" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ39" t="n">
-        <v>999</v>
       </c>
       <c r="AR39" t="n">
         <v>0.876</v>
@@ -8177,12 +6083,6 @@
         <is>
           <t>Role Conflict</t>
         </is>
-      </c>
-      <c r="AT39" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU39" t="n">
-        <v>999</v>
       </c>
       <c r="AV39" t="n">
         <v>0.619</v>
@@ -8216,9 +6116,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F40" t="n">
-        <v>999</v>
-      </c>
       <c r="G40" t="inlineStr">
         <is>
           <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
@@ -8247,11 +6144,6 @@
           <t>1 = Journal article</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N40" t="inlineStr">
         <is>
           <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
@@ -8262,29 +6154,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q40" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S40" t="inlineStr">
         <is>
           <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="T40" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -8295,15 +6172,9 @@
       <c r="V40" t="n">
         <v>382</v>
       </c>
-      <c r="W40" t="n">
-        <v>999</v>
-      </c>
       <c r="X40" t="n">
         <v>65.2</v>
       </c>
-      <c r="Y40" t="n">
-        <v>999</v>
-      </c>
       <c r="Z40" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -8323,11 +6194,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE40" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF40" t="inlineStr">
         <is>
           <t>Bettencourt et al. (2005)</t>
@@ -8352,11 +6218,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL40" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM40" t="inlineStr">
         <is>
           <t>Rizzo, House, and Lirtzman (1970)</t>
@@ -8371,12 +6232,6 @@
         <is>
           <t>Service Delivery</t>
         </is>
-      </c>
-      <c r="AP40" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ40" t="n">
-        <v>999</v>
       </c>
       <c r="AR40" t="n">
         <v>0.876</v>
@@ -8385,12 +6240,6 @@
         <is>
           <t>Role Ambiguity</t>
         </is>
-      </c>
-      <c r="AT40" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU40" t="n">
-        <v>999</v>
       </c>
       <c r="AV40" t="n">
         <v>0.777</v>
@@ -8424,9 +6273,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F41" t="n">
-        <v>999</v>
-      </c>
       <c r="G41" t="inlineStr">
         <is>
           <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
@@ -8455,11 +6301,6 @@
           <t>1 = Journal article</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N41" t="inlineStr">
         <is>
           <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
@@ -8470,29 +6311,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q41" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S41" t="inlineStr">
         <is>
           <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="T41" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -8503,15 +6329,9 @@
       <c r="V41" t="n">
         <v>382</v>
       </c>
-      <c r="W41" t="n">
-        <v>999</v>
-      </c>
       <c r="X41" t="n">
         <v>65.2</v>
       </c>
-      <c r="Y41" t="n">
-        <v>999</v>
-      </c>
       <c r="Z41" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -8531,11 +6351,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE41" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF41" t="inlineStr">
         <is>
           <t>Bettencourt et al. (2005)</t>
@@ -8560,11 +6375,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL41" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM41" t="inlineStr">
         <is>
           <t>Seibert, Kraimer, and Crant (2001)</t>
@@ -8579,12 +6389,6 @@
         <is>
           <t>Service Delivery</t>
         </is>
-      </c>
-      <c r="AP41" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ41" t="n">
-        <v>999</v>
       </c>
       <c r="AR41" t="n">
         <v>0.876</v>
@@ -8593,12 +6397,6 @@
         <is>
           <t>Proactive Personality</t>
         </is>
-      </c>
-      <c r="AT41" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU41" t="n">
-        <v>999</v>
       </c>
       <c r="AV41" t="n">
         <v>0.894</v>
@@ -8632,9 +6430,6 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="F42" t="n">
-        <v>999</v>
-      </c>
       <c r="G42" t="inlineStr">
         <is>
           <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
@@ -8663,11 +6458,6 @@
           <t>1 = Journal article</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N42" t="inlineStr">
         <is>
           <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
@@ -8678,29 +6468,14 @@
           <t>0 = No</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="Q42" t="inlineStr">
         <is>
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S42" t="inlineStr">
         <is>
           <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="T42" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -8711,15 +6486,9 @@
       <c r="V42" t="n">
         <v>382</v>
       </c>
-      <c r="W42" t="n">
-        <v>999</v>
-      </c>
       <c r="X42" t="n">
         <v>65.2</v>
       </c>
-      <c r="Y42" t="n">
-        <v>999</v>
-      </c>
       <c r="Z42" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -8739,11 +6508,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE42" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF42" t="inlineStr">
         <is>
           <t>Bettencourt et al. (2005)</t>
@@ -8768,11 +6532,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL42" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM42" t="inlineStr">
         <is>
           <t>Zhou and George’s (2001) 4-item scale</t>
@@ -8787,12 +6546,6 @@
         <is>
           <t>Service Delivery</t>
         </is>
-      </c>
-      <c r="AP42" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ42" t="n">
-        <v>999</v>
       </c>
       <c r="AR42" t="n">
         <v>0.876</v>
@@ -8801,12 +6554,6 @@
         <is>
           <t>Employee Creativity</t>
         </is>
-      </c>
-      <c r="AT42" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU42" t="n">
-        <v>999</v>
       </c>
       <c r="AV42" t="n">
         <v>0.839</v>
@@ -8832,9 +6579,6 @@
       <c r="C43" t="n">
         <v>1</v>
       </c>
-      <c r="D43" t="n">
-        <v>999</v>
-      </c>
       <c r="E43" t="inlineStr">
         <is>
           <t>0 = exclude</t>
@@ -8873,11 +6617,6 @@
           <t>1 = Journal article</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="N43" t="inlineStr">
         <is>
           <t>Jonathon N. Cummings (2004). Work Groups, Structural Diversity, and Knowledge Sharing in a Global Organization. Management Science.</t>
@@ -8898,19 +6637,9 @@
           <t>1 = Cross-sectional design</t>
         </is>
       </c>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="S43" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="T43" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -8921,91 +6650,10 @@
       <c r="V43" t="n">
         <v>182</v>
       </c>
-      <c r="W43" t="n">
-        <v>999</v>
-      </c>
-      <c r="X43" t="n">
-        <v>999</v>
-      </c>
-      <c r="Y43" t="n">
-        <v>999</v>
-      </c>
       <c r="Z43" t="inlineStr">
         <is>
           <t>Work group members / leaders</t>
         </is>
-      </c>
-      <c r="AA43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AB43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AC43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AD43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AE43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AF43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AG43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AH43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AK43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AL43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AM43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AN43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AO43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AP43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AQ43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AR43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AS43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AT43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AU43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AV43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AW43" t="n">
-        <v>999</v>
-      </c>
-      <c r="AX43" t="n">
-        <v>999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Streamline extraction schema: Blank Article Descriptors, blank SampleID, and clean terminate for excluded papers
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/70_94_109.xlsx
+++ b/03_Coding_Sheets/70_94_109.xlsx
@@ -717,53 +717,12 @@
       <c r="B4" t="n">
         <v>70</v>
       </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -862,53 +821,12 @@
       <c r="B5" t="n">
         <v>70</v>
       </c>
-      <c r="C5" t="n">
-        <v>1</v>
-      </c>
       <c r="D5" t="n">
         <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -1007,53 +925,12 @@
       <c r="B6" t="n">
         <v>70</v>
       </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
       <c r="D6" t="n">
         <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1152,53 +1029,12 @@
       <c r="B7" t="n">
         <v>70</v>
       </c>
-      <c r="C7" t="n">
-        <v>1</v>
-      </c>
       <c r="D7" t="n">
         <v>4</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1300,53 +1136,12 @@
       <c r="B8" t="n">
         <v>70</v>
       </c>
-      <c r="C8" t="n">
-        <v>1</v>
-      </c>
       <c r="D8" t="n">
         <v>5</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1448,53 +1243,12 @@
       <c r="B9" t="n">
         <v>70</v>
       </c>
-      <c r="C9" t="n">
-        <v>1</v>
-      </c>
       <c r="D9" t="n">
         <v>6</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1584,53 +1338,12 @@
       <c r="B10" t="n">
         <v>70</v>
       </c>
-      <c r="C10" t="n">
-        <v>1</v>
-      </c>
       <c r="D10" t="n">
         <v>7</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1729,53 +1442,12 @@
       <c r="B11" t="n">
         <v>70</v>
       </c>
-      <c r="C11" t="n">
-        <v>1</v>
-      </c>
       <c r="D11" t="n">
         <v>8</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -1877,53 +1549,12 @@
       <c r="B12" t="n">
         <v>70</v>
       </c>
-      <c r="C12" t="n">
-        <v>1</v>
-      </c>
       <c r="D12" t="n">
         <v>9</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K12" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -2025,53 +1656,12 @@
       <c r="B13" t="n">
         <v>70</v>
       </c>
-      <c r="C13" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" t="n">
         <v>10</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K13" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -2170,53 +1760,12 @@
       <c r="B14" t="n">
         <v>70</v>
       </c>
-      <c r="C14" t="n">
-        <v>1</v>
-      </c>
       <c r="D14" t="n">
         <v>11</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K14" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -2315,53 +1864,12 @@
       <c r="B15" t="n">
         <v>70</v>
       </c>
-      <c r="C15" t="n">
-        <v>1</v>
-      </c>
       <c r="D15" t="n">
         <v>12</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K15" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -2463,53 +1971,12 @@
       <c r="B16" t="n">
         <v>70</v>
       </c>
-      <c r="C16" t="n">
-        <v>1</v>
-      </c>
       <c r="D16" t="n">
         <v>13</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K16" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -2611,53 +2078,12 @@
       <c r="B17" t="n">
         <v>70</v>
       </c>
-      <c r="C17" t="n">
-        <v>1</v>
-      </c>
       <c r="D17" t="n">
         <v>14</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K17" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -2759,53 +2185,12 @@
       <c r="B18" t="n">
         <v>70</v>
       </c>
-      <c r="C18" t="n">
-        <v>1</v>
-      </c>
       <c r="D18" t="n">
         <v>15</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K18" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -2907,53 +2292,12 @@
       <c r="B19" t="n">
         <v>70</v>
       </c>
-      <c r="C19" t="n">
-        <v>1</v>
-      </c>
       <c r="D19" t="n">
         <v>16</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K19" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -3055,53 +2399,12 @@
       <c r="B20" t="n">
         <v>70</v>
       </c>
-      <c r="C20" t="n">
-        <v>1</v>
-      </c>
       <c r="D20" t="n">
         <v>17</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K20" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -3203,53 +2506,12 @@
       <c r="B21" t="n">
         <v>70</v>
       </c>
-      <c r="C21" t="n">
-        <v>1</v>
-      </c>
       <c r="D21" t="n">
         <v>18</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K21" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -3354,53 +2616,12 @@
       <c r="B22" t="n">
         <v>70</v>
       </c>
-      <c r="C22" t="n">
-        <v>1</v>
-      </c>
       <c r="D22" t="n">
         <v>19</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K22" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -3505,53 +2726,12 @@
       <c r="B23" t="n">
         <v>70</v>
       </c>
-      <c r="C23" t="n">
-        <v>1</v>
-      </c>
       <c r="D23" t="n">
         <v>20</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K23" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -3644,53 +2824,12 @@
       <c r="B24" t="n">
         <v>70</v>
       </c>
-      <c r="C24" t="n">
-        <v>1</v>
-      </c>
       <c r="D24" t="n">
         <v>21</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K24" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -3792,53 +2931,12 @@
       <c r="B25" t="n">
         <v>70</v>
       </c>
-      <c r="C25" t="n">
-        <v>1</v>
-      </c>
       <c r="D25" t="n">
         <v>22</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K25" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -3943,53 +3041,12 @@
       <c r="B26" t="n">
         <v>70</v>
       </c>
-      <c r="C26" t="n">
-        <v>1</v>
-      </c>
       <c r="D26" t="n">
         <v>23</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K26" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -4094,53 +3151,12 @@
       <c r="B27" t="n">
         <v>70</v>
       </c>
-      <c r="C27" t="n">
-        <v>1</v>
-      </c>
       <c r="D27" t="n">
         <v>24</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K27" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -4242,53 +3258,12 @@
       <c r="B28" t="n">
         <v>70</v>
       </c>
-      <c r="C28" t="n">
-        <v>1</v>
-      </c>
       <c r="D28" t="n">
         <v>25</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K28" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -4390,53 +3365,12 @@
       <c r="B29" t="n">
         <v>70</v>
       </c>
-      <c r="C29" t="n">
-        <v>1</v>
-      </c>
       <c r="D29" t="n">
         <v>26</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K29" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -4541,53 +3475,12 @@
       <c r="B30" t="n">
         <v>70</v>
       </c>
-      <c r="C30" t="n">
-        <v>1</v>
-      </c>
       <c r="D30" t="n">
         <v>27</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Examines the relationship between dual commitment (organizational and professional) and boundary spanning activity among technical professionals in R&amp;D organizations.</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Doctoral Dissertation, University of California</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Carol Sexton</t>
-        </is>
-      </c>
-      <c r="K30" t="n">
-        <v>1995</v>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>2 = Dissertation</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>Carol Sexton (1995). Dual Commitment and Boundary Spanning Activity of R&amp;D Professionals. Doctoral Dissertation, University of California.</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -4692,53 +3585,12 @@
       <c r="B31" t="n">
         <v>94</v>
       </c>
-      <c r="C31" t="n">
-        <v>1</v>
-      </c>
       <c r="D31" t="n">
         <v>1</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>Journal of Hospitality and Tourism Management</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang</t>
-        </is>
-      </c>
-      <c r="K31" t="n">
-        <v>2021</v>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -4849,53 +3701,12 @@
       <c r="B32" t="n">
         <v>94</v>
       </c>
-      <c r="C32" t="n">
-        <v>1</v>
-      </c>
       <c r="D32" t="n">
         <v>2</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>Journal of Hospitality and Tourism Management</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang</t>
-        </is>
-      </c>
-      <c r="K32" t="n">
-        <v>2021</v>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -5006,53 +3817,12 @@
       <c r="B33" t="n">
         <v>94</v>
       </c>
-      <c r="C33" t="n">
-        <v>1</v>
-      </c>
       <c r="D33" t="n">
         <v>3</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>Journal of Hospitality and Tourism Management</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang</t>
-        </is>
-      </c>
-      <c r="K33" t="n">
-        <v>2021</v>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -5163,53 +3933,12 @@
       <c r="B34" t="n">
         <v>94</v>
       </c>
-      <c r="C34" t="n">
-        <v>1</v>
-      </c>
       <c r="D34" t="n">
         <v>4</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>Journal of Hospitality and Tourism Management</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang</t>
-        </is>
-      </c>
-      <c r="K34" t="n">
-        <v>2021</v>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -5320,53 +4049,12 @@
       <c r="B35" t="n">
         <v>94</v>
       </c>
-      <c r="C35" t="n">
-        <v>1</v>
-      </c>
       <c r="D35" t="n">
         <v>5</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>Journal of Hospitality and Tourism Management</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang</t>
-        </is>
-      </c>
-      <c r="K35" t="n">
-        <v>2021</v>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -5477,53 +4165,12 @@
       <c r="B36" t="n">
         <v>94</v>
       </c>
-      <c r="C36" t="n">
-        <v>1</v>
-      </c>
       <c r="D36" t="n">
         <v>6</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>Journal of Hospitality and Tourism Management</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang</t>
-        </is>
-      </c>
-      <c r="K36" t="n">
-        <v>2021</v>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -5634,53 +4281,12 @@
       <c r="B37" t="n">
         <v>94</v>
       </c>
-      <c r="C37" t="n">
-        <v>1</v>
-      </c>
       <c r="D37" t="n">
         <v>7</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>Journal of Hospitality and Tourism Management</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang</t>
-        </is>
-      </c>
-      <c r="K37" t="n">
-        <v>2021</v>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
@@ -5791,53 +4397,12 @@
       <c r="B38" t="n">
         <v>94</v>
       </c>
-      <c r="C38" t="n">
-        <v>1</v>
-      </c>
       <c r="D38" t="n">
         <v>8</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>Journal of Hospitality and Tourism Management</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang</t>
-        </is>
-      </c>
-      <c r="K38" t="n">
-        <v>2021</v>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -5948,53 +4513,12 @@
       <c r="B39" t="n">
         <v>94</v>
       </c>
-      <c r="C39" t="n">
-        <v>1</v>
-      </c>
       <c r="D39" t="n">
         <v>9</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>Journal of Hospitality and Tourism Management</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang</t>
-        </is>
-      </c>
-      <c r="K39" t="n">
-        <v>2021</v>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -6105,53 +4629,12 @@
       <c r="B40" t="n">
         <v>94</v>
       </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
       <c r="D40" t="n">
         <v>10</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>Journal of Hospitality and Tourism Management</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang</t>
-        </is>
-      </c>
-      <c r="K40" t="n">
-        <v>2021</v>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
-        </is>
-      </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -6262,53 +4745,12 @@
       <c r="B41" t="n">
         <v>94</v>
       </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
       <c r="D41" t="n">
         <v>11</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>Journal of Hospitality and Tourism Management</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang</t>
-        </is>
-      </c>
-      <c r="K41" t="n">
-        <v>2021</v>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
-        </is>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -6419,53 +4861,12 @@
       <c r="B42" t="n">
         <v>94</v>
       </c>
-      <c r="C42" t="n">
-        <v>1</v>
-      </c>
       <c r="D42" t="n">
         <v>12</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
           <t>1 = include</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Investigates how role stress and proactive personality affect hotel frontline employees' creativity and customer-oriented boundary-spanning behaviors (COBSBs).</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>Journal of Hospitality and Tourism Management</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang</t>
-        </is>
-      </c>
-      <c r="K42" t="n">
-        <v>2021</v>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>Shih-Yi Chien, Albert Jing-Fuh Yang, &amp; Yung-Chin Huang (2021). Hotel frontline service employees’ creativity and customer-oriented boundary-spanning behaviors: The effects of role stress and proactive personality. Journal of Hospitality and Tourism Management.</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>0 = No</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -6576,9 +4977,6 @@
       <c r="B43" t="n">
         <v>109</v>
       </c>
-      <c r="C43" t="n">
-        <v>1</v>
-      </c>
       <c r="E43" t="inlineStr">
         <is>
           <t>0 = exclude</t>
@@ -6587,72 +4985,6 @@
       <c r="F43" t="inlineStr">
         <is>
           <t>3 = Non-individual level (team/firm/org analysis)</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Examines structural diversity and external knowledge sharing in 182 work groups across a global telecommunications company.</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Work Groups, Structural Diversity, and Knowledge Sharing in a Global Organization</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>Management Science</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Jonathon N. Cummings</t>
-        </is>
-      </c>
-      <c r="K43" t="n">
-        <v>2004</v>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>Jonathon N. Cummings (2004). Work Groups, Structural Diversity, and Knowledge Sharing in a Global Organization. Management Science.</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>0 = No</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>[Level of Analysis: Aggregated Data]. Verbatim Evidence: "[Qualitative and Quantitative Evidence] "There was at least one respondent from each work group, and responses were averaged across members and applied to the entire group." [Footnote 1] "Selection bias analyses were conducted at the group level of analysis (N = 182)." [Table 2] "Table 2 Correlation Matrix with Main Study Variables (N = 182 Work Groups)" [Sample] "Data used to test the above hypotheses (see Figure 1 for a complete model) come from a sample of 182 work groups and include (1) corporate database records, (2) 20 group interviews, (3) 182 surveys of group leaders, (4) 957 surveys of group members, and (5) senior executives’ ratings of group performance." [Preliminary Analyses] "Second, intraclass correlations justifying a group-level analysis were significant for intragroup and external knowledge sharing.""</t>
-        </is>
-      </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional design</t>
-        </is>
-      </c>
-      <c r="S43" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="U43" t="inlineStr">
-        <is>
-          <t>0 = Domestic</t>
-        </is>
-      </c>
-      <c r="V43" t="n">
-        <v>182</v>
-      </c>
-      <c r="Z43" t="inlineStr">
-        <is>
-          <t>Work group members / leaders</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Institutionalize Dual Missing Data Protocol (999 numeric / None text) across all rules, skills, and extraction data
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/70_94_109.xlsx
+++ b/03_Coding_Sheets/70_94_109.xlsx
@@ -743,10 +743,22 @@
       <c r="V4" t="n">
         <v>253</v>
       </c>
+      <c r="W4" t="n">
+        <v>999</v>
+      </c>
+      <c r="X4" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>999</v>
+      </c>
       <c r="Z4" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
+      </c>
+      <c r="AA4" t="n">
+        <v>999</v>
       </c>
       <c r="AB4" t="n">
         <v>7.5</v>
@@ -798,10 +810,28 @@
           <t>BSA</t>
         </is>
       </c>
+      <c r="AP4" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>999</v>
+      </c>
       <c r="AS4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
+      </c>
+      <c r="AT4" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>999</v>
       </c>
       <c r="AW4" t="n">
         <v>0.05</v>
@@ -847,10 +877,22 @@
       <c r="V5" t="n">
         <v>253</v>
       </c>
+      <c r="W5" t="n">
+        <v>999</v>
+      </c>
+      <c r="X5" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>999</v>
+      </c>
       <c r="Z5" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
+      </c>
+      <c r="AA5" t="n">
+        <v>999</v>
       </c>
       <c r="AB5" t="n">
         <v>7.5</v>
@@ -902,10 +944,28 @@
           <t>BSA</t>
         </is>
       </c>
+      <c r="AP5" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>999</v>
+      </c>
       <c r="AS5" t="inlineStr">
         <is>
           <t>Org. Size</t>
         </is>
+      </c>
+      <c r="AT5" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>999</v>
       </c>
       <c r="AW5" t="n">
         <v>0.03</v>
@@ -951,10 +1011,22 @@
       <c r="V6" t="n">
         <v>253</v>
       </c>
+      <c r="W6" t="n">
+        <v>999</v>
+      </c>
+      <c r="X6" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>999</v>
+      </c>
       <c r="Z6" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
+      </c>
+      <c r="AA6" t="n">
+        <v>999</v>
       </c>
       <c r="AB6" t="n">
         <v>7.5</v>
@@ -1006,10 +1078,28 @@
           <t>BSA</t>
         </is>
       </c>
+      <c r="AP6" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>999</v>
+      </c>
       <c r="AS6" t="inlineStr">
         <is>
           <t>Industry</t>
         </is>
+      </c>
+      <c r="AT6" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>999</v>
       </c>
       <c r="AW6" t="n">
         <v>0.02</v>
@@ -1055,10 +1145,22 @@
       <c r="V7" t="n">
         <v>253</v>
       </c>
+      <c r="W7" t="n">
+        <v>999</v>
+      </c>
+      <c r="X7" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>999</v>
+      </c>
       <c r="Z7" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
+      </c>
+      <c r="AA7" t="n">
+        <v>999</v>
       </c>
       <c r="AB7" t="n">
         <v>7.5</v>
@@ -1110,10 +1212,25 @@
           <t>BSA</t>
         </is>
       </c>
+      <c r="AP7" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>999</v>
+      </c>
       <c r="AS7" t="inlineStr">
         <is>
           <t>Org. Comm.</t>
         </is>
+      </c>
+      <c r="AT7" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>999</v>
       </c>
       <c r="AV7" t="n">
         <v>0.92</v>
@@ -1162,10 +1279,22 @@
       <c r="V8" t="n">
         <v>253</v>
       </c>
+      <c r="W8" t="n">
+        <v>999</v>
+      </c>
+      <c r="X8" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>999</v>
+      </c>
       <c r="Z8" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
+      </c>
+      <c r="AA8" t="n">
+        <v>999</v>
       </c>
       <c r="AB8" t="n">
         <v>7.5</v>
@@ -1217,10 +1346,25 @@
           <t>BSA</t>
         </is>
       </c>
+      <c r="AP8" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>999</v>
+      </c>
       <c r="AS8" t="inlineStr">
         <is>
           <t>Prof. Comm.</t>
         </is>
+      </c>
+      <c r="AT8" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>999</v>
       </c>
       <c r="AV8" t="n">
         <v>0.9</v>
@@ -1269,10 +1413,22 @@
       <c r="V9" t="n">
         <v>253</v>
       </c>
+      <c r="W9" t="n">
+        <v>999</v>
+      </c>
+      <c r="X9" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>999</v>
+      </c>
       <c r="Z9" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
+      </c>
+      <c r="AA9" t="n">
+        <v>999</v>
       </c>
       <c r="AB9" t="n">
         <v>7.5</v>
@@ -1295,6 +1451,15 @@
           <t>This was done by obtaining percentile ranking of subjects on intraunit and extraunit communication activity scores and using the mean of the two ranks as the boundary spanning score.</t>
         </is>
       </c>
+      <c r="AH9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>999</v>
+      </c>
       <c r="AK9" t="inlineStr">
         <is>
           <t>1 = Self-report</t>
@@ -1315,10 +1480,28 @@
           <t>BSA</t>
         </is>
       </c>
+      <c r="AP9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>999</v>
+      </c>
       <c r="AS9" t="inlineStr">
         <is>
           <t>Dual Comm.</t>
         </is>
+      </c>
+      <c r="AT9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>999</v>
       </c>
       <c r="AW9" t="n">
         <v>-0.1</v>
@@ -1364,10 +1547,22 @@
       <c r="V10" t="n">
         <v>253</v>
       </c>
+      <c r="W10" t="n">
+        <v>999</v>
+      </c>
+      <c r="X10" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>999</v>
+      </c>
       <c r="Z10" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
+      </c>
+      <c r="AA10" t="n">
+        <v>999</v>
       </c>
       <c r="AB10" t="n">
         <v>7.5</v>
@@ -1419,10 +1614,28 @@
           <t>BSA</t>
         </is>
       </c>
+      <c r="AP10" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>999</v>
+      </c>
       <c r="AS10" t="inlineStr">
         <is>
           <t>Complexity</t>
         </is>
+      </c>
+      <c r="AT10" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>999</v>
       </c>
       <c r="AW10" t="n">
         <v>-0.01</v>
@@ -1468,10 +1681,22 @@
       <c r="V11" t="n">
         <v>253</v>
       </c>
+      <c r="W11" t="n">
+        <v>999</v>
+      </c>
+      <c r="X11" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>999</v>
+      </c>
       <c r="Z11" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
+      </c>
+      <c r="AA11" t="n">
+        <v>999</v>
       </c>
       <c r="AB11" t="n">
         <v>7.5</v>
@@ -1523,10 +1748,25 @@
           <t>BSA</t>
         </is>
       </c>
+      <c r="AP11" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>999</v>
+      </c>
       <c r="AS11" t="inlineStr">
         <is>
           <t>Uncertainty</t>
         </is>
+      </c>
+      <c r="AT11" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>999</v>
       </c>
       <c r="AV11" t="n">
         <v>0.76</v>
@@ -1575,10 +1815,22 @@
       <c r="V12" t="n">
         <v>253</v>
       </c>
+      <c r="W12" t="n">
+        <v>999</v>
+      </c>
+      <c r="X12" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>999</v>
+      </c>
       <c r="Z12" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
+      </c>
+      <c r="AA12" t="n">
+        <v>999</v>
       </c>
       <c r="AB12" t="n">
         <v>7.5</v>
@@ -1630,10 +1882,25 @@
           <t>BSA</t>
         </is>
       </c>
+      <c r="AP12" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR12" t="n">
+        <v>999</v>
+      </c>
       <c r="AS12" t="inlineStr">
         <is>
           <t>Interdepend.</t>
         </is>
+      </c>
+      <c r="AT12" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>999</v>
       </c>
       <c r="AV12" t="n">
         <v>0.63</v>
@@ -1682,10 +1949,22 @@
       <c r="V13" t="n">
         <v>253</v>
       </c>
+      <c r="W13" t="n">
+        <v>999</v>
+      </c>
+      <c r="X13" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>999</v>
+      </c>
       <c r="Z13" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
+      </c>
+      <c r="AA13" t="n">
+        <v>999</v>
       </c>
       <c r="AB13" t="n">
         <v>7.5</v>
@@ -1737,10 +2016,28 @@
           <t>BSA</t>
         </is>
       </c>
+      <c r="AP13" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>999</v>
+      </c>
       <c r="AS13" t="inlineStr">
         <is>
           <t>Degree</t>
         </is>
+      </c>
+      <c r="AT13" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>999</v>
       </c>
       <c r="AW13" t="n">
         <v>-0.06</v>
@@ -1786,10 +2083,22 @@
       <c r="V14" t="n">
         <v>253</v>
       </c>
+      <c r="W14" t="n">
+        <v>999</v>
+      </c>
+      <c r="X14" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>999</v>
+      </c>
       <c r="Z14" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
+      </c>
+      <c r="AA14" t="n">
+        <v>999</v>
       </c>
       <c r="AB14" t="n">
         <v>7.5</v>
@@ -1841,10 +2150,28 @@
           <t>BSA</t>
         </is>
       </c>
+      <c r="AP14" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>999</v>
+      </c>
       <c r="AS14" t="inlineStr">
         <is>
           <t>Occupation</t>
         </is>
+      </c>
+      <c r="AT14" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>999</v>
       </c>
       <c r="AW14" t="n">
         <v>0.12</v>
@@ -1890,10 +2217,22 @@
       <c r="V15" t="n">
         <v>253</v>
       </c>
+      <c r="W15" t="n">
+        <v>999</v>
+      </c>
+      <c r="X15" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>999</v>
+      </c>
       <c r="Z15" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
+      </c>
+      <c r="AA15" t="n">
+        <v>999</v>
       </c>
       <c r="AB15" t="n">
         <v>7.5</v>
@@ -1945,10 +2284,25 @@
           <t>BSA</t>
         </is>
       </c>
+      <c r="AP15" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>999</v>
+      </c>
       <c r="AS15" t="inlineStr">
         <is>
           <t>Prof. Control</t>
         </is>
+      </c>
+      <c r="AT15" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU15" t="n">
+        <v>999</v>
       </c>
       <c r="AV15" t="n">
         <v>0.61</v>
@@ -1997,10 +2351,22 @@
       <c r="V16" t="n">
         <v>253</v>
       </c>
+      <c r="W16" t="n">
+        <v>999</v>
+      </c>
+      <c r="X16" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>999</v>
+      </c>
       <c r="Z16" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
         </is>
+      </c>
+      <c r="AA16" t="n">
+        <v>999</v>
       </c>
       <c r="AB16" t="n">
         <v>7.5</v>
@@ -2052,10 +2418,25 @@
           <t>BSA</t>
         </is>
       </c>
+      <c r="AP16" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR16" t="n">
+        <v>999</v>
+      </c>
       <c r="AS16" t="inlineStr">
         <is>
           <t>Prof. Incent.</t>
         </is>
+      </c>
+      <c r="AT16" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>999</v>
       </c>
       <c r="AV16" t="n">
         <v>0.72</v>
@@ -2104,6 +2485,15 @@
       <c r="V17" t="n">
         <v>253</v>
       </c>
+      <c r="W17" t="n">
+        <v>999</v>
+      </c>
+      <c r="X17" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>999</v>
+      </c>
       <c r="Z17" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -2162,10 +2552,28 @@
           <t>External Com.</t>
         </is>
       </c>
+      <c r="AP17" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR17" t="n">
+        <v>999</v>
+      </c>
       <c r="AS17" t="inlineStr">
         <is>
           <t>Internal Com.</t>
         </is>
+      </c>
+      <c r="AT17" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU17" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV17" t="n">
+        <v>999</v>
       </c>
       <c r="AW17" t="n">
         <v>0.1</v>
@@ -2211,6 +2619,15 @@
       <c r="V18" t="n">
         <v>253</v>
       </c>
+      <c r="W18" t="n">
+        <v>999</v>
+      </c>
+      <c r="X18" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>999</v>
+      </c>
       <c r="Z18" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -2269,10 +2686,28 @@
           <t>External Com.</t>
         </is>
       </c>
+      <c r="AP18" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ18" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR18" t="n">
+        <v>999</v>
+      </c>
       <c r="AS18" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
+      </c>
+      <c r="AT18" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU18" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV18" t="n">
+        <v>999</v>
       </c>
       <c r="AW18" t="n">
         <v>0.11</v>
@@ -2318,6 +2753,15 @@
       <c r="V19" t="n">
         <v>253</v>
       </c>
+      <c r="W19" t="n">
+        <v>999</v>
+      </c>
+      <c r="X19" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>999</v>
+      </c>
       <c r="Z19" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -2376,10 +2820,28 @@
           <t>External Com.</t>
         </is>
       </c>
+      <c r="AP19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR19" t="n">
+        <v>999</v>
+      </c>
       <c r="AS19" t="inlineStr">
         <is>
           <t>Org. Size</t>
         </is>
+      </c>
+      <c r="AT19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV19" t="n">
+        <v>999</v>
       </c>
       <c r="AW19" t="n">
         <v>-0.05</v>
@@ -2425,6 +2887,15 @@
       <c r="V20" t="n">
         <v>253</v>
       </c>
+      <c r="W20" t="n">
+        <v>999</v>
+      </c>
+      <c r="X20" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>999</v>
+      </c>
       <c r="Z20" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -2483,10 +2954,28 @@
           <t>External Com.</t>
         </is>
       </c>
+      <c r="AP20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR20" t="n">
+        <v>999</v>
+      </c>
       <c r="AS20" t="inlineStr">
         <is>
           <t>Industry</t>
         </is>
+      </c>
+      <c r="AT20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV20" t="n">
+        <v>999</v>
       </c>
       <c r="AW20" t="n">
         <v>-0.21</v>
@@ -2532,6 +3021,15 @@
       <c r="V21" t="n">
         <v>253</v>
       </c>
+      <c r="W21" t="n">
+        <v>999</v>
+      </c>
+      <c r="X21" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>999</v>
+      </c>
       <c r="Z21" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -2590,10 +3088,25 @@
           <t>External Com.</t>
         </is>
       </c>
+      <c r="AP21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR21" t="n">
+        <v>999</v>
+      </c>
       <c r="AS21" t="inlineStr">
         <is>
           <t>Org. Comm.</t>
         </is>
+      </c>
+      <c r="AT21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU21" t="n">
+        <v>999</v>
       </c>
       <c r="AV21" t="n">
         <v>0.92</v>
@@ -2642,6 +3155,15 @@
       <c r="V22" t="n">
         <v>253</v>
       </c>
+      <c r="W22" t="n">
+        <v>999</v>
+      </c>
+      <c r="X22" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>999</v>
+      </c>
       <c r="Z22" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -2700,10 +3222,25 @@
           <t>External Com.</t>
         </is>
       </c>
+      <c r="AP22" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR22" t="n">
+        <v>999</v>
+      </c>
       <c r="AS22" t="inlineStr">
         <is>
           <t>Prof. Comm.</t>
         </is>
+      </c>
+      <c r="AT22" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU22" t="n">
+        <v>999</v>
       </c>
       <c r="AV22" t="n">
         <v>0.9</v>
@@ -2752,6 +3289,15 @@
       <c r="V23" t="n">
         <v>253</v>
       </c>
+      <c r="W23" t="n">
+        <v>999</v>
+      </c>
+      <c r="X23" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>999</v>
+      </c>
       <c r="Z23" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -2781,6 +3327,15 @@
           <t>Extraunit communication frequency was measured by asking subjects to report frequency of work-related communication on a six-point scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day) with each of 12 categories of individuals over the past month.</t>
         </is>
       </c>
+      <c r="AH23" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ23" t="n">
+        <v>999</v>
+      </c>
       <c r="AK23" t="inlineStr">
         <is>
           <t>1 = Self-report</t>
@@ -2801,10 +3356,28 @@
           <t>External Com.</t>
         </is>
       </c>
+      <c r="AP23" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ23" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR23" t="n">
+        <v>999</v>
+      </c>
       <c r="AS23" t="inlineStr">
         <is>
           <t>Dual Comm.</t>
         </is>
+      </c>
+      <c r="AT23" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU23" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV23" t="n">
+        <v>999</v>
       </c>
       <c r="AW23" t="n">
         <v>-0.05</v>
@@ -2850,6 +3423,15 @@
       <c r="V24" t="n">
         <v>253</v>
       </c>
+      <c r="W24" t="n">
+        <v>999</v>
+      </c>
+      <c r="X24" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>999</v>
+      </c>
       <c r="Z24" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -2908,10 +3490,28 @@
           <t>External Com.</t>
         </is>
       </c>
+      <c r="AP24" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR24" t="n">
+        <v>999</v>
+      </c>
       <c r="AS24" t="inlineStr">
         <is>
           <t>Complexity</t>
         </is>
+      </c>
+      <c r="AT24" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU24" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV24" t="n">
+        <v>999</v>
       </c>
       <c r="AW24" t="n">
         <v>0.1</v>
@@ -2957,6 +3557,15 @@
       <c r="V25" t="n">
         <v>253</v>
       </c>
+      <c r="W25" t="n">
+        <v>999</v>
+      </c>
+      <c r="X25" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>999</v>
+      </c>
       <c r="Z25" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -3015,10 +3624,25 @@
           <t>External Com.</t>
         </is>
       </c>
+      <c r="AP25" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ25" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR25" t="n">
+        <v>999</v>
+      </c>
       <c r="AS25" t="inlineStr">
         <is>
           <t>Uncertainty</t>
         </is>
+      </c>
+      <c r="AT25" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU25" t="n">
+        <v>999</v>
       </c>
       <c r="AV25" t="n">
         <v>0.76</v>
@@ -3067,6 +3691,15 @@
       <c r="V26" t="n">
         <v>253</v>
       </c>
+      <c r="W26" t="n">
+        <v>999</v>
+      </c>
+      <c r="X26" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>999</v>
+      </c>
       <c r="Z26" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -3125,10 +3758,25 @@
           <t>External Com.</t>
         </is>
       </c>
+      <c r="AP26" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ26" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR26" t="n">
+        <v>999</v>
+      </c>
       <c r="AS26" t="inlineStr">
         <is>
           <t>Interdepend.</t>
         </is>
+      </c>
+      <c r="AT26" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU26" t="n">
+        <v>999</v>
       </c>
       <c r="AV26" t="n">
         <v>0.63</v>
@@ -3177,6 +3825,15 @@
       <c r="V27" t="n">
         <v>253</v>
       </c>
+      <c r="W27" t="n">
+        <v>999</v>
+      </c>
+      <c r="X27" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>999</v>
+      </c>
       <c r="Z27" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -3235,10 +3892,28 @@
           <t>External Com.</t>
         </is>
       </c>
+      <c r="AP27" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ27" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR27" t="n">
+        <v>999</v>
+      </c>
       <c r="AS27" t="inlineStr">
         <is>
           <t>Degree</t>
         </is>
+      </c>
+      <c r="AT27" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU27" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV27" t="n">
+        <v>999</v>
       </c>
       <c r="AW27" t="n">
         <v>0.17</v>
@@ -3284,6 +3959,15 @@
       <c r="V28" t="n">
         <v>253</v>
       </c>
+      <c r="W28" t="n">
+        <v>999</v>
+      </c>
+      <c r="X28" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>999</v>
+      </c>
       <c r="Z28" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -3342,10 +4026,28 @@
           <t>External Com.</t>
         </is>
       </c>
+      <c r="AP28" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ28" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR28" t="n">
+        <v>999</v>
+      </c>
       <c r="AS28" t="inlineStr">
         <is>
           <t>Occupation</t>
         </is>
+      </c>
+      <c r="AT28" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU28" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV28" t="n">
+        <v>999</v>
       </c>
       <c r="AW28" t="n">
         <v>-0.13</v>
@@ -3391,6 +4093,15 @@
       <c r="V29" t="n">
         <v>253</v>
       </c>
+      <c r="W29" t="n">
+        <v>999</v>
+      </c>
+      <c r="X29" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>999</v>
+      </c>
       <c r="Z29" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -3449,10 +4160,25 @@
           <t>External Com.</t>
         </is>
       </c>
+      <c r="AP29" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ29" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR29" t="n">
+        <v>999</v>
+      </c>
       <c r="AS29" t="inlineStr">
         <is>
           <t>Prof. Control</t>
         </is>
+      </c>
+      <c r="AT29" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU29" t="n">
+        <v>999</v>
       </c>
       <c r="AV29" t="n">
         <v>0.61</v>
@@ -3501,6 +4227,15 @@
       <c r="V30" t="n">
         <v>253</v>
       </c>
+      <c r="W30" t="n">
+        <v>999</v>
+      </c>
+      <c r="X30" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>999</v>
+      </c>
       <c r="Z30" t="inlineStr">
         <is>
           <t>R&amp;D technical professionals</t>
@@ -3559,10 +4294,25 @@
           <t>External Com.</t>
         </is>
       </c>
+      <c r="AP30" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ30" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR30" t="n">
+        <v>999</v>
+      </c>
       <c r="AS30" t="inlineStr">
         <is>
           <t>Prof. Incent.</t>
         </is>
+      </c>
+      <c r="AT30" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU30" t="n">
+        <v>999</v>
       </c>
       <c r="AV30" t="n">
         <v>0.72</v>
@@ -3611,9 +4361,15 @@
       <c r="V31" t="n">
         <v>382</v>
       </c>
+      <c r="W31" t="n">
+        <v>999</v>
+      </c>
       <c r="X31" t="n">
         <v>65.2</v>
       </c>
+      <c r="Y31" t="n">
+        <v>999</v>
+      </c>
       <c r="Z31" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -3672,6 +4428,12 @@
           <t>External Representation</t>
         </is>
       </c>
+      <c r="AP31" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>999</v>
+      </c>
       <c r="AR31" t="n">
         <v>0.871</v>
       </c>
@@ -3679,6 +4441,12 @@
         <is>
           <t>Role Conflict</t>
         </is>
+      </c>
+      <c r="AT31" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>999</v>
       </c>
       <c r="AV31" t="n">
         <v>0.619</v>
@@ -3727,9 +4495,15 @@
       <c r="V32" t="n">
         <v>382</v>
       </c>
+      <c r="W32" t="n">
+        <v>999</v>
+      </c>
       <c r="X32" t="n">
         <v>65.2</v>
       </c>
+      <c r="Y32" t="n">
+        <v>999</v>
+      </c>
       <c r="Z32" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -3788,6 +4562,12 @@
           <t>External Representation</t>
         </is>
       </c>
+      <c r="AP32" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>999</v>
+      </c>
       <c r="AR32" t="n">
         <v>0.871</v>
       </c>
@@ -3795,6 +4575,12 @@
         <is>
           <t>Role Ambiguity</t>
         </is>
+      </c>
+      <c r="AT32" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU32" t="n">
+        <v>999</v>
       </c>
       <c r="AV32" t="n">
         <v>0.777</v>
@@ -3843,9 +4629,15 @@
       <c r="V33" t="n">
         <v>382</v>
       </c>
+      <c r="W33" t="n">
+        <v>999</v>
+      </c>
       <c r="X33" t="n">
         <v>65.2</v>
       </c>
+      <c r="Y33" t="n">
+        <v>999</v>
+      </c>
       <c r="Z33" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -3904,6 +4696,12 @@
           <t>External Representation</t>
         </is>
       </c>
+      <c r="AP33" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ33" t="n">
+        <v>999</v>
+      </c>
       <c r="AR33" t="n">
         <v>0.871</v>
       </c>
@@ -3911,6 +4709,12 @@
         <is>
           <t>Proactive Personality</t>
         </is>
+      </c>
+      <c r="AT33" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU33" t="n">
+        <v>999</v>
       </c>
       <c r="AV33" t="n">
         <v>0.894</v>
@@ -3959,9 +4763,15 @@
       <c r="V34" t="n">
         <v>382</v>
       </c>
+      <c r="W34" t="n">
+        <v>999</v>
+      </c>
       <c r="X34" t="n">
         <v>65.2</v>
       </c>
+      <c r="Y34" t="n">
+        <v>999</v>
+      </c>
       <c r="Z34" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -4020,6 +4830,12 @@
           <t>External Representation</t>
         </is>
       </c>
+      <c r="AP34" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ34" t="n">
+        <v>999</v>
+      </c>
       <c r="AR34" t="n">
         <v>0.871</v>
       </c>
@@ -4027,6 +4843,12 @@
         <is>
           <t>Employee Creativity</t>
         </is>
+      </c>
+      <c r="AT34" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU34" t="n">
+        <v>999</v>
       </c>
       <c r="AV34" t="n">
         <v>0.839</v>
@@ -4075,9 +4897,15 @@
       <c r="V35" t="n">
         <v>382</v>
       </c>
+      <c r="W35" t="n">
+        <v>999</v>
+      </c>
       <c r="X35" t="n">
         <v>65.2</v>
       </c>
+      <c r="Y35" t="n">
+        <v>999</v>
+      </c>
       <c r="Z35" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -4136,6 +4964,12 @@
           <t>Internal Influence</t>
         </is>
       </c>
+      <c r="AP35" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ35" t="n">
+        <v>999</v>
+      </c>
       <c r="AR35" t="n">
         <v>0.872</v>
       </c>
@@ -4143,6 +4977,12 @@
         <is>
           <t>Role Conflict</t>
         </is>
+      </c>
+      <c r="AT35" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU35" t="n">
+        <v>999</v>
       </c>
       <c r="AV35" t="n">
         <v>0.619</v>
@@ -4191,9 +5031,15 @@
       <c r="V36" t="n">
         <v>382</v>
       </c>
+      <c r="W36" t="n">
+        <v>999</v>
+      </c>
       <c r="X36" t="n">
         <v>65.2</v>
       </c>
+      <c r="Y36" t="n">
+        <v>999</v>
+      </c>
       <c r="Z36" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -4252,6 +5098,12 @@
           <t>Internal Influence</t>
         </is>
       </c>
+      <c r="AP36" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ36" t="n">
+        <v>999</v>
+      </c>
       <c r="AR36" t="n">
         <v>0.872</v>
       </c>
@@ -4259,6 +5111,12 @@
         <is>
           <t>Role Ambiguity</t>
         </is>
+      </c>
+      <c r="AT36" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU36" t="n">
+        <v>999</v>
       </c>
       <c r="AV36" t="n">
         <v>0.777</v>
@@ -4307,9 +5165,15 @@
       <c r="V37" t="n">
         <v>382</v>
       </c>
+      <c r="W37" t="n">
+        <v>999</v>
+      </c>
       <c r="X37" t="n">
         <v>65.2</v>
       </c>
+      <c r="Y37" t="n">
+        <v>999</v>
+      </c>
       <c r="Z37" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -4368,6 +5232,12 @@
           <t>Internal Influence</t>
         </is>
       </c>
+      <c r="AP37" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ37" t="n">
+        <v>999</v>
+      </c>
       <c r="AR37" t="n">
         <v>0.872</v>
       </c>
@@ -4375,6 +5245,12 @@
         <is>
           <t>Proactive Personality</t>
         </is>
+      </c>
+      <c r="AT37" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU37" t="n">
+        <v>999</v>
       </c>
       <c r="AV37" t="n">
         <v>0.894</v>
@@ -4423,9 +5299,15 @@
       <c r="V38" t="n">
         <v>382</v>
       </c>
+      <c r="W38" t="n">
+        <v>999</v>
+      </c>
       <c r="X38" t="n">
         <v>65.2</v>
       </c>
+      <c r="Y38" t="n">
+        <v>999</v>
+      </c>
       <c r="Z38" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -4484,6 +5366,12 @@
           <t>Internal Influence</t>
         </is>
       </c>
+      <c r="AP38" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ38" t="n">
+        <v>999</v>
+      </c>
       <c r="AR38" t="n">
         <v>0.872</v>
       </c>
@@ -4491,6 +5379,12 @@
         <is>
           <t>Employee Creativity</t>
         </is>
+      </c>
+      <c r="AT38" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU38" t="n">
+        <v>999</v>
       </c>
       <c r="AV38" t="n">
         <v>0.839</v>
@@ -4539,9 +5433,15 @@
       <c r="V39" t="n">
         <v>382</v>
       </c>
+      <c r="W39" t="n">
+        <v>999</v>
+      </c>
       <c r="X39" t="n">
         <v>65.2</v>
       </c>
+      <c r="Y39" t="n">
+        <v>999</v>
+      </c>
       <c r="Z39" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -4600,6 +5500,12 @@
           <t>Service Delivery</t>
         </is>
       </c>
+      <c r="AP39" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ39" t="n">
+        <v>999</v>
+      </c>
       <c r="AR39" t="n">
         <v>0.876</v>
       </c>
@@ -4607,6 +5513,12 @@
         <is>
           <t>Role Conflict</t>
         </is>
+      </c>
+      <c r="AT39" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU39" t="n">
+        <v>999</v>
       </c>
       <c r="AV39" t="n">
         <v>0.619</v>
@@ -4655,9 +5567,15 @@
       <c r="V40" t="n">
         <v>382</v>
       </c>
+      <c r="W40" t="n">
+        <v>999</v>
+      </c>
       <c r="X40" t="n">
         <v>65.2</v>
       </c>
+      <c r="Y40" t="n">
+        <v>999</v>
+      </c>
       <c r="Z40" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -4716,6 +5634,12 @@
           <t>Service Delivery</t>
         </is>
       </c>
+      <c r="AP40" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ40" t="n">
+        <v>999</v>
+      </c>
       <c r="AR40" t="n">
         <v>0.876</v>
       </c>
@@ -4723,6 +5647,12 @@
         <is>
           <t>Role Ambiguity</t>
         </is>
+      </c>
+      <c r="AT40" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU40" t="n">
+        <v>999</v>
       </c>
       <c r="AV40" t="n">
         <v>0.777</v>
@@ -4771,9 +5701,15 @@
       <c r="V41" t="n">
         <v>382</v>
       </c>
+      <c r="W41" t="n">
+        <v>999</v>
+      </c>
       <c r="X41" t="n">
         <v>65.2</v>
       </c>
+      <c r="Y41" t="n">
+        <v>999</v>
+      </c>
       <c r="Z41" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -4832,6 +5768,12 @@
           <t>Service Delivery</t>
         </is>
       </c>
+      <c r="AP41" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ41" t="n">
+        <v>999</v>
+      </c>
       <c r="AR41" t="n">
         <v>0.876</v>
       </c>
@@ -4839,6 +5781,12 @@
         <is>
           <t>Proactive Personality</t>
         </is>
+      </c>
+      <c r="AT41" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU41" t="n">
+        <v>999</v>
       </c>
       <c r="AV41" t="n">
         <v>0.894</v>
@@ -4887,9 +5835,15 @@
       <c r="V42" t="n">
         <v>382</v>
       </c>
+      <c r="W42" t="n">
+        <v>999</v>
+      </c>
       <c r="X42" t="n">
         <v>65.2</v>
       </c>
+      <c r="Y42" t="n">
+        <v>999</v>
+      </c>
       <c r="Z42" t="inlineStr">
         <is>
           <t>Hotel frontline service employees</t>
@@ -4948,6 +5902,12 @@
           <t>Service Delivery</t>
         </is>
       </c>
+      <c r="AP42" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ42" t="n">
+        <v>999</v>
+      </c>
       <c r="AR42" t="n">
         <v>0.876</v>
       </c>
@@ -4955,6 +5915,12 @@
         <is>
           <t>Employee Creativity</t>
         </is>
+      </c>
+      <c r="AT42" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU42" t="n">
+        <v>999</v>
       </c>
       <c r="AV42" t="n">
         <v>0.839</v>

</xml_diff>

<commit_message>
Fix Mean and SD data mapping for Paper 70 and Paper 94 in 70_94_109.xlsx
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/70_94_109.xlsx
+++ b/03_Coding_Sheets/70_94_109.xlsx
@@ -744,13 +744,13 @@
         <v>253</v>
       </c>
       <c r="W4" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X4" t="n">
         <v>999</v>
       </c>
       <c r="Y4" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -811,10 +811,10 @@
         </is>
       </c>
       <c r="AP4" t="n">
-        <v>999</v>
+        <v>50.51</v>
       </c>
       <c r="AQ4" t="n">
-        <v>999</v>
+        <v>21.54</v>
       </c>
       <c r="AR4" t="n">
         <v>999</v>
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="AT4" t="n">
-        <v>999</v>
+        <v>2.94</v>
       </c>
       <c r="AU4" t="n">
-        <v>999</v>
+        <v>1.08</v>
       </c>
       <c r="AV4" t="n">
         <v>999</v>
@@ -878,13 +878,13 @@
         <v>253</v>
       </c>
       <c r="W5" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X5" t="n">
         <v>999</v>
       </c>
       <c r="Y5" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
@@ -945,10 +945,10 @@
         </is>
       </c>
       <c r="AP5" t="n">
-        <v>999</v>
+        <v>50.51</v>
       </c>
       <c r="AQ5" t="n">
-        <v>999</v>
+        <v>21.54</v>
       </c>
       <c r="AR5" t="n">
         <v>999</v>
@@ -959,10 +959,10 @@
         </is>
       </c>
       <c r="AT5" t="n">
-        <v>999</v>
+        <v>2.58</v>
       </c>
       <c r="AU5" t="n">
-        <v>999</v>
+        <v>0.66</v>
       </c>
       <c r="AV5" t="n">
         <v>999</v>
@@ -1012,13 +1012,13 @@
         <v>253</v>
       </c>
       <c r="W6" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X6" t="n">
         <v>999</v>
       </c>
       <c r="Y6" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1079,10 +1079,10 @@
         </is>
       </c>
       <c r="AP6" t="n">
-        <v>999</v>
+        <v>50.51</v>
       </c>
       <c r="AQ6" t="n">
-        <v>999</v>
+        <v>21.54</v>
       </c>
       <c r="AR6" t="n">
         <v>999</v>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="AT6" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="AU6" t="n">
-        <v>999</v>
+        <v>0.49</v>
       </c>
       <c r="AV6" t="n">
         <v>999</v>
@@ -1146,13 +1146,13 @@
         <v>253</v>
       </c>
       <c r="W7" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X7" t="n">
         <v>999</v>
       </c>
       <c r="Y7" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
@@ -1213,10 +1213,10 @@
         </is>
       </c>
       <c r="AP7" t="n">
-        <v>999</v>
+        <v>50.51</v>
       </c>
       <c r="AQ7" t="n">
-        <v>999</v>
+        <v>21.54</v>
       </c>
       <c r="AR7" t="n">
         <v>999</v>
@@ -1227,10 +1227,10 @@
         </is>
       </c>
       <c r="AT7" t="n">
-        <v>999</v>
+        <v>5.06</v>
       </c>
       <c r="AU7" t="n">
-        <v>999</v>
+        <v>1.24</v>
       </c>
       <c r="AV7" t="n">
         <v>0.92</v>
@@ -1280,13 +1280,13 @@
         <v>253</v>
       </c>
       <c r="W8" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X8" t="n">
         <v>999</v>
       </c>
       <c r="Y8" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         </is>
       </c>
       <c r="AP8" t="n">
-        <v>999</v>
+        <v>50.51</v>
       </c>
       <c r="AQ8" t="n">
-        <v>999</v>
+        <v>21.54</v>
       </c>
       <c r="AR8" t="n">
         <v>999</v>
@@ -1361,10 +1361,10 @@
         </is>
       </c>
       <c r="AT8" t="n">
-        <v>999</v>
+        <v>5.23</v>
       </c>
       <c r="AU8" t="n">
-        <v>999</v>
+        <v>1.06</v>
       </c>
       <c r="AV8" t="n">
         <v>0.9</v>
@@ -1414,13 +1414,13 @@
         <v>253</v>
       </c>
       <c r="W9" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X9" t="n">
         <v>999</v>
       </c>
       <c r="Y9" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
@@ -1481,10 +1481,10 @@
         </is>
       </c>
       <c r="AP9" t="n">
-        <v>999</v>
+        <v>50.51</v>
       </c>
       <c r="AQ9" t="n">
-        <v>999</v>
+        <v>21.54</v>
       </c>
       <c r="AR9" t="n">
         <v>999</v>
@@ -1495,10 +1495,10 @@
         </is>
       </c>
       <c r="AT9" t="n">
-        <v>999</v>
+        <v>27.07</v>
       </c>
       <c r="AU9" t="n">
-        <v>999</v>
+        <v>10.03</v>
       </c>
       <c r="AV9" t="n">
         <v>999</v>
@@ -1548,13 +1548,13 @@
         <v>253</v>
       </c>
       <c r="W10" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X10" t="n">
         <v>999</v>
       </c>
       <c r="Y10" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -1615,10 +1615,10 @@
         </is>
       </c>
       <c r="AP10" t="n">
-        <v>999</v>
+        <v>50.51</v>
       </c>
       <c r="AQ10" t="n">
-        <v>999</v>
+        <v>21.54</v>
       </c>
       <c r="AR10" t="n">
         <v>999</v>
@@ -1629,10 +1629,10 @@
         </is>
       </c>
       <c r="AT10" t="n">
-        <v>999</v>
+        <v>53.33</v>
       </c>
       <c r="AU10" t="n">
-        <v>999</v>
+        <v>14.67</v>
       </c>
       <c r="AV10" t="n">
         <v>999</v>
@@ -1682,13 +1682,13 @@
         <v>253</v>
       </c>
       <c r="W11" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X11" t="n">
         <v>999</v>
       </c>
       <c r="Y11" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
@@ -1749,10 +1749,10 @@
         </is>
       </c>
       <c r="AP11" t="n">
-        <v>999</v>
+        <v>50.51</v>
       </c>
       <c r="AQ11" t="n">
-        <v>999</v>
+        <v>21.54</v>
       </c>
       <c r="AR11" t="n">
         <v>999</v>
@@ -1763,10 +1763,10 @@
         </is>
       </c>
       <c r="AT11" t="n">
-        <v>999</v>
+        <v>5.2</v>
       </c>
       <c r="AU11" t="n">
-        <v>999</v>
+        <v>1.1</v>
       </c>
       <c r="AV11" t="n">
         <v>0.76</v>
@@ -1816,13 +1816,13 @@
         <v>253</v>
       </c>
       <c r="W12" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X12" t="n">
         <v>999</v>
       </c>
       <c r="Y12" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
@@ -1883,10 +1883,10 @@
         </is>
       </c>
       <c r="AP12" t="n">
-        <v>999</v>
+        <v>50.51</v>
       </c>
       <c r="AQ12" t="n">
-        <v>999</v>
+        <v>21.54</v>
       </c>
       <c r="AR12" t="n">
         <v>999</v>
@@ -1897,10 +1897,10 @@
         </is>
       </c>
       <c r="AT12" t="n">
-        <v>999</v>
+        <v>3.53</v>
       </c>
       <c r="AU12" t="n">
-        <v>999</v>
+        <v>1.36</v>
       </c>
       <c r="AV12" t="n">
         <v>0.63</v>
@@ -1950,13 +1950,13 @@
         <v>253</v>
       </c>
       <c r="W13" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X13" t="n">
         <v>999</v>
       </c>
       <c r="Y13" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -2017,10 +2017,10 @@
         </is>
       </c>
       <c r="AP13" t="n">
-        <v>999</v>
+        <v>50.51</v>
       </c>
       <c r="AQ13" t="n">
-        <v>999</v>
+        <v>21.54</v>
       </c>
       <c r="AR13" t="n">
         <v>999</v>
@@ -2031,10 +2031,10 @@
         </is>
       </c>
       <c r="AT13" t="n">
-        <v>999</v>
+        <v>2.58</v>
       </c>
       <c r="AU13" t="n">
-        <v>999</v>
+        <v>1.17</v>
       </c>
       <c r="AV13" t="n">
         <v>999</v>
@@ -2084,13 +2084,13 @@
         <v>253</v>
       </c>
       <c r="W14" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X14" t="n">
         <v>999</v>
       </c>
       <c r="Y14" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
@@ -2151,10 +2151,10 @@
         </is>
       </c>
       <c r="AP14" t="n">
-        <v>999</v>
+        <v>50.51</v>
       </c>
       <c r="AQ14" t="n">
-        <v>999</v>
+        <v>21.54</v>
       </c>
       <c r="AR14" t="n">
         <v>999</v>
@@ -2165,10 +2165,10 @@
         </is>
       </c>
       <c r="AT14" t="n">
-        <v>999</v>
+        <v>1.83</v>
       </c>
       <c r="AU14" t="n">
-        <v>999</v>
+        <v>0.54</v>
       </c>
       <c r="AV14" t="n">
         <v>999</v>
@@ -2218,13 +2218,13 @@
         <v>253</v>
       </c>
       <c r="W15" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X15" t="n">
         <v>999</v>
       </c>
       <c r="Y15" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
@@ -2285,10 +2285,10 @@
         </is>
       </c>
       <c r="AP15" t="n">
-        <v>999</v>
+        <v>50.51</v>
       </c>
       <c r="AQ15" t="n">
-        <v>999</v>
+        <v>21.54</v>
       </c>
       <c r="AR15" t="n">
         <v>999</v>
@@ -2299,10 +2299,10 @@
         </is>
       </c>
       <c r="AT15" t="n">
-        <v>999</v>
+        <v>3.28</v>
       </c>
       <c r="AU15" t="n">
-        <v>999</v>
+        <v>1.25</v>
       </c>
       <c r="AV15" t="n">
         <v>0.61</v>
@@ -2352,13 +2352,13 @@
         <v>253</v>
       </c>
       <c r="W16" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X16" t="n">
         <v>999</v>
       </c>
       <c r="Y16" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2419,10 +2419,10 @@
         </is>
       </c>
       <c r="AP16" t="n">
-        <v>999</v>
+        <v>50.51</v>
       </c>
       <c r="AQ16" t="n">
-        <v>999</v>
+        <v>21.54</v>
       </c>
       <c r="AR16" t="n">
         <v>999</v>
@@ -2433,10 +2433,10 @@
         </is>
       </c>
       <c r="AT16" t="n">
-        <v>999</v>
+        <v>4.08</v>
       </c>
       <c r="AU16" t="n">
-        <v>999</v>
+        <v>1.34</v>
       </c>
       <c r="AV16" t="n">
         <v>0.72</v>
@@ -2486,13 +2486,13 @@
         <v>253</v>
       </c>
       <c r="W17" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X17" t="n">
         <v>999</v>
       </c>
       <c r="Y17" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
@@ -2553,10 +2553,10 @@
         </is>
       </c>
       <c r="AP17" t="n">
-        <v>999</v>
+        <v>0.19</v>
       </c>
       <c r="AQ17" t="n">
-        <v>999</v>
+        <v>0.12</v>
       </c>
       <c r="AR17" t="n">
         <v>999</v>
@@ -2567,10 +2567,10 @@
         </is>
       </c>
       <c r="AT17" t="n">
-        <v>999</v>
+        <v>2.19</v>
       </c>
       <c r="AU17" t="n">
-        <v>999</v>
+        <v>1.02</v>
       </c>
       <c r="AV17" t="n">
         <v>999</v>
@@ -2620,13 +2620,13 @@
         <v>253</v>
       </c>
       <c r="W18" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X18" t="n">
         <v>999</v>
       </c>
       <c r="Y18" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
@@ -2687,10 +2687,10 @@
         </is>
       </c>
       <c r="AP18" t="n">
-        <v>999</v>
+        <v>0.19</v>
       </c>
       <c r="AQ18" t="n">
-        <v>999</v>
+        <v>0.12</v>
       </c>
       <c r="AR18" t="n">
         <v>999</v>
@@ -2701,10 +2701,10 @@
         </is>
       </c>
       <c r="AT18" t="n">
-        <v>999</v>
+        <v>2.94</v>
       </c>
       <c r="AU18" t="n">
-        <v>999</v>
+        <v>1.08</v>
       </c>
       <c r="AV18" t="n">
         <v>999</v>
@@ -2754,13 +2754,13 @@
         <v>253</v>
       </c>
       <c r="W19" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X19" t="n">
         <v>999</v>
       </c>
       <c r="Y19" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
@@ -2821,10 +2821,10 @@
         </is>
       </c>
       <c r="AP19" t="n">
-        <v>999</v>
+        <v>0.19</v>
       </c>
       <c r="AQ19" t="n">
-        <v>999</v>
+        <v>0.12</v>
       </c>
       <c r="AR19" t="n">
         <v>999</v>
@@ -2835,10 +2835,10 @@
         </is>
       </c>
       <c r="AT19" t="n">
-        <v>999</v>
+        <v>2.58</v>
       </c>
       <c r="AU19" t="n">
-        <v>999</v>
+        <v>0.66</v>
       </c>
       <c r="AV19" t="n">
         <v>999</v>
@@ -2888,13 +2888,13 @@
         <v>253</v>
       </c>
       <c r="W20" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X20" t="n">
         <v>999</v>
       </c>
       <c r="Y20" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
@@ -2955,10 +2955,10 @@
         </is>
       </c>
       <c r="AP20" t="n">
-        <v>999</v>
+        <v>0.19</v>
       </c>
       <c r="AQ20" t="n">
-        <v>999</v>
+        <v>0.12</v>
       </c>
       <c r="AR20" t="n">
         <v>999</v>
@@ -2969,10 +2969,10 @@
         </is>
       </c>
       <c r="AT20" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="AU20" t="n">
-        <v>999</v>
+        <v>0.49</v>
       </c>
       <c r="AV20" t="n">
         <v>999</v>
@@ -3022,13 +3022,13 @@
         <v>253</v>
       </c>
       <c r="W21" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X21" t="n">
         <v>999</v>
       </c>
       <c r="Y21" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
@@ -3089,10 +3089,10 @@
         </is>
       </c>
       <c r="AP21" t="n">
-        <v>999</v>
+        <v>0.19</v>
       </c>
       <c r="AQ21" t="n">
-        <v>999</v>
+        <v>0.12</v>
       </c>
       <c r="AR21" t="n">
         <v>999</v>
@@ -3103,10 +3103,10 @@
         </is>
       </c>
       <c r="AT21" t="n">
-        <v>999</v>
+        <v>5.06</v>
       </c>
       <c r="AU21" t="n">
-        <v>999</v>
+        <v>1.24</v>
       </c>
       <c r="AV21" t="n">
         <v>0.92</v>
@@ -3156,13 +3156,13 @@
         <v>253</v>
       </c>
       <c r="W22" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X22" t="n">
         <v>999</v>
       </c>
       <c r="Y22" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -3223,10 +3223,10 @@
         </is>
       </c>
       <c r="AP22" t="n">
-        <v>999</v>
+        <v>0.19</v>
       </c>
       <c r="AQ22" t="n">
-        <v>999</v>
+        <v>0.12</v>
       </c>
       <c r="AR22" t="n">
         <v>999</v>
@@ -3237,10 +3237,10 @@
         </is>
       </c>
       <c r="AT22" t="n">
-        <v>999</v>
+        <v>5.23</v>
       </c>
       <c r="AU22" t="n">
-        <v>999</v>
+        <v>1.06</v>
       </c>
       <c r="AV22" t="n">
         <v>0.9</v>
@@ -3290,13 +3290,13 @@
         <v>253</v>
       </c>
       <c r="W23" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X23" t="n">
         <v>999</v>
       </c>
       <c r="Y23" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -3357,10 +3357,10 @@
         </is>
       </c>
       <c r="AP23" t="n">
-        <v>999</v>
+        <v>0.19</v>
       </c>
       <c r="AQ23" t="n">
-        <v>999</v>
+        <v>0.12</v>
       </c>
       <c r="AR23" t="n">
         <v>999</v>
@@ -3371,10 +3371,10 @@
         </is>
       </c>
       <c r="AT23" t="n">
-        <v>999</v>
+        <v>27.07</v>
       </c>
       <c r="AU23" t="n">
-        <v>999</v>
+        <v>10.03</v>
       </c>
       <c r="AV23" t="n">
         <v>999</v>
@@ -3424,13 +3424,13 @@
         <v>253</v>
       </c>
       <c r="W24" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X24" t="n">
         <v>999</v>
       </c>
       <c r="Y24" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
@@ -3491,10 +3491,10 @@
         </is>
       </c>
       <c r="AP24" t="n">
-        <v>999</v>
+        <v>0.19</v>
       </c>
       <c r="AQ24" t="n">
-        <v>999</v>
+        <v>0.12</v>
       </c>
       <c r="AR24" t="n">
         <v>999</v>
@@ -3505,10 +3505,10 @@
         </is>
       </c>
       <c r="AT24" t="n">
-        <v>999</v>
+        <v>53.33</v>
       </c>
       <c r="AU24" t="n">
-        <v>999</v>
+        <v>14.67</v>
       </c>
       <c r="AV24" t="n">
         <v>999</v>
@@ -3558,13 +3558,13 @@
         <v>253</v>
       </c>
       <c r="W25" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X25" t="n">
         <v>999</v>
       </c>
       <c r="Y25" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
@@ -3625,10 +3625,10 @@
         </is>
       </c>
       <c r="AP25" t="n">
-        <v>999</v>
+        <v>0.19</v>
       </c>
       <c r="AQ25" t="n">
-        <v>999</v>
+        <v>0.12</v>
       </c>
       <c r="AR25" t="n">
         <v>999</v>
@@ -3639,10 +3639,10 @@
         </is>
       </c>
       <c r="AT25" t="n">
-        <v>999</v>
+        <v>5.2</v>
       </c>
       <c r="AU25" t="n">
-        <v>999</v>
+        <v>1.1</v>
       </c>
       <c r="AV25" t="n">
         <v>0.76</v>
@@ -3692,13 +3692,13 @@
         <v>253</v>
       </c>
       <c r="W26" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X26" t="n">
         <v>999</v>
       </c>
       <c r="Y26" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
@@ -3759,10 +3759,10 @@
         </is>
       </c>
       <c r="AP26" t="n">
-        <v>999</v>
+        <v>0.19</v>
       </c>
       <c r="AQ26" t="n">
-        <v>999</v>
+        <v>0.12</v>
       </c>
       <c r="AR26" t="n">
         <v>999</v>
@@ -3773,10 +3773,10 @@
         </is>
       </c>
       <c r="AT26" t="n">
-        <v>999</v>
+        <v>3.53</v>
       </c>
       <c r="AU26" t="n">
-        <v>999</v>
+        <v>1.36</v>
       </c>
       <c r="AV26" t="n">
         <v>0.63</v>
@@ -3826,13 +3826,13 @@
         <v>253</v>
       </c>
       <c r="W27" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X27" t="n">
         <v>999</v>
       </c>
       <c r="Y27" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
@@ -3893,10 +3893,10 @@
         </is>
       </c>
       <c r="AP27" t="n">
-        <v>999</v>
+        <v>0.19</v>
       </c>
       <c r="AQ27" t="n">
-        <v>999</v>
+        <v>0.12</v>
       </c>
       <c r="AR27" t="n">
         <v>999</v>
@@ -3907,10 +3907,10 @@
         </is>
       </c>
       <c r="AT27" t="n">
-        <v>999</v>
+        <v>2.58</v>
       </c>
       <c r="AU27" t="n">
-        <v>999</v>
+        <v>1.17</v>
       </c>
       <c r="AV27" t="n">
         <v>999</v>
@@ -3960,13 +3960,13 @@
         <v>253</v>
       </c>
       <c r="W28" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X28" t="n">
         <v>999</v>
       </c>
       <c r="Y28" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
@@ -4027,10 +4027,10 @@
         </is>
       </c>
       <c r="AP28" t="n">
-        <v>999</v>
+        <v>0.19</v>
       </c>
       <c r="AQ28" t="n">
-        <v>999</v>
+        <v>0.12</v>
       </c>
       <c r="AR28" t="n">
         <v>999</v>
@@ -4041,10 +4041,10 @@
         </is>
       </c>
       <c r="AT28" t="n">
-        <v>999</v>
+        <v>1.83</v>
       </c>
       <c r="AU28" t="n">
-        <v>999</v>
+        <v>0.54</v>
       </c>
       <c r="AV28" t="n">
         <v>999</v>
@@ -4094,13 +4094,13 @@
         <v>253</v>
       </c>
       <c r="W29" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X29" t="n">
         <v>999</v>
       </c>
       <c r="Y29" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
@@ -4161,10 +4161,10 @@
         </is>
       </c>
       <c r="AP29" t="n">
-        <v>999</v>
+        <v>0.19</v>
       </c>
       <c r="AQ29" t="n">
-        <v>999</v>
+        <v>0.12</v>
       </c>
       <c r="AR29" t="n">
         <v>999</v>
@@ -4175,10 +4175,10 @@
         </is>
       </c>
       <c r="AT29" t="n">
-        <v>999</v>
+        <v>3.28</v>
       </c>
       <c r="AU29" t="n">
-        <v>999</v>
+        <v>1.25</v>
       </c>
       <c r="AV29" t="n">
         <v>0.61</v>
@@ -4228,13 +4228,13 @@
         <v>253</v>
       </c>
       <c r="W30" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X30" t="n">
         <v>999</v>
       </c>
       <c r="Y30" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
@@ -4295,10 +4295,10 @@
         </is>
       </c>
       <c r="AP30" t="n">
-        <v>999</v>
+        <v>0.19</v>
       </c>
       <c r="AQ30" t="n">
-        <v>999</v>
+        <v>0.12</v>
       </c>
       <c r="AR30" t="n">
         <v>999</v>
@@ -4309,10 +4309,10 @@
         </is>
       </c>
       <c r="AT30" t="n">
-        <v>999</v>
+        <v>4.08</v>
       </c>
       <c r="AU30" t="n">
-        <v>999</v>
+        <v>1.34</v>
       </c>
       <c r="AV30" t="n">
         <v>0.72</v>
@@ -4429,10 +4429,10 @@
         </is>
       </c>
       <c r="AP31" t="n">
-        <v>999</v>
+        <v>5.46</v>
       </c>
       <c r="AQ31" t="n">
-        <v>999</v>
+        <v>0.8</v>
       </c>
       <c r="AR31" t="n">
         <v>0.871</v>
@@ -4443,10 +4443,10 @@
         </is>
       </c>
       <c r="AT31" t="n">
-        <v>999</v>
+        <v>3.35</v>
       </c>
       <c r="AU31" t="n">
-        <v>999</v>
+        <v>0.93</v>
       </c>
       <c r="AV31" t="n">
         <v>0.619</v>
@@ -4563,10 +4563,10 @@
         </is>
       </c>
       <c r="AP32" t="n">
-        <v>999</v>
+        <v>5.46</v>
       </c>
       <c r="AQ32" t="n">
-        <v>999</v>
+        <v>0.8</v>
       </c>
       <c r="AR32" t="n">
         <v>0.871</v>
@@ -4577,10 +4577,10 @@
         </is>
       </c>
       <c r="AT32" t="n">
-        <v>999</v>
+        <v>2.86</v>
       </c>
       <c r="AU32" t="n">
-        <v>999</v>
+        <v>1.11</v>
       </c>
       <c r="AV32" t="n">
         <v>0.777</v>
@@ -4697,10 +4697,10 @@
         </is>
       </c>
       <c r="AP33" t="n">
-        <v>999</v>
+        <v>5.46</v>
       </c>
       <c r="AQ33" t="n">
-        <v>999</v>
+        <v>0.8</v>
       </c>
       <c r="AR33" t="n">
         <v>0.871</v>
@@ -4711,10 +4711,10 @@
         </is>
       </c>
       <c r="AT33" t="n">
-        <v>999</v>
+        <v>2.88</v>
       </c>
       <c r="AU33" t="n">
-        <v>999</v>
+        <v>1.1</v>
       </c>
       <c r="AV33" t="n">
         <v>0.894</v>
@@ -4831,10 +4831,10 @@
         </is>
       </c>
       <c r="AP34" t="n">
-        <v>999</v>
+        <v>5.46</v>
       </c>
       <c r="AQ34" t="n">
-        <v>999</v>
+        <v>0.8</v>
       </c>
       <c r="AR34" t="n">
         <v>0.871</v>
@@ -4845,10 +4845,10 @@
         </is>
       </c>
       <c r="AT34" t="n">
-        <v>999</v>
+        <v>5.68</v>
       </c>
       <c r="AU34" t="n">
-        <v>999</v>
+        <v>0.86</v>
       </c>
       <c r="AV34" t="n">
         <v>0.839</v>
@@ -4965,10 +4965,10 @@
         </is>
       </c>
       <c r="AP35" t="n">
-        <v>999</v>
+        <v>5.63</v>
       </c>
       <c r="AQ35" t="n">
-        <v>999</v>
+        <v>0.88</v>
       </c>
       <c r="AR35" t="n">
         <v>0.872</v>
@@ -4979,10 +4979,10 @@
         </is>
       </c>
       <c r="AT35" t="n">
-        <v>999</v>
+        <v>3.35</v>
       </c>
       <c r="AU35" t="n">
-        <v>999</v>
+        <v>0.93</v>
       </c>
       <c r="AV35" t="n">
         <v>0.619</v>
@@ -5099,10 +5099,10 @@
         </is>
       </c>
       <c r="AP36" t="n">
-        <v>999</v>
+        <v>5.63</v>
       </c>
       <c r="AQ36" t="n">
-        <v>999</v>
+        <v>0.88</v>
       </c>
       <c r="AR36" t="n">
         <v>0.872</v>
@@ -5113,10 +5113,10 @@
         </is>
       </c>
       <c r="AT36" t="n">
-        <v>999</v>
+        <v>2.86</v>
       </c>
       <c r="AU36" t="n">
-        <v>999</v>
+        <v>1.11</v>
       </c>
       <c r="AV36" t="n">
         <v>0.777</v>
@@ -5233,10 +5233,10 @@
         </is>
       </c>
       <c r="AP37" t="n">
-        <v>999</v>
+        <v>5.63</v>
       </c>
       <c r="AQ37" t="n">
-        <v>999</v>
+        <v>0.88</v>
       </c>
       <c r="AR37" t="n">
         <v>0.872</v>
@@ -5247,10 +5247,10 @@
         </is>
       </c>
       <c r="AT37" t="n">
-        <v>999</v>
+        <v>2.88</v>
       </c>
       <c r="AU37" t="n">
-        <v>999</v>
+        <v>1.1</v>
       </c>
       <c r="AV37" t="n">
         <v>0.894</v>
@@ -5367,10 +5367,10 @@
         </is>
       </c>
       <c r="AP38" t="n">
-        <v>999</v>
+        <v>5.63</v>
       </c>
       <c r="AQ38" t="n">
-        <v>999</v>
+        <v>0.88</v>
       </c>
       <c r="AR38" t="n">
         <v>0.872</v>
@@ -5381,10 +5381,10 @@
         </is>
       </c>
       <c r="AT38" t="n">
-        <v>999</v>
+        <v>5.68</v>
       </c>
       <c r="AU38" t="n">
-        <v>999</v>
+        <v>0.86</v>
       </c>
       <c r="AV38" t="n">
         <v>0.839</v>
@@ -5501,10 +5501,10 @@
         </is>
       </c>
       <c r="AP39" t="n">
-        <v>999</v>
+        <v>5.81</v>
       </c>
       <c r="AQ39" t="n">
-        <v>999</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="AR39" t="n">
         <v>0.876</v>
@@ -5515,10 +5515,10 @@
         </is>
       </c>
       <c r="AT39" t="n">
-        <v>999</v>
+        <v>3.35</v>
       </c>
       <c r="AU39" t="n">
-        <v>999</v>
+        <v>0.93</v>
       </c>
       <c r="AV39" t="n">
         <v>0.619</v>
@@ -5635,10 +5635,10 @@
         </is>
       </c>
       <c r="AP40" t="n">
-        <v>999</v>
+        <v>5.81</v>
       </c>
       <c r="AQ40" t="n">
-        <v>999</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="AR40" t="n">
         <v>0.876</v>
@@ -5649,10 +5649,10 @@
         </is>
       </c>
       <c r="AT40" t="n">
-        <v>999</v>
+        <v>2.86</v>
       </c>
       <c r="AU40" t="n">
-        <v>999</v>
+        <v>1.11</v>
       </c>
       <c r="AV40" t="n">
         <v>0.777</v>
@@ -5769,10 +5769,10 @@
         </is>
       </c>
       <c r="AP41" t="n">
-        <v>999</v>
+        <v>5.81</v>
       </c>
       <c r="AQ41" t="n">
-        <v>999</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="AR41" t="n">
         <v>0.876</v>
@@ -5783,10 +5783,10 @@
         </is>
       </c>
       <c r="AT41" t="n">
-        <v>999</v>
+        <v>2.88</v>
       </c>
       <c r="AU41" t="n">
-        <v>999</v>
+        <v>1.1</v>
       </c>
       <c r="AV41" t="n">
         <v>0.894</v>
@@ -5903,10 +5903,10 @@
         </is>
       </c>
       <c r="AP42" t="n">
-        <v>999</v>
+        <v>5.81</v>
       </c>
       <c r="AQ42" t="n">
-        <v>999</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="AR42" t="n">
         <v>0.876</v>
@@ -5917,10 +5917,10 @@
         </is>
       </c>
       <c r="AT42" t="n">
-        <v>999</v>
+        <v>5.68</v>
       </c>
       <c r="AU42" t="n">
-        <v>999</v>
+        <v>0.86</v>
       </c>
       <c r="AV42" t="n">
         <v>0.839</v>

</xml_diff>

<commit_message>
feat(p70): elevate Internal Com. to 3rd BSB dimension per gatekeeper model and expand Cartesian pairings to 39 rows
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/70_94_109.xlsx
+++ b/03_Coding_Sheets/70_94_109.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX43"/>
+  <dimension ref="A1:AX55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1638,11 +1638,11 @@
         <v>999</v>
       </c>
       <c r="AW10" t="n">
-        <v>-0.01</v>
+        <v>0.03</v>
       </c>
       <c r="AX10" t="inlineStr">
         <is>
-          <t>Table 3.9 (p. 65), Row: 13. Complexity, Col: 1, Raw: -.01 | Global composite: [Methodology, p. 147] "This was done by obtaining percentile ranking of subjects on intraunit and extraunit communication activity scores and using the mean of the two ranks as the boundary spanning score."</t>
+          <t>Table 3.9 (p. 65), Row: 13. Complexity, Col: 1, Raw: .03 | Global composite: [Methodology, p. 147] "This was done by obtaining percentile ranking of subjects on intraunit and extraunit communication activity scores and using the mean of the two ranks as the boundary spanning score."</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2527,7 @@
         <v>1</v>
       </c>
       <c r="AI17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ17" t="n">
         <v>5</v>
@@ -2539,12 +2539,12 @@
       </c>
       <c r="AM17" t="inlineStr">
         <is>
-          <t>Intraunit communication frequency</t>
+          <t>job title</t>
         </is>
       </c>
       <c r="AN17" t="inlineStr">
         <is>
-          <t>Subjects were asked about communication frequency within the last month with every other technical professional in the unit, using a 6-point Likert-type scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day).</t>
+          <t>For the purposes of this study, the large number of categorical values reported for job title were collapsed into 5 values, ranging from associate member (1) to manager (5).</t>
         </is>
       </c>
       <c r="AO17" t="inlineStr">
@@ -2563,24 +2563,24 @@
       </c>
       <c r="AS17" t="inlineStr">
         <is>
-          <t>Internal Com.</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="AT17" t="n">
-        <v>2.19</v>
+        <v>2.94</v>
       </c>
       <c r="AU17" t="n">
-        <v>1.02</v>
+        <v>1.08</v>
       </c>
       <c r="AV17" t="n">
         <v>999</v>
       </c>
       <c r="AW17" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="AX17" t="inlineStr">
         <is>
-          <t>Table 3.9 (p. 65), Row: 3. External Com., Col: 2, Raw: .10</t>
+          <t>Table 3.9 (p. 65), Row: 7. Status, Col: 3, Raw: .11</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2664,7 @@
         <v>1</v>
       </c>
       <c r="AJ18" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AK18" t="inlineStr">
         <is>
@@ -2673,12 +2673,12 @@
       </c>
       <c r="AM18" t="inlineStr">
         <is>
-          <t>job title</t>
+          <t>Organizational size</t>
         </is>
       </c>
       <c r="AN18" t="inlineStr">
         <is>
-          <t>For the purposes of this study, the large number of categorical values reported for job title were collapsed into 5 values, ranging from associate member (1) to manager (5).</t>
+          <t>Organizations were ranked from 1 (small) to 3 (large)</t>
         </is>
       </c>
       <c r="AO18" t="inlineStr">
@@ -2697,24 +2697,24 @@
       </c>
       <c r="AS18" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Org. Size</t>
         </is>
       </c>
       <c r="AT18" t="n">
-        <v>2.94</v>
+        <v>2.58</v>
       </c>
       <c r="AU18" t="n">
-        <v>1.08</v>
+        <v>0.66</v>
       </c>
       <c r="AV18" t="n">
         <v>999</v>
       </c>
       <c r="AW18" t="n">
-        <v>0.11</v>
+        <v>-0.05</v>
       </c>
       <c r="AX18" t="inlineStr">
         <is>
-          <t>Table 3.9 (p. 65), Row: 7. Status, Col: 3, Raw: .11</t>
+          <t>Table 3.9 (p. 65), Row: 8. Org. Size, Col: 3, Raw: -.05</t>
         </is>
       </c>
     </row>
@@ -2795,10 +2795,10 @@
         <v>1</v>
       </c>
       <c r="AI19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AK19" t="inlineStr">
         <is>
@@ -2807,12 +2807,12 @@
       </c>
       <c r="AM19" t="inlineStr">
         <is>
-          <t>Organizational size</t>
+          <t>dichotomous variable</t>
         </is>
       </c>
       <c r="AN19" t="inlineStr">
         <is>
-          <t>Organizations were ranked from 1 (small) to 3 (large)</t>
+          <t>Because the majority of the sample (62 per cent) was engaged in research related to the microelectronics industry, it was decided to create a dichotomous variable to control for structural differences.</t>
         </is>
       </c>
       <c r="AO19" t="inlineStr">
@@ -2831,24 +2831,24 @@
       </c>
       <c r="AS19" t="inlineStr">
         <is>
-          <t>Org. Size</t>
+          <t>Industry</t>
         </is>
       </c>
       <c r="AT19" t="n">
-        <v>2.58</v>
+        <v>0.62</v>
       </c>
       <c r="AU19" t="n">
-        <v>0.66</v>
+        <v>0.49</v>
       </c>
       <c r="AV19" t="n">
         <v>999</v>
       </c>
       <c r="AW19" t="n">
-        <v>-0.05</v>
+        <v>-0.23</v>
       </c>
       <c r="AX19" t="inlineStr">
         <is>
-          <t>Table 3.9 (p. 65), Row: 8. Org. Size, Col: 3, Raw: -.05</t>
+          <t>Table 3.9 (p. 65), Row: 9. Industry, Col: 3, Raw: -.23**</t>
         </is>
       </c>
     </row>
@@ -2926,13 +2926,13 @@
         </is>
       </c>
       <c r="AH20" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="AI20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ20" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="AK20" t="inlineStr">
         <is>
@@ -2941,12 +2941,12 @@
       </c>
       <c r="AM20" t="inlineStr">
         <is>
-          <t>dichotomous variable</t>
+          <t>Organizational Commitment Questionnaire</t>
         </is>
       </c>
       <c r="AN20" t="inlineStr">
         <is>
-          <t>Because the majority of the sample (62 per cent) was engaged in research related to the microelectronics industry, it was decided to create a dichotomous variable to control for structural differences.</t>
+          <t>A 9-item short form was used (Angle &amp; Perry, 1981).</t>
         </is>
       </c>
       <c r="AO20" t="inlineStr">
@@ -2965,24 +2965,24 @@
       </c>
       <c r="AS20" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>Org. Comm.</t>
         </is>
       </c>
       <c r="AT20" t="n">
-        <v>0.62</v>
+        <v>5.06</v>
       </c>
       <c r="AU20" t="n">
-        <v>0.49</v>
+        <v>1.24</v>
       </c>
       <c r="AV20" t="n">
-        <v>999</v>
+        <v>0.92</v>
       </c>
       <c r="AW20" t="n">
-        <v>-0.21</v>
+        <v>0.09</v>
       </c>
       <c r="AX20" t="inlineStr">
         <is>
-          <t>Table 3.9 (p. 65), Row: 9. Industry, Col: 3, Raw: -.21**</t>
+          <t>Table 3.9 (p. 65), Row: 10. Org. Comm., Col: 3, Raw: .09</t>
         </is>
       </c>
     </row>
@@ -3075,12 +3075,12 @@
       </c>
       <c r="AM21" t="inlineStr">
         <is>
-          <t>Organizational Commitment Questionnaire</t>
+          <t>format similar to the OCQ</t>
         </is>
       </c>
       <c r="AN21" t="inlineStr">
         <is>
-          <t>A 9-item short form was used (Angle &amp; Perry, 1981).</t>
+          <t>Both sets of commitment items were measured using a 7-point Likert-type scale from 1=strongly disagree to 7=strongly agree.</t>
         </is>
       </c>
       <c r="AO21" t="inlineStr">
@@ -3099,24 +3099,24 @@
       </c>
       <c r="AS21" t="inlineStr">
         <is>
-          <t>Org. Comm.</t>
+          <t>Prof. Comm.</t>
         </is>
       </c>
       <c r="AT21" t="n">
-        <v>5.06</v>
+        <v>5.23</v>
       </c>
       <c r="AU21" t="n">
-        <v>1.24</v>
+        <v>1.06</v>
       </c>
       <c r="AV21" t="n">
-        <v>0.92</v>
+        <v>0.9</v>
       </c>
       <c r="AW21" t="n">
-        <v>0.09</v>
+        <v>0.03</v>
       </c>
       <c r="AX21" t="inlineStr">
         <is>
-          <t>Table 3.9 (p. 65), Row: 10. Org. Comm., Col: 3, Raw: .09</t>
+          <t>Table 3.9 (p. 65), Row: 11. Prof. Comm., Col: 3, Raw: .03</t>
         </is>
       </c>
     </row>
@@ -3194,13 +3194,13 @@
         </is>
       </c>
       <c r="AH22" t="n">
-        <v>9</v>
+        <v>999</v>
       </c>
       <c r="AI22" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="AJ22" t="n">
-        <v>7</v>
+        <v>999</v>
       </c>
       <c r="AK22" t="inlineStr">
         <is>
@@ -3209,12 +3209,12 @@
       </c>
       <c r="AM22" t="inlineStr">
         <is>
-          <t>format similar to the OCQ</t>
+          <t>interaction variable</t>
         </is>
       </c>
       <c r="AN22" t="inlineStr">
         <is>
-          <t>Both sets of commitment items were measured using a 7-point Likert-type scale from 1=strongly disagree to 7=strongly agree.</t>
+          <t>An interaction variable was created from the cross product of organizational commitment and professional commitment mean scale scores.</t>
         </is>
       </c>
       <c r="AO22" t="inlineStr">
@@ -3233,24 +3233,24 @@
       </c>
       <c r="AS22" t="inlineStr">
         <is>
-          <t>Prof. Comm.</t>
+          <t>Dual Comm.</t>
         </is>
       </c>
       <c r="AT22" t="n">
-        <v>5.23</v>
+        <v>27.07</v>
       </c>
       <c r="AU22" t="n">
-        <v>1.06</v>
+        <v>10.03</v>
       </c>
       <c r="AV22" t="n">
-        <v>0.9</v>
+        <v>999</v>
       </c>
       <c r="AW22" t="n">
-        <v>0.03</v>
+        <v>-0.05</v>
       </c>
       <c r="AX22" t="inlineStr">
         <is>
-          <t>Table 3.9 (p. 65), Row: 11. Prof. Comm., Col: 3, Raw: .03</t>
+          <t>Table 3.9 (p. 65), Row: 12. Dual Comm., Col: 3, Raw: -.05</t>
         </is>
       </c>
     </row>
@@ -3328,13 +3328,13 @@
         </is>
       </c>
       <c r="AH23" t="n">
-        <v>999</v>
+        <v>4</v>
       </c>
       <c r="AI23" t="n">
-        <v>999</v>
+        <v>25</v>
       </c>
       <c r="AJ23" t="n">
-        <v>999</v>
+        <v>100</v>
       </c>
       <c r="AK23" t="inlineStr">
         <is>
@@ -3343,12 +3343,12 @@
       </c>
       <c r="AM23" t="inlineStr">
         <is>
-          <t>interaction variable</t>
+          <t>weighted sum of the percentages</t>
         </is>
       </c>
       <c r="AN23" t="inlineStr">
         <is>
-          <t>An interaction variable was created from the cross product of organizational commitment and professional commitment mean scale scores.</t>
+          <t>Subjects were asked to indicate what percentage of their work falls into each of four categories.</t>
         </is>
       </c>
       <c r="AO23" t="inlineStr">
@@ -3367,24 +3367,24 @@
       </c>
       <c r="AS23" t="inlineStr">
         <is>
-          <t>Dual Comm.</t>
+          <t>Complexity</t>
         </is>
       </c>
       <c r="AT23" t="n">
-        <v>27.07</v>
+        <v>53.33</v>
       </c>
       <c r="AU23" t="n">
-        <v>10.03</v>
+        <v>14.67</v>
       </c>
       <c r="AV23" t="n">
         <v>999</v>
       </c>
       <c r="AW23" t="n">
-        <v>-0.05</v>
+        <v>0.1</v>
       </c>
       <c r="AX23" t="inlineStr">
         <is>
-          <t>Table 3.9 (p. 65), Row: 12. Dual Comm., Col: 3, Raw: -.05</t>
+          <t>Table 3.9 (p. 65), Row: 13. Complexity, Col: 3, Raw: .10</t>
         </is>
       </c>
     </row>
@@ -3462,13 +3462,13 @@
         </is>
       </c>
       <c r="AH24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AI24" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="AJ24" t="n">
-        <v>100</v>
+        <v>7</v>
       </c>
       <c r="AK24" t="inlineStr">
         <is>
@@ -3477,12 +3477,12 @@
       </c>
       <c r="AM24" t="inlineStr">
         <is>
-          <t>weighted sum of the percentages</t>
+          <t>three-item scale</t>
         </is>
       </c>
       <c r="AN24" t="inlineStr">
         <is>
-          <t>Subjects were asked to indicate what percentage of their work falls into each of four categories.</t>
+          <t>A three-item scale was constructed and asked subjects to rate the extent of change of their task requirements on a seven-point scale ranging from 1 (almost no change) to 7 (constantly changing).</t>
         </is>
       </c>
       <c r="AO24" t="inlineStr">
@@ -3501,24 +3501,24 @@
       </c>
       <c r="AS24" t="inlineStr">
         <is>
-          <t>Complexity</t>
+          <t>Uncertainty</t>
         </is>
       </c>
       <c r="AT24" t="n">
-        <v>53.33</v>
+        <v>5.2</v>
       </c>
       <c r="AU24" t="n">
-        <v>14.67</v>
+        <v>1.1</v>
       </c>
       <c r="AV24" t="n">
-        <v>999</v>
+        <v>0.76</v>
       </c>
       <c r="AW24" t="n">
-        <v>0.1</v>
+        <v>0.19</v>
       </c>
       <c r="AX24" t="inlineStr">
         <is>
-          <t>Table 3.9 (p. 65), Row: 13. Complexity, Col: 3, Raw: .10</t>
+          <t>Table 3.9 (p. 65), Row: 14. Uncertainty, Col: 3, Raw: .19**</t>
         </is>
       </c>
     </row>
@@ -3611,12 +3611,12 @@
       </c>
       <c r="AM25" t="inlineStr">
         <is>
-          <t>three-item scale</t>
+          <t>Extraproject Coordination scale</t>
         </is>
       </c>
       <c r="AN25" t="inlineStr">
         <is>
-          <t>A three-item scale was constructed and asked subjects to rate the extent of change of their task requirements on a seven-point scale ranging from 1 (almost no change) to 7 (constantly changing).</t>
+          <t>The decision was made to delete the intraproject coordination item.</t>
         </is>
       </c>
       <c r="AO25" t="inlineStr">
@@ -3635,24 +3635,24 @@
       </c>
       <c r="AS25" t="inlineStr">
         <is>
-          <t>Uncertainty</t>
+          <t>Interdepend.</t>
         </is>
       </c>
       <c r="AT25" t="n">
-        <v>5.2</v>
+        <v>3.53</v>
       </c>
       <c r="AU25" t="n">
-        <v>1.1</v>
+        <v>1.36</v>
       </c>
       <c r="AV25" t="n">
-        <v>0.76</v>
+        <v>0.63</v>
       </c>
       <c r="AW25" t="n">
-        <v>0.19</v>
+        <v>0.27</v>
       </c>
       <c r="AX25" t="inlineStr">
         <is>
-          <t>Table 3.9 (p. 65), Row: 14. Uncertainty, Col: 3, Raw: .19**</t>
+          <t>Table 3.9 (p. 65), Row: 15. Interdepend., Col: 3, Raw: .27**</t>
         </is>
       </c>
     </row>
@@ -3730,13 +3730,13 @@
         </is>
       </c>
       <c r="AH26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AI26" t="n">
         <v>1</v>
       </c>
       <c r="AJ26" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AK26" t="inlineStr">
         <is>
@@ -3745,12 +3745,12 @@
       </c>
       <c r="AM26" t="inlineStr">
         <is>
-          <t>Extraproject Coordination scale</t>
+          <t>highest degree attained</t>
         </is>
       </c>
       <c r="AN26" t="inlineStr">
         <is>
-          <t>The decision was made to delete the intraproject coordination item.</t>
+          <t>In addition, individual variables of highest degree attained and profession were used to indicate the individual's level of professionalization.</t>
         </is>
       </c>
       <c r="AO26" t="inlineStr">
@@ -3769,24 +3769,24 @@
       </c>
       <c r="AS26" t="inlineStr">
         <is>
-          <t>Interdepend.</t>
+          <t>Degree</t>
         </is>
       </c>
       <c r="AT26" t="n">
-        <v>3.53</v>
+        <v>2.58</v>
       </c>
       <c r="AU26" t="n">
-        <v>1.36</v>
+        <v>1.17</v>
       </c>
       <c r="AV26" t="n">
-        <v>0.63</v>
+        <v>999</v>
       </c>
       <c r="AW26" t="n">
-        <v>0.27</v>
+        <v>0.17</v>
       </c>
       <c r="AX26" t="inlineStr">
         <is>
-          <t>Table 3.9 (p. 65), Row: 15. Interdepend., Col: 3, Raw: .27**</t>
+          <t>Table 3.9 (p. 65), Row: 16. Degree, Col: 3, Raw: .17**</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
         <v>1</v>
       </c>
       <c r="AJ27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AK27" t="inlineStr">
         <is>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="AM27" t="inlineStr">
         <is>
-          <t>highest degree attained</t>
+          <t>profession</t>
         </is>
       </c>
       <c r="AN27" t="inlineStr">
@@ -3903,24 +3903,24 @@
       </c>
       <c r="AS27" t="inlineStr">
         <is>
-          <t>Degree</t>
+          <t>Occupation</t>
         </is>
       </c>
       <c r="AT27" t="n">
-        <v>2.58</v>
+        <v>1.83</v>
       </c>
       <c r="AU27" t="n">
-        <v>1.17</v>
+        <v>0.54</v>
       </c>
       <c r="AV27" t="n">
         <v>999</v>
       </c>
       <c r="AW27" t="n">
-        <v>0.17</v>
+        <v>-0.13</v>
       </c>
       <c r="AX27" t="inlineStr">
         <is>
-          <t>Table 3.9 (p. 65), Row: 16. Degree, Col: 3, Raw: .17**</t>
+          <t>Table 3.9 (p. 65), Row: 17. Occupation, Col: 3, Raw: -.13*</t>
         </is>
       </c>
     </row>
@@ -3998,13 +3998,13 @@
         </is>
       </c>
       <c r="AH28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI28" t="n">
         <v>1</v>
       </c>
       <c r="AJ28" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AK28" t="inlineStr">
         <is>
@@ -4013,12 +4013,12 @@
       </c>
       <c r="AM28" t="inlineStr">
         <is>
-          <t>profession</t>
+          <t>Professional Control</t>
         </is>
       </c>
       <c r="AN28" t="inlineStr">
         <is>
-          <t>In addition, individual variables of highest degree attained and profession were used to indicate the individual's level of professionalization.</t>
+          <t>The estimate of scale reliability for each of these scales was .61 for Professional Control and .32 for Autonomy.</t>
         </is>
       </c>
       <c r="AO28" t="inlineStr">
@@ -4037,24 +4037,24 @@
       </c>
       <c r="AS28" t="inlineStr">
         <is>
-          <t>Occupation</t>
+          <t>Prof. Control</t>
         </is>
       </c>
       <c r="AT28" t="n">
-        <v>1.83</v>
+        <v>3.28</v>
       </c>
       <c r="AU28" t="n">
-        <v>0.54</v>
+        <v>1.25</v>
       </c>
       <c r="AV28" t="n">
-        <v>999</v>
+        <v>0.61</v>
       </c>
       <c r="AW28" t="n">
-        <v>-0.13</v>
+        <v>0.13</v>
       </c>
       <c r="AX28" t="inlineStr">
         <is>
-          <t>Table 3.9 (p. 65), Row: 17. Occupation, Col: 3, Raw: -.13*</t>
+          <t>Table 3.9 (p. 65), Row: 18. Prof. Control, Col: 3, Raw: .13*</t>
         </is>
       </c>
     </row>
@@ -4132,7 +4132,7 @@
         </is>
       </c>
       <c r="AH29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AI29" t="n">
         <v>1</v>
@@ -4147,12 +4147,12 @@
       </c>
       <c r="AM29" t="inlineStr">
         <is>
-          <t>Professional Control</t>
+          <t>Professional Incentives</t>
         </is>
       </c>
       <c r="AN29" t="inlineStr">
         <is>
-          <t>The estimate of scale reliability for each of these scales was .61 for Professional Control and .32 for Autonomy.</t>
+          <t>The first factor, labeled "Professional Incentives" was straightforward: the underlying construct is organizational adoption of professional values.</t>
         </is>
       </c>
       <c r="AO29" t="inlineStr">
@@ -4171,24 +4171,24 @@
       </c>
       <c r="AS29" t="inlineStr">
         <is>
-          <t>Prof. Control</t>
+          <t>Prof. Incent.</t>
         </is>
       </c>
       <c r="AT29" t="n">
-        <v>3.28</v>
+        <v>4.08</v>
       </c>
       <c r="AU29" t="n">
-        <v>1.25</v>
+        <v>1.34</v>
       </c>
       <c r="AV29" t="n">
-        <v>0.61</v>
+        <v>0.72</v>
       </c>
       <c r="AW29" t="n">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="AX29" t="inlineStr">
         <is>
-          <t>Table 3.9 (p. 65), Row: 18. Prof. Control, Col: 3, Raw: .13*</t>
+          <t>Table 3.9 (p. 65), Row: 19. Prof. Incent., Col: 3, Raw: .11</t>
         </is>
       </c>
     </row>
@@ -4242,7 +4242,7 @@
         </is>
       </c>
       <c r="AA30" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AB30" t="n">
         <v>0</v>
@@ -4257,22 +4257,22 @@
       </c>
       <c r="AF30" t="inlineStr">
         <is>
-          <t>Extraunit communication frequency</t>
+          <t>Intraunit communication frequency</t>
         </is>
       </c>
       <c r="AG30" t="inlineStr">
         <is>
-          <t>Extraunit communication frequency was measured by asking subjects to report frequency of work-related communication on a six-point scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day) with each of 12 categories of individuals over the past month.</t>
+          <t>Subjects were asked about communication frequency within the last month with every other technical professional in the unit, using a 6-point Likert-type scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day).</t>
         </is>
       </c>
       <c r="AH30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AI30" t="n">
         <v>1</v>
       </c>
       <c r="AJ30" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AK30" t="inlineStr">
         <is>
@@ -4281,48 +4281,48 @@
       </c>
       <c r="AM30" t="inlineStr">
         <is>
-          <t>Professional Incentives</t>
+          <t>job title</t>
         </is>
       </c>
       <c r="AN30" t="inlineStr">
         <is>
-          <t>The first factor, labeled "Professional Incentives" was straightforward: the underlying construct is organizational adoption of professional values.</t>
+          <t>For the purposes of this study, the large number of categorical values reported for job title were collapsed into 5 values, ranging from associate member (1) to manager (5).</t>
         </is>
       </c>
       <c r="AO30" t="inlineStr">
         <is>
-          <t>External Com.</t>
+          <t>Internal Com.</t>
         </is>
       </c>
       <c r="AP30" t="n">
-        <v>0.19</v>
+        <v>2.19</v>
       </c>
       <c r="AQ30" t="n">
-        <v>0.12</v>
+        <v>1.02</v>
       </c>
       <c r="AR30" t="n">
         <v>999</v>
       </c>
       <c r="AS30" t="inlineStr">
         <is>
-          <t>Prof. Incent.</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="AT30" t="n">
-        <v>4.08</v>
+        <v>2.94</v>
       </c>
       <c r="AU30" t="n">
-        <v>1.34</v>
+        <v>1.08</v>
       </c>
       <c r="AV30" t="n">
-        <v>0.72</v>
+        <v>999</v>
       </c>
       <c r="AW30" t="n">
-        <v>0.11</v>
+        <v>-0.05</v>
       </c>
       <c r="AX30" t="inlineStr">
         <is>
-          <t>Table 3.9 (p. 65), Row: 19. Prof. Incent., Col: 3, Raw: .11</t>
+          <t>Table 3.9 (p. 65), Row: 7. Status, Col: 2, Raw: -.05</t>
         </is>
       </c>
     </row>
@@ -4333,10 +4333,10 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -4350,7 +4350,7 @@
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -4359,55 +4359,55 @@
         </is>
       </c>
       <c r="V31" t="n">
-        <v>382</v>
+        <v>253</v>
       </c>
       <c r="W31" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X31" t="n">
-        <v>65.2</v>
+        <v>999</v>
       </c>
       <c r="Y31" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>Hotel frontline service employees</t>
+          <t>R&amp;D technical professionals</t>
         </is>
       </c>
       <c r="AA31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>Intraunit communication frequency</t>
+        </is>
+      </c>
+      <c r="AG31" t="inlineStr">
+        <is>
+          <t>Subjects were asked about communication frequency within the last month with every other technical professional in the unit, using a 6-point Likert-type scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day).</t>
+        </is>
+      </c>
+      <c r="AH31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ31" t="n">
         <v>3</v>
       </c>
-      <c r="AB31" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC31" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD31" t="inlineStr">
-        <is>
-          <t>1 = Self-report</t>
-        </is>
-      </c>
-      <c r="AF31" t="inlineStr">
-        <is>
-          <t>Bettencourt et al. (2005)</t>
-        </is>
-      </c>
-      <c r="AG31" t="inlineStr">
-        <is>
-          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
-        </is>
-      </c>
-      <c r="AH31" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI31" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ31" t="n">
-        <v>7</v>
-      </c>
       <c r="AK31" t="inlineStr">
         <is>
           <t>1 = Self-report</t>
@@ -4415,48 +4415,48 @@
       </c>
       <c r="AM31" t="inlineStr">
         <is>
-          <t>Rizzo, House, and Lirtzman (1970)</t>
+          <t>Organizational size</t>
         </is>
       </c>
       <c r="AN31" t="inlineStr">
         <is>
-          <t>For role ambiguity and role conflict, a 6-item scale (3 items each) from Rizzo, House, and Lirtzman (1970) was employed.</t>
+          <t>Organizations were ranked from 1 (small) to 3 (large)</t>
         </is>
       </c>
       <c r="AO31" t="inlineStr">
         <is>
-          <t>External Representation</t>
+          <t>Internal Com.</t>
         </is>
       </c>
       <c r="AP31" t="n">
-        <v>5.46</v>
+        <v>2.19</v>
       </c>
       <c r="AQ31" t="n">
-        <v>0.8</v>
+        <v>1.02</v>
       </c>
       <c r="AR31" t="n">
-        <v>0.871</v>
+        <v>999</v>
       </c>
       <c r="AS31" t="inlineStr">
         <is>
-          <t>Role Conflict</t>
+          <t>Org. Size</t>
         </is>
       </c>
       <c r="AT31" t="n">
-        <v>3.35</v>
+        <v>2.58</v>
       </c>
       <c r="AU31" t="n">
-        <v>0.93</v>
+        <v>0.66</v>
       </c>
       <c r="AV31" t="n">
-        <v>0.619</v>
+        <v>999</v>
       </c>
       <c r="AW31" t="n">
-        <v>-0.368</v>
+        <v>0.11</v>
       </c>
       <c r="AX31" t="inlineStr">
         <is>
-          <t>Table 2 (p. 28), Row: ER, Col: RC, Raw: − 0.368** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+          <t>Table 3.9 (p. 65), Row: 8. Org. Size, Col: 2, Raw: .11</t>
         </is>
       </c>
     </row>
@@ -4467,10 +4467,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -4484,7 +4484,7 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -4493,30 +4493,30 @@
         </is>
       </c>
       <c r="V32" t="n">
-        <v>382</v>
+        <v>253</v>
       </c>
       <c r="W32" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X32" t="n">
-        <v>65.2</v>
+        <v>999</v>
       </c>
       <c r="Y32" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>Hotel frontline service employees</t>
+          <t>R&amp;D technical professionals</t>
         </is>
       </c>
       <c r="AA32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC32" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD32" t="inlineStr">
         <is>
@@ -4525,22 +4525,22 @@
       </c>
       <c r="AF32" t="inlineStr">
         <is>
-          <t>Bettencourt et al. (2005)</t>
+          <t>Intraunit communication frequency</t>
         </is>
       </c>
       <c r="AG32" t="inlineStr">
         <is>
-          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+          <t>Subjects were asked about communication frequency within the last month with every other technical professional in the unit, using a 6-point Likert-type scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day).</t>
         </is>
       </c>
       <c r="AH32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AI32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ32" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AK32" t="inlineStr">
         <is>
@@ -4549,48 +4549,48 @@
       </c>
       <c r="AM32" t="inlineStr">
         <is>
-          <t>Rizzo, House, and Lirtzman (1970)</t>
+          <t>dichotomous variable</t>
         </is>
       </c>
       <c r="AN32" t="inlineStr">
         <is>
-          <t>For role ambiguity and role conflict, a 6-item scale (3 items each) from Rizzo, House, and Lirtzman (1970) was employed.</t>
+          <t>Because the majority of the sample (62 per cent) was engaged in research related to the microelectronics industry, it was decided to create a dichotomous variable to control for structural differences.</t>
         </is>
       </c>
       <c r="AO32" t="inlineStr">
         <is>
-          <t>External Representation</t>
+          <t>Internal Com.</t>
         </is>
       </c>
       <c r="AP32" t="n">
-        <v>5.46</v>
+        <v>2.19</v>
       </c>
       <c r="AQ32" t="n">
-        <v>0.8</v>
+        <v>1.02</v>
       </c>
       <c r="AR32" t="n">
-        <v>0.871</v>
+        <v>999</v>
       </c>
       <c r="AS32" t="inlineStr">
         <is>
-          <t>Role Ambiguity</t>
+          <t>Industry</t>
         </is>
       </c>
       <c r="AT32" t="n">
-        <v>2.86</v>
+        <v>0.62</v>
       </c>
       <c r="AU32" t="n">
-        <v>1.11</v>
+        <v>0.49</v>
       </c>
       <c r="AV32" t="n">
-        <v>0.777</v>
+        <v>999</v>
       </c>
       <c r="AW32" t="n">
-        <v>-0.391</v>
+        <v>0.25</v>
       </c>
       <c r="AX32" t="inlineStr">
         <is>
-          <t>Table 2 (p. 28), Row: ER, Col: RA, Raw: − 0.391** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+          <t>Table 3.9 (p. 65), Row: 9. Industry, Col: 2, Raw: .25**</t>
         </is>
       </c>
     </row>
@@ -4601,10 +4601,10 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="D33" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -4618,7 +4618,7 @@
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4627,30 +4627,30 @@
         </is>
       </c>
       <c r="V33" t="n">
-        <v>382</v>
+        <v>253</v>
       </c>
       <c r="W33" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X33" t="n">
-        <v>65.2</v>
+        <v>999</v>
       </c>
       <c r="Y33" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t>Hotel frontline service employees</t>
+          <t>R&amp;D technical professionals</t>
         </is>
       </c>
       <c r="AA33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC33" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD33" t="inlineStr">
         <is>
@@ -4659,16 +4659,16 @@
       </c>
       <c r="AF33" t="inlineStr">
         <is>
-          <t>Bettencourt et al. (2005)</t>
+          <t>Intraunit communication frequency</t>
         </is>
       </c>
       <c r="AG33" t="inlineStr">
         <is>
-          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+          <t>Subjects were asked about communication frequency within the last month with every other technical professional in the unit, using a 6-point Likert-type scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day).</t>
         </is>
       </c>
       <c r="AH33" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AI33" t="n">
         <v>1</v>
@@ -4683,48 +4683,48 @@
       </c>
       <c r="AM33" t="inlineStr">
         <is>
-          <t>Seibert, Kraimer, and Crant (2001)</t>
+          <t>Organizational Commitment Questionnaire</t>
         </is>
       </c>
       <c r="AN33" t="inlineStr">
         <is>
-          <t>A 3-item scale from Seibert, Kraimer, and Crant (2001) was utilized to assess proactive personality.</t>
+          <t>A 9-item short form was used (Angle &amp; Perry, 1981).</t>
         </is>
       </c>
       <c r="AO33" t="inlineStr">
         <is>
-          <t>External Representation</t>
+          <t>Internal Com.</t>
         </is>
       </c>
       <c r="AP33" t="n">
-        <v>5.46</v>
+        <v>2.19</v>
       </c>
       <c r="AQ33" t="n">
-        <v>0.8</v>
+        <v>1.02</v>
       </c>
       <c r="AR33" t="n">
-        <v>0.871</v>
+        <v>999</v>
       </c>
       <c r="AS33" t="inlineStr">
         <is>
-          <t>Proactive Personality</t>
+          <t>Org. Comm.</t>
         </is>
       </c>
       <c r="AT33" t="n">
-        <v>2.88</v>
+        <v>5.06</v>
       </c>
       <c r="AU33" t="n">
-        <v>1.1</v>
+        <v>1.24</v>
       </c>
       <c r="AV33" t="n">
-        <v>0.894</v>
+        <v>0.92</v>
       </c>
       <c r="AW33" t="n">
-        <v>0.083</v>
+        <v>0.16</v>
       </c>
       <c r="AX33" t="inlineStr">
         <is>
-          <t>Table 2 (p. 28), Row: ER, Col: PP, Raw: 0.083 | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+          <t>Table 3.9 (p. 65), Row: 10. Org. Comm., Col: 2, Raw: .16*</t>
         </is>
       </c>
     </row>
@@ -4735,10 +4735,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="D34" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -4752,7 +4752,7 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4761,30 +4761,30 @@
         </is>
       </c>
       <c r="V34" t="n">
-        <v>382</v>
+        <v>253</v>
       </c>
       <c r="W34" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X34" t="n">
-        <v>65.2</v>
+        <v>999</v>
       </c>
       <c r="Y34" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>Hotel frontline service employees</t>
+          <t>R&amp;D technical professionals</t>
         </is>
       </c>
       <c r="AA34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC34" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD34" t="inlineStr">
         <is>
@@ -4793,16 +4793,16 @@
       </c>
       <c r="AF34" t="inlineStr">
         <is>
-          <t>Bettencourt et al. (2005)</t>
+          <t>Intraunit communication frequency</t>
         </is>
       </c>
       <c r="AG34" t="inlineStr">
         <is>
-          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+          <t>Subjects were asked about communication frequency within the last month with every other technical professional in the unit, using a 6-point Likert-type scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day).</t>
         </is>
       </c>
       <c r="AH34" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="AI34" t="n">
         <v>1</v>
@@ -4817,48 +4817,48 @@
       </c>
       <c r="AM34" t="inlineStr">
         <is>
-          <t>Zhou and George’s (2001) 4-item scale</t>
+          <t>format similar to the OCQ</t>
         </is>
       </c>
       <c r="AN34" t="inlineStr">
         <is>
-          <t>For the measure of employee creativity, Zhou and George’s (2001) 4-item scale from was employed.</t>
+          <t>Both sets of commitment items were measured using a 7-point Likert-type scale from 1=strongly disagree to 7=strongly agree.</t>
         </is>
       </c>
       <c r="AO34" t="inlineStr">
         <is>
-          <t>External Representation</t>
+          <t>Internal Com.</t>
         </is>
       </c>
       <c r="AP34" t="n">
-        <v>5.46</v>
+        <v>2.19</v>
       </c>
       <c r="AQ34" t="n">
-        <v>0.8</v>
+        <v>1.02</v>
       </c>
       <c r="AR34" t="n">
-        <v>0.871</v>
+        <v>999</v>
       </c>
       <c r="AS34" t="inlineStr">
         <is>
-          <t>Employee Creativity</t>
+          <t>Prof. Comm.</t>
         </is>
       </c>
       <c r="AT34" t="n">
-        <v>5.68</v>
+        <v>5.23</v>
       </c>
       <c r="AU34" t="n">
-        <v>0.86</v>
+        <v>1.06</v>
       </c>
       <c r="AV34" t="n">
-        <v>0.839</v>
+        <v>0.9</v>
       </c>
       <c r="AW34" t="n">
-        <v>0.476</v>
+        <v>-0.01</v>
       </c>
       <c r="AX34" t="inlineStr">
         <is>
-          <t>Table 2 (p. 28), Row: ER, Col: EC, Raw: 0.476** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+          <t>Table 3.9 (p. 65), Row: 11. Prof. Comm., Col: 2, Raw: -.01</t>
         </is>
       </c>
     </row>
@@ -4869,57 +4869,57 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="D35" t="n">
+        <v>32</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V35" t="n">
+        <v>253</v>
+      </c>
+      <c r="W35" t="n">
+        <v>38.65</v>
+      </c>
+      <c r="X35" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>R&amp;D technical professionals</t>
+        </is>
+      </c>
+      <c r="AA35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC35" t="n">
         <v>5</v>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>1 = include</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional design</t>
-        </is>
-      </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="U35" t="inlineStr">
-        <is>
-          <t>0 = Domestic</t>
-        </is>
-      </c>
-      <c r="V35" t="n">
-        <v>382</v>
-      </c>
-      <c r="W35" t="n">
-        <v>999</v>
-      </c>
-      <c r="X35" t="n">
-        <v>65.2</v>
-      </c>
-      <c r="Y35" t="n">
-        <v>999</v>
-      </c>
-      <c r="Z35" t="inlineStr">
-        <is>
-          <t>Hotel frontline service employees</t>
-        </is>
-      </c>
-      <c r="AA35" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB35" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC35" t="n">
-        <v>7</v>
-      </c>
       <c r="AD35" t="inlineStr">
         <is>
           <t>1 = Self-report</t>
@@ -4927,22 +4927,22 @@
       </c>
       <c r="AF35" t="inlineStr">
         <is>
-          <t>Bettencourt et al. (2005)</t>
+          <t>Intraunit communication frequency</t>
         </is>
       </c>
       <c r="AG35" t="inlineStr">
         <is>
-          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+          <t>Subjects were asked about communication frequency within the last month with every other technical professional in the unit, using a 6-point Likert-type scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day).</t>
         </is>
       </c>
       <c r="AH35" t="n">
-        <v>3</v>
+        <v>999</v>
       </c>
       <c r="AI35" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="AJ35" t="n">
-        <v>7</v>
+        <v>999</v>
       </c>
       <c r="AK35" t="inlineStr">
         <is>
@@ -4951,48 +4951,48 @@
       </c>
       <c r="AM35" t="inlineStr">
         <is>
-          <t>Rizzo, House, and Lirtzman (1970)</t>
+          <t>interaction variable</t>
         </is>
       </c>
       <c r="AN35" t="inlineStr">
         <is>
-          <t>For role ambiguity and role conflict, a 6-item scale (3 items each) from Rizzo, House, and Lirtzman (1970) was employed.</t>
+          <t>An interaction variable was created from the cross product of organizational commitment and professional commitment mean scale scores.</t>
         </is>
       </c>
       <c r="AO35" t="inlineStr">
         <is>
-          <t>Internal Influence</t>
+          <t>Internal Com.</t>
         </is>
       </c>
       <c r="AP35" t="n">
-        <v>5.63</v>
+        <v>2.19</v>
       </c>
       <c r="AQ35" t="n">
-        <v>0.88</v>
+        <v>1.02</v>
       </c>
       <c r="AR35" t="n">
-        <v>0.872</v>
+        <v>999</v>
       </c>
       <c r="AS35" t="inlineStr">
         <is>
-          <t>Role Conflict</t>
+          <t>Dual Comm.</t>
         </is>
       </c>
       <c r="AT35" t="n">
-        <v>3.35</v>
+        <v>27.07</v>
       </c>
       <c r="AU35" t="n">
-        <v>0.93</v>
+        <v>10.03</v>
       </c>
       <c r="AV35" t="n">
-        <v>0.619</v>
+        <v>999</v>
       </c>
       <c r="AW35" t="n">
-        <v>-0.311</v>
+        <v>-0.09</v>
       </c>
       <c r="AX35" t="inlineStr">
         <is>
-          <t>Table 2 (p. 28), Row: II, Col: RC, Raw: − 0.311** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+          <t>Table 3.9 (p. 65), Row: 12. Dual Comm., Col: 2, Raw: -.09</t>
         </is>
       </c>
     </row>
@@ -5003,10 +5003,10 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="D36" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -5020,7 +5020,7 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -5029,30 +5029,30 @@
         </is>
       </c>
       <c r="V36" t="n">
-        <v>382</v>
+        <v>253</v>
       </c>
       <c r="W36" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X36" t="n">
-        <v>65.2</v>
+        <v>999</v>
       </c>
       <c r="Y36" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>Hotel frontline service employees</t>
+          <t>R&amp;D technical professionals</t>
         </is>
       </c>
       <c r="AA36" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC36" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD36" t="inlineStr">
         <is>
@@ -5061,22 +5061,22 @@
       </c>
       <c r="AF36" t="inlineStr">
         <is>
-          <t>Bettencourt et al. (2005)</t>
+          <t>Intraunit communication frequency</t>
         </is>
       </c>
       <c r="AG36" t="inlineStr">
         <is>
-          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+          <t>Subjects were asked about communication frequency within the last month with every other technical professional in the unit, using a 6-point Likert-type scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day).</t>
         </is>
       </c>
       <c r="AH36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AI36" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="AJ36" t="n">
-        <v>7</v>
+        <v>100</v>
       </c>
       <c r="AK36" t="inlineStr">
         <is>
@@ -5085,48 +5085,48 @@
       </c>
       <c r="AM36" t="inlineStr">
         <is>
-          <t>Rizzo, House, and Lirtzman (1970)</t>
+          <t>weighted sum of the percentages</t>
         </is>
       </c>
       <c r="AN36" t="inlineStr">
         <is>
-          <t>For role ambiguity and role conflict, a 6-item scale (3 items each) from Rizzo, House, and Lirtzman (1970) was employed.</t>
+          <t>Subjects were asked to indicate what percentage of their work falls into each of four categories.</t>
         </is>
       </c>
       <c r="AO36" t="inlineStr">
         <is>
-          <t>Internal Influence</t>
+          <t>Internal Com.</t>
         </is>
       </c>
       <c r="AP36" t="n">
-        <v>5.63</v>
+        <v>2.19</v>
       </c>
       <c r="AQ36" t="n">
-        <v>0.88</v>
+        <v>1.02</v>
       </c>
       <c r="AR36" t="n">
-        <v>0.872</v>
+        <v>999</v>
       </c>
       <c r="AS36" t="inlineStr">
         <is>
-          <t>Role Ambiguity</t>
+          <t>Complexity</t>
         </is>
       </c>
       <c r="AT36" t="n">
-        <v>2.86</v>
+        <v>53.33</v>
       </c>
       <c r="AU36" t="n">
-        <v>1.11</v>
+        <v>14.67</v>
       </c>
       <c r="AV36" t="n">
-        <v>0.777</v>
+        <v>999</v>
       </c>
       <c r="AW36" t="n">
-        <v>-0.368</v>
+        <v>-0.01</v>
       </c>
       <c r="AX36" t="inlineStr">
         <is>
-          <t>Table 2 (p. 28), Row: II, Col: RA, Raw: − 0.368** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+          <t>Table 3.9 (p. 65), Row: 13. Complexity, Col: 2, Raw: -.01</t>
         </is>
       </c>
     </row>
@@ -5137,10 +5137,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="D37" t="n">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -5163,30 +5163,30 @@
         </is>
       </c>
       <c r="V37" t="n">
-        <v>382</v>
+        <v>253</v>
       </c>
       <c r="W37" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X37" t="n">
-        <v>65.2</v>
+        <v>999</v>
       </c>
       <c r="Y37" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z37" t="inlineStr">
         <is>
-          <t>Hotel frontline service employees</t>
+          <t>R&amp;D technical professionals</t>
         </is>
       </c>
       <c r="AA37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC37" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD37" t="inlineStr">
         <is>
@@ -5195,12 +5195,12 @@
       </c>
       <c r="AF37" t="inlineStr">
         <is>
-          <t>Bettencourt et al. (2005)</t>
+          <t>Intraunit communication frequency</t>
         </is>
       </c>
       <c r="AG37" t="inlineStr">
         <is>
-          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+          <t>Subjects were asked about communication frequency within the last month with every other technical professional in the unit, using a 6-point Likert-type scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day).</t>
         </is>
       </c>
       <c r="AH37" t="n">
@@ -5219,48 +5219,48 @@
       </c>
       <c r="AM37" t="inlineStr">
         <is>
-          <t>Seibert, Kraimer, and Crant (2001)</t>
+          <t>three-item scale</t>
         </is>
       </c>
       <c r="AN37" t="inlineStr">
         <is>
-          <t>A 3-item scale from Seibert, Kraimer, and Crant (2001) was utilized to assess proactive personality.</t>
+          <t>A three-item scale was constructed and asked subjects to rate the extent of change of their task requirements on a seven-point scale ranging from 1 (almost no change) to 7 (constantly changing).</t>
         </is>
       </c>
       <c r="AO37" t="inlineStr">
         <is>
-          <t>Internal Influence</t>
+          <t>Internal Com.</t>
         </is>
       </c>
       <c r="AP37" t="n">
-        <v>5.63</v>
+        <v>2.19</v>
       </c>
       <c r="AQ37" t="n">
-        <v>0.88</v>
+        <v>1.02</v>
       </c>
       <c r="AR37" t="n">
-        <v>0.872</v>
+        <v>999</v>
       </c>
       <c r="AS37" t="inlineStr">
         <is>
-          <t>Proactive Personality</t>
+          <t>Uncertainty</t>
         </is>
       </c>
       <c r="AT37" t="n">
-        <v>2.88</v>
+        <v>5.2</v>
       </c>
       <c r="AU37" t="n">
         <v>1.1</v>
       </c>
       <c r="AV37" t="n">
-        <v>0.894</v>
+        <v>0.76</v>
       </c>
       <c r="AW37" t="n">
-        <v>0.049</v>
+        <v>0.14</v>
       </c>
       <c r="AX37" t="inlineStr">
         <is>
-          <t>Table 2 (p. 28), Row: II, Col: PP, Raw: 0.049 | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+          <t>Table 3.9 (p. 65), Row: 14. Uncertainty, Col: 2, Raw: .14*</t>
         </is>
       </c>
     </row>
@@ -5271,10 +5271,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="D38" t="n">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -5288,7 +5288,7 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -5297,48 +5297,48 @@
         </is>
       </c>
       <c r="V38" t="n">
-        <v>382</v>
+        <v>253</v>
       </c>
       <c r="W38" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X38" t="n">
-        <v>65.2</v>
+        <v>999</v>
       </c>
       <c r="Y38" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
-          <t>Hotel frontline service employees</t>
+          <t>R&amp;D technical professionals</t>
         </is>
       </c>
       <c r="AA38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF38" t="inlineStr">
+        <is>
+          <t>Intraunit communication frequency</t>
+        </is>
+      </c>
+      <c r="AG38" t="inlineStr">
+        <is>
+          <t>Subjects were asked about communication frequency within the last month with every other technical professional in the unit, using a 6-point Likert-type scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day).</t>
+        </is>
+      </c>
+      <c r="AH38" t="n">
         <v>3</v>
-      </c>
-      <c r="AB38" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC38" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD38" t="inlineStr">
-        <is>
-          <t>1 = Self-report</t>
-        </is>
-      </c>
-      <c r="AF38" t="inlineStr">
-        <is>
-          <t>Bettencourt et al. (2005)</t>
-        </is>
-      </c>
-      <c r="AG38" t="inlineStr">
-        <is>
-          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
-        </is>
-      </c>
-      <c r="AH38" t="n">
-        <v>4</v>
       </c>
       <c r="AI38" t="n">
         <v>1</v>
@@ -5353,48 +5353,48 @@
       </c>
       <c r="AM38" t="inlineStr">
         <is>
-          <t>Zhou and George’s (2001) 4-item scale</t>
+          <t>Extraproject Coordination scale</t>
         </is>
       </c>
       <c r="AN38" t="inlineStr">
         <is>
-          <t>For the measure of employee creativity, Zhou and George’s (2001) 4-item scale from was employed.</t>
+          <t>The decision was made to delete the intraproject coordination item.</t>
         </is>
       </c>
       <c r="AO38" t="inlineStr">
         <is>
-          <t>Internal Influence</t>
+          <t>Internal Com.</t>
         </is>
       </c>
       <c r="AP38" t="n">
-        <v>5.63</v>
+        <v>2.19</v>
       </c>
       <c r="AQ38" t="n">
-        <v>0.88</v>
+        <v>1.02</v>
       </c>
       <c r="AR38" t="n">
-        <v>0.872</v>
+        <v>999</v>
       </c>
       <c r="AS38" t="inlineStr">
         <is>
-          <t>Employee Creativity</t>
+          <t>Interdepend.</t>
         </is>
       </c>
       <c r="AT38" t="n">
-        <v>5.68</v>
+        <v>3.53</v>
       </c>
       <c r="AU38" t="n">
-        <v>0.86</v>
+        <v>1.36</v>
       </c>
       <c r="AV38" t="n">
-        <v>0.839</v>
+        <v>0.63</v>
       </c>
       <c r="AW38" t="n">
-        <v>0.669</v>
+        <v>0.12</v>
       </c>
       <c r="AX38" t="inlineStr">
         <is>
-          <t>Table 2 (p. 28), Row: II, Col: EC, Raw: 0.669** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+          <t>Table 3.9 (p. 65), Row: 15. Interdepend., Col: 2, Raw: .12*</t>
         </is>
       </c>
     </row>
@@ -5405,10 +5405,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="D39" t="n">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -5422,7 +5422,7 @@
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -5431,30 +5431,30 @@
         </is>
       </c>
       <c r="V39" t="n">
-        <v>382</v>
+        <v>253</v>
       </c>
       <c r="W39" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X39" t="n">
-        <v>65.2</v>
+        <v>999</v>
       </c>
       <c r="Y39" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z39" t="inlineStr">
         <is>
-          <t>Hotel frontline service employees</t>
+          <t>R&amp;D technical professionals</t>
         </is>
       </c>
       <c r="AA39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC39" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD39" t="inlineStr">
         <is>
@@ -5463,22 +5463,22 @@
       </c>
       <c r="AF39" t="inlineStr">
         <is>
-          <t>Bettencourt et al. (2005)</t>
+          <t>Intraunit communication frequency</t>
         </is>
       </c>
       <c r="AG39" t="inlineStr">
         <is>
-          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+          <t>Subjects were asked about communication frequency within the last month with every other technical professional in the unit, using a 6-point Likert-type scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day).</t>
         </is>
       </c>
       <c r="AH39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AI39" t="n">
         <v>1</v>
       </c>
       <c r="AJ39" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AK39" t="inlineStr">
         <is>
@@ -5487,48 +5487,48 @@
       </c>
       <c r="AM39" t="inlineStr">
         <is>
-          <t>Rizzo, House, and Lirtzman (1970)</t>
+          <t>highest degree attained</t>
         </is>
       </c>
       <c r="AN39" t="inlineStr">
         <is>
-          <t>For role ambiguity and role conflict, a 6-item scale (3 items each) from Rizzo, House, and Lirtzman (1970) was employed.</t>
+          <t>In addition, individual variables of highest degree attained and profession were used to indicate the individual's level of professionalization.</t>
         </is>
       </c>
       <c r="AO39" t="inlineStr">
         <is>
-          <t>Service Delivery</t>
+          <t>Internal Com.</t>
         </is>
       </c>
       <c r="AP39" t="n">
-        <v>5.81</v>
+        <v>2.19</v>
       </c>
       <c r="AQ39" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.02</v>
       </c>
       <c r="AR39" t="n">
-        <v>0.876</v>
+        <v>999</v>
       </c>
       <c r="AS39" t="inlineStr">
         <is>
-          <t>Role Conflict</t>
+          <t>Degree</t>
         </is>
       </c>
       <c r="AT39" t="n">
-        <v>3.35</v>
+        <v>2.58</v>
       </c>
       <c r="AU39" t="n">
-        <v>0.93</v>
+        <v>1.17</v>
       </c>
       <c r="AV39" t="n">
-        <v>0.619</v>
+        <v>999</v>
       </c>
       <c r="AW39" t="n">
-        <v>-0.287</v>
+        <v>-0.23</v>
       </c>
       <c r="AX39" t="inlineStr">
         <is>
-          <t>Table 2 (p. 28), Row: SD, Col: RC, Raw: − 0.287** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+          <t>Table 3.9 (p. 65), Row: 16. Degree, Col: 2, Raw: -.23**</t>
         </is>
       </c>
     </row>
@@ -5539,10 +5539,10 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="D40" t="n">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -5556,7 +5556,7 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -5565,55 +5565,55 @@
         </is>
       </c>
       <c r="V40" t="n">
-        <v>382</v>
+        <v>253</v>
       </c>
       <c r="W40" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X40" t="n">
-        <v>65.2</v>
+        <v>999</v>
       </c>
       <c r="Y40" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z40" t="inlineStr">
         <is>
-          <t>Hotel frontline service employees</t>
+          <t>R&amp;D technical professionals</t>
         </is>
       </c>
       <c r="AA40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC40" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF40" t="inlineStr">
+        <is>
+          <t>Intraunit communication frequency</t>
+        </is>
+      </c>
+      <c r="AG40" t="inlineStr">
+        <is>
+          <t>Subjects were asked about communication frequency within the last month with every other technical professional in the unit, using a 6-point Likert-type scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day).</t>
+        </is>
+      </c>
+      <c r="AH40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ40" t="n">
         <v>3</v>
       </c>
-      <c r="AB40" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC40" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD40" t="inlineStr">
-        <is>
-          <t>1 = Self-report</t>
-        </is>
-      </c>
-      <c r="AF40" t="inlineStr">
-        <is>
-          <t>Bettencourt et al. (2005)</t>
-        </is>
-      </c>
-      <c r="AG40" t="inlineStr">
-        <is>
-          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
-        </is>
-      </c>
-      <c r="AH40" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI40" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ40" t="n">
-        <v>7</v>
-      </c>
       <c r="AK40" t="inlineStr">
         <is>
           <t>1 = Self-report</t>
@@ -5621,48 +5621,48 @@
       </c>
       <c r="AM40" t="inlineStr">
         <is>
-          <t>Rizzo, House, and Lirtzman (1970)</t>
+          <t>profession</t>
         </is>
       </c>
       <c r="AN40" t="inlineStr">
         <is>
-          <t>For role ambiguity and role conflict, a 6-item scale (3 items each) from Rizzo, House, and Lirtzman (1970) was employed.</t>
+          <t>In addition, individual variables of highest degree attained and profession were used to indicate the individual's level of professionalization.</t>
         </is>
       </c>
       <c r="AO40" t="inlineStr">
         <is>
-          <t>Service Delivery</t>
+          <t>Internal Com.</t>
         </is>
       </c>
       <c r="AP40" t="n">
-        <v>5.81</v>
+        <v>2.19</v>
       </c>
       <c r="AQ40" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.02</v>
       </c>
       <c r="AR40" t="n">
-        <v>0.876</v>
+        <v>999</v>
       </c>
       <c r="AS40" t="inlineStr">
         <is>
-          <t>Role Ambiguity</t>
+          <t>Occupation</t>
         </is>
       </c>
       <c r="AT40" t="n">
-        <v>2.86</v>
+        <v>1.83</v>
       </c>
       <c r="AU40" t="n">
-        <v>1.11</v>
+        <v>0.54</v>
       </c>
       <c r="AV40" t="n">
-        <v>0.777</v>
+        <v>999</v>
       </c>
       <c r="AW40" t="n">
-        <v>-0.374</v>
+        <v>0.3</v>
       </c>
       <c r="AX40" t="inlineStr">
         <is>
-          <t>Table 2 (p. 28), Row: SD, Col: RA, Raw: − 0.374** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+          <t>Table 3.9 (p. 65), Row: 17. Occupation, Col: 2, Raw: .30**</t>
         </is>
       </c>
     </row>
@@ -5673,10 +5673,10 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="D41" t="n">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -5690,7 +5690,7 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -5699,30 +5699,30 @@
         </is>
       </c>
       <c r="V41" t="n">
-        <v>382</v>
+        <v>253</v>
       </c>
       <c r="W41" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X41" t="n">
-        <v>65.2</v>
+        <v>999</v>
       </c>
       <c r="Y41" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z41" t="inlineStr">
         <is>
-          <t>Hotel frontline service employees</t>
+          <t>R&amp;D technical professionals</t>
         </is>
       </c>
       <c r="AA41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC41" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD41" t="inlineStr">
         <is>
@@ -5731,16 +5731,16 @@
       </c>
       <c r="AF41" t="inlineStr">
         <is>
-          <t>Bettencourt et al. (2005)</t>
+          <t>Intraunit communication frequency</t>
         </is>
       </c>
       <c r="AG41" t="inlineStr">
         <is>
-          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+          <t>Subjects were asked about communication frequency within the last month with every other technical professional in the unit, using a 6-point Likert-type scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day).</t>
         </is>
       </c>
       <c r="AH41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AI41" t="n">
         <v>1</v>
@@ -5755,48 +5755,48 @@
       </c>
       <c r="AM41" t="inlineStr">
         <is>
-          <t>Seibert, Kraimer, and Crant (2001)</t>
+          <t>Professional Control</t>
         </is>
       </c>
       <c r="AN41" t="inlineStr">
         <is>
-          <t>A 3-item scale from Seibert, Kraimer, and Crant (2001) was utilized to assess proactive personality.</t>
+          <t>The estimate of scale reliability for each of these scales was .61 for Professional Control and .32 for Autonomy.</t>
         </is>
       </c>
       <c r="AO41" t="inlineStr">
         <is>
-          <t>Service Delivery</t>
+          <t>Internal Com.</t>
         </is>
       </c>
       <c r="AP41" t="n">
-        <v>5.81</v>
+        <v>2.19</v>
       </c>
       <c r="AQ41" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.02</v>
       </c>
       <c r="AR41" t="n">
-        <v>0.876</v>
+        <v>999</v>
       </c>
       <c r="AS41" t="inlineStr">
         <is>
-          <t>Proactive Personality</t>
+          <t>Prof. Control</t>
         </is>
       </c>
       <c r="AT41" t="n">
-        <v>2.88</v>
+        <v>3.28</v>
       </c>
       <c r="AU41" t="n">
-        <v>1.1</v>
+        <v>1.25</v>
       </c>
       <c r="AV41" t="n">
-        <v>0.894</v>
+        <v>0.61</v>
       </c>
       <c r="AW41" t="n">
-        <v>-0.174</v>
+        <v>-0.1</v>
       </c>
       <c r="AX41" t="inlineStr">
         <is>
-          <t>Table 2 (p. 28), Row: SD, Col: PP, Raw: − 0.174** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+          <t>Table 3.9 (p. 65), Row: 18. Prof. Control, Col: 2, Raw: -.10</t>
         </is>
       </c>
     </row>
@@ -5807,10 +5807,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="D42" t="n">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -5824,7 +5824,7 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5833,48 +5833,48 @@
         </is>
       </c>
       <c r="V42" t="n">
-        <v>382</v>
+        <v>253</v>
       </c>
       <c r="W42" t="n">
-        <v>999</v>
+        <v>38.65</v>
       </c>
       <c r="X42" t="n">
-        <v>65.2</v>
+        <v>999</v>
       </c>
       <c r="Y42" t="n">
-        <v>999</v>
+        <v>0.62</v>
       </c>
       <c r="Z42" t="inlineStr">
         <is>
-          <t>Hotel frontline service employees</t>
+          <t>R&amp;D technical professionals</t>
         </is>
       </c>
       <c r="AA42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC42" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF42" t="inlineStr">
+        <is>
+          <t>Intraunit communication frequency</t>
+        </is>
+      </c>
+      <c r="AG42" t="inlineStr">
+        <is>
+          <t>Subjects were asked about communication frequency within the last month with every other technical professional in the unit, using a 6-point Likert-type scale (0=never, 1=about once a month, 2=less than once a week, 3=about once a week, 4=more than once a week, 5=almost every day).</t>
+        </is>
+      </c>
+      <c r="AH42" t="n">
         <v>3</v>
-      </c>
-      <c r="AB42" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC42" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD42" t="inlineStr">
-        <is>
-          <t>1 = Self-report</t>
-        </is>
-      </c>
-      <c r="AF42" t="inlineStr">
-        <is>
-          <t>Bettencourt et al. (2005)</t>
-        </is>
-      </c>
-      <c r="AG42" t="inlineStr">
-        <is>
-          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
-        </is>
-      </c>
-      <c r="AH42" t="n">
-        <v>4</v>
       </c>
       <c r="AI42" t="n">
         <v>1</v>
@@ -5889,48 +5889,48 @@
       </c>
       <c r="AM42" t="inlineStr">
         <is>
-          <t>Zhou and George’s (2001) 4-item scale</t>
+          <t>Professional Incentives</t>
         </is>
       </c>
       <c r="AN42" t="inlineStr">
         <is>
-          <t>For the measure of employee creativity, Zhou and George’s (2001) 4-item scale from was employed.</t>
+          <t>The first factor, labeled "Professional Incentives" was straightforward: the underlying construct is organizational adoption of professional values.</t>
         </is>
       </c>
       <c r="AO42" t="inlineStr">
         <is>
-          <t>Service Delivery</t>
+          <t>Internal Com.</t>
         </is>
       </c>
       <c r="AP42" t="n">
-        <v>5.81</v>
+        <v>2.19</v>
       </c>
       <c r="AQ42" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.02</v>
       </c>
       <c r="AR42" t="n">
-        <v>0.876</v>
+        <v>999</v>
       </c>
       <c r="AS42" t="inlineStr">
         <is>
-          <t>Employee Creativity</t>
+          <t>Prof. Incent.</t>
         </is>
       </c>
       <c r="AT42" t="n">
-        <v>5.68</v>
+        <v>4.08</v>
       </c>
       <c r="AU42" t="n">
-        <v>0.86</v>
+        <v>1.34</v>
       </c>
       <c r="AV42" t="n">
-        <v>0.839</v>
+        <v>0.72</v>
       </c>
       <c r="AW42" t="n">
-        <v>0.669</v>
+        <v>-0.12</v>
       </c>
       <c r="AX42" t="inlineStr">
         <is>
-          <t>Table 2 (p. 28), Row: SD, Col: EC, Raw: 0.669** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+          <t>Table 3.9 (p. 65), Row: 19. Prof. Incent., Col: 2, Raw: -.12*</t>
         </is>
       </c>
     </row>
@@ -5941,14 +5941,1622 @@
         </is>
       </c>
       <c r="B43" t="n">
+        <v>94</v>
+      </c>
+      <c r="D43" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V43" t="n">
+        <v>382</v>
+      </c>
+      <c r="W43" t="n">
+        <v>999</v>
+      </c>
+      <c r="X43" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="Y43" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>Hotel frontline service employees</t>
+        </is>
+      </c>
+      <c r="AA43" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC43" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF43" t="inlineStr">
+        <is>
+          <t>Bettencourt et al. (2005)</t>
+        </is>
+      </c>
+      <c r="AG43" t="inlineStr">
+        <is>
+          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+        </is>
+      </c>
+      <c r="AH43" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ43" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK43" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM43" t="inlineStr">
+        <is>
+          <t>Rizzo, House, and Lirtzman (1970)</t>
+        </is>
+      </c>
+      <c r="AN43" t="inlineStr">
+        <is>
+          <t>For role ambiguity and role conflict, a 6-item scale (3 items each) from Rizzo, House, and Lirtzman (1970) was employed.</t>
+        </is>
+      </c>
+      <c r="AO43" t="inlineStr">
+        <is>
+          <t>External Representation</t>
+        </is>
+      </c>
+      <c r="AP43" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="AQ43" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AR43" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="AS43" t="inlineStr">
+        <is>
+          <t>Role Conflict</t>
+        </is>
+      </c>
+      <c r="AT43" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="AU43" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="AV43" t="n">
+        <v>0.619</v>
+      </c>
+      <c r="AW43" t="n">
+        <v>-0.368</v>
+      </c>
+      <c r="AX43" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 28), Row: ER, Col: RC, Raw: − 0.368** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>94</v>
+      </c>
+      <c r="D44" t="n">
+        <v>2</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V44" t="n">
+        <v>382</v>
+      </c>
+      <c r="W44" t="n">
+        <v>999</v>
+      </c>
+      <c r="X44" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="Y44" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>Hotel frontline service employees</t>
+        </is>
+      </c>
+      <c r="AA44" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB44" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC44" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF44" t="inlineStr">
+        <is>
+          <t>Bettencourt et al. (2005)</t>
+        </is>
+      </c>
+      <c r="AG44" t="inlineStr">
+        <is>
+          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+        </is>
+      </c>
+      <c r="AH44" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI44" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ44" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK44" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM44" t="inlineStr">
+        <is>
+          <t>Rizzo, House, and Lirtzman (1970)</t>
+        </is>
+      </c>
+      <c r="AN44" t="inlineStr">
+        <is>
+          <t>For role ambiguity and role conflict, a 6-item scale (3 items each) from Rizzo, House, and Lirtzman (1970) was employed.</t>
+        </is>
+      </c>
+      <c r="AO44" t="inlineStr">
+        <is>
+          <t>External Representation</t>
+        </is>
+      </c>
+      <c r="AP44" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="AQ44" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AR44" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="AS44" t="inlineStr">
+        <is>
+          <t>Role Ambiguity</t>
+        </is>
+      </c>
+      <c r="AT44" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="AU44" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="AV44" t="n">
+        <v>0.777</v>
+      </c>
+      <c r="AW44" t="n">
+        <v>-0.391</v>
+      </c>
+      <c r="AX44" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 28), Row: ER, Col: RA, Raw: − 0.391** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>94</v>
+      </c>
+      <c r="D45" t="n">
+        <v>3</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V45" t="n">
+        <v>382</v>
+      </c>
+      <c r="W45" t="n">
+        <v>999</v>
+      </c>
+      <c r="X45" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>Hotel frontline service employees</t>
+        </is>
+      </c>
+      <c r="AA45" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC45" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF45" t="inlineStr">
+        <is>
+          <t>Bettencourt et al. (2005)</t>
+        </is>
+      </c>
+      <c r="AG45" t="inlineStr">
+        <is>
+          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+        </is>
+      </c>
+      <c r="AH45" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ45" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK45" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM45" t="inlineStr">
+        <is>
+          <t>Seibert, Kraimer, and Crant (2001)</t>
+        </is>
+      </c>
+      <c r="AN45" t="inlineStr">
+        <is>
+          <t>A 3-item scale from Seibert, Kraimer, and Crant (2001) was utilized to assess proactive personality.</t>
+        </is>
+      </c>
+      <c r="AO45" t="inlineStr">
+        <is>
+          <t>External Representation</t>
+        </is>
+      </c>
+      <c r="AP45" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="AQ45" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AR45" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="AS45" t="inlineStr">
+        <is>
+          <t>Proactive Personality</t>
+        </is>
+      </c>
+      <c r="AT45" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="AU45" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AV45" t="n">
+        <v>0.894</v>
+      </c>
+      <c r="AW45" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="AX45" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 28), Row: ER, Col: PP, Raw: 0.083 | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>94</v>
+      </c>
+      <c r="D46" t="n">
+        <v>4</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V46" t="n">
+        <v>382</v>
+      </c>
+      <c r="W46" t="n">
+        <v>999</v>
+      </c>
+      <c r="X46" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>Hotel frontline service employees</t>
+        </is>
+      </c>
+      <c r="AA46" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC46" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF46" t="inlineStr">
+        <is>
+          <t>Bettencourt et al. (2005)</t>
+        </is>
+      </c>
+      <c r="AG46" t="inlineStr">
+        <is>
+          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+        </is>
+      </c>
+      <c r="AH46" t="n">
+        <v>4</v>
+      </c>
+      <c r="AI46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ46" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK46" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM46" t="inlineStr">
+        <is>
+          <t>Zhou and George’s (2001) 4-item scale</t>
+        </is>
+      </c>
+      <c r="AN46" t="inlineStr">
+        <is>
+          <t>For the measure of employee creativity, Zhou and George’s (2001) 4-item scale from was employed.</t>
+        </is>
+      </c>
+      <c r="AO46" t="inlineStr">
+        <is>
+          <t>External Representation</t>
+        </is>
+      </c>
+      <c r="AP46" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="AQ46" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AR46" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="AS46" t="inlineStr">
+        <is>
+          <t>Employee Creativity</t>
+        </is>
+      </c>
+      <c r="AT46" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="AU46" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AV46" t="n">
+        <v>0.839</v>
+      </c>
+      <c r="AW46" t="n">
+        <v>0.476</v>
+      </c>
+      <c r="AX46" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 28), Row: ER, Col: EC, Raw: 0.476** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>94</v>
+      </c>
+      <c r="D47" t="n">
+        <v>5</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V47" t="n">
+        <v>382</v>
+      </c>
+      <c r="W47" t="n">
+        <v>999</v>
+      </c>
+      <c r="X47" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>Hotel frontline service employees</t>
+        </is>
+      </c>
+      <c r="AA47" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC47" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF47" t="inlineStr">
+        <is>
+          <t>Bettencourt et al. (2005)</t>
+        </is>
+      </c>
+      <c r="AG47" t="inlineStr">
+        <is>
+          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+        </is>
+      </c>
+      <c r="AH47" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ47" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK47" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM47" t="inlineStr">
+        <is>
+          <t>Rizzo, House, and Lirtzman (1970)</t>
+        </is>
+      </c>
+      <c r="AN47" t="inlineStr">
+        <is>
+          <t>For role ambiguity and role conflict, a 6-item scale (3 items each) from Rizzo, House, and Lirtzman (1970) was employed.</t>
+        </is>
+      </c>
+      <c r="AO47" t="inlineStr">
+        <is>
+          <t>Internal Influence</t>
+        </is>
+      </c>
+      <c r="AP47" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="AQ47" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="AR47" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="AS47" t="inlineStr">
+        <is>
+          <t>Role Conflict</t>
+        </is>
+      </c>
+      <c r="AT47" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="AU47" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="AV47" t="n">
+        <v>0.619</v>
+      </c>
+      <c r="AW47" t="n">
+        <v>-0.311</v>
+      </c>
+      <c r="AX47" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 28), Row: II, Col: RC, Raw: − 0.311** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>94</v>
+      </c>
+      <c r="D48" t="n">
+        <v>6</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V48" t="n">
+        <v>382</v>
+      </c>
+      <c r="W48" t="n">
+        <v>999</v>
+      </c>
+      <c r="X48" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="Y48" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>Hotel frontline service employees</t>
+        </is>
+      </c>
+      <c r="AA48" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC48" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF48" t="inlineStr">
+        <is>
+          <t>Bettencourt et al. (2005)</t>
+        </is>
+      </c>
+      <c r="AG48" t="inlineStr">
+        <is>
+          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+        </is>
+      </c>
+      <c r="AH48" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ48" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK48" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM48" t="inlineStr">
+        <is>
+          <t>Rizzo, House, and Lirtzman (1970)</t>
+        </is>
+      </c>
+      <c r="AN48" t="inlineStr">
+        <is>
+          <t>For role ambiguity and role conflict, a 6-item scale (3 items each) from Rizzo, House, and Lirtzman (1970) was employed.</t>
+        </is>
+      </c>
+      <c r="AO48" t="inlineStr">
+        <is>
+          <t>Internal Influence</t>
+        </is>
+      </c>
+      <c r="AP48" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="AQ48" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="AR48" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="AS48" t="inlineStr">
+        <is>
+          <t>Role Ambiguity</t>
+        </is>
+      </c>
+      <c r="AT48" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="AU48" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="AV48" t="n">
+        <v>0.777</v>
+      </c>
+      <c r="AW48" t="n">
+        <v>-0.368</v>
+      </c>
+      <c r="AX48" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 28), Row: II, Col: RA, Raw: − 0.368** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>94</v>
+      </c>
+      <c r="D49" t="n">
+        <v>7</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V49" t="n">
+        <v>382</v>
+      </c>
+      <c r="W49" t="n">
+        <v>999</v>
+      </c>
+      <c r="X49" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="Y49" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>Hotel frontline service employees</t>
+        </is>
+      </c>
+      <c r="AA49" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB49" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC49" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF49" t="inlineStr">
+        <is>
+          <t>Bettencourt et al. (2005)</t>
+        </is>
+      </c>
+      <c r="AG49" t="inlineStr">
+        <is>
+          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+        </is>
+      </c>
+      <c r="AH49" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI49" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ49" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK49" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM49" t="inlineStr">
+        <is>
+          <t>Seibert, Kraimer, and Crant (2001)</t>
+        </is>
+      </c>
+      <c r="AN49" t="inlineStr">
+        <is>
+          <t>A 3-item scale from Seibert, Kraimer, and Crant (2001) was utilized to assess proactive personality.</t>
+        </is>
+      </c>
+      <c r="AO49" t="inlineStr">
+        <is>
+          <t>Internal Influence</t>
+        </is>
+      </c>
+      <c r="AP49" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="AQ49" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="AR49" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="AS49" t="inlineStr">
+        <is>
+          <t>Proactive Personality</t>
+        </is>
+      </c>
+      <c r="AT49" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="AU49" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AV49" t="n">
+        <v>0.894</v>
+      </c>
+      <c r="AW49" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="AX49" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 28), Row: II, Col: PP, Raw: 0.049 | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>94</v>
+      </c>
+      <c r="D50" t="n">
+        <v>8</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V50" t="n">
+        <v>382</v>
+      </c>
+      <c r="W50" t="n">
+        <v>999</v>
+      </c>
+      <c r="X50" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="Y50" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>Hotel frontline service employees</t>
+        </is>
+      </c>
+      <c r="AA50" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB50" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC50" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF50" t="inlineStr">
+        <is>
+          <t>Bettencourt et al. (2005)</t>
+        </is>
+      </c>
+      <c r="AG50" t="inlineStr">
+        <is>
+          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+        </is>
+      </c>
+      <c r="AH50" t="n">
+        <v>4</v>
+      </c>
+      <c r="AI50" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ50" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK50" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM50" t="inlineStr">
+        <is>
+          <t>Zhou and George’s (2001) 4-item scale</t>
+        </is>
+      </c>
+      <c r="AN50" t="inlineStr">
+        <is>
+          <t>For the measure of employee creativity, Zhou and George’s (2001) 4-item scale from was employed.</t>
+        </is>
+      </c>
+      <c r="AO50" t="inlineStr">
+        <is>
+          <t>Internal Influence</t>
+        </is>
+      </c>
+      <c r="AP50" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="AQ50" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="AR50" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="AS50" t="inlineStr">
+        <is>
+          <t>Employee Creativity</t>
+        </is>
+      </c>
+      <c r="AT50" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="AU50" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AV50" t="n">
+        <v>0.839</v>
+      </c>
+      <c r="AW50" t="n">
+        <v>0.669</v>
+      </c>
+      <c r="AX50" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 28), Row: II, Col: EC, Raw: 0.669** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>94</v>
+      </c>
+      <c r="D51" t="n">
+        <v>9</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V51" t="n">
+        <v>382</v>
+      </c>
+      <c r="W51" t="n">
+        <v>999</v>
+      </c>
+      <c r="X51" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="Y51" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>Hotel frontline service employees</t>
+        </is>
+      </c>
+      <c r="AA51" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB51" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC51" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD51" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF51" t="inlineStr">
+        <is>
+          <t>Bettencourt et al. (2005)</t>
+        </is>
+      </c>
+      <c r="AG51" t="inlineStr">
+        <is>
+          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+        </is>
+      </c>
+      <c r="AH51" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI51" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ51" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK51" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM51" t="inlineStr">
+        <is>
+          <t>Rizzo, House, and Lirtzman (1970)</t>
+        </is>
+      </c>
+      <c r="AN51" t="inlineStr">
+        <is>
+          <t>For role ambiguity and role conflict, a 6-item scale (3 items each) from Rizzo, House, and Lirtzman (1970) was employed.</t>
+        </is>
+      </c>
+      <c r="AO51" t="inlineStr">
+        <is>
+          <t>Service Delivery</t>
+        </is>
+      </c>
+      <c r="AP51" t="n">
+        <v>5.81</v>
+      </c>
+      <c r="AQ51" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="AR51" t="n">
+        <v>0.876</v>
+      </c>
+      <c r="AS51" t="inlineStr">
+        <is>
+          <t>Role Conflict</t>
+        </is>
+      </c>
+      <c r="AT51" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="AU51" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="AV51" t="n">
+        <v>0.619</v>
+      </c>
+      <c r="AW51" t="n">
+        <v>-0.287</v>
+      </c>
+      <c r="AX51" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 28), Row: SD, Col: RC, Raw: − 0.287** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>94</v>
+      </c>
+      <c r="D52" t="n">
+        <v>10</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V52" t="n">
+        <v>382</v>
+      </c>
+      <c r="W52" t="n">
+        <v>999</v>
+      </c>
+      <c r="X52" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="Y52" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z52" t="inlineStr">
+        <is>
+          <t>Hotel frontline service employees</t>
+        </is>
+      </c>
+      <c r="AA52" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC52" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD52" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF52" t="inlineStr">
+        <is>
+          <t>Bettencourt et al. (2005)</t>
+        </is>
+      </c>
+      <c r="AG52" t="inlineStr">
+        <is>
+          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+        </is>
+      </c>
+      <c r="AH52" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ52" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK52" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM52" t="inlineStr">
+        <is>
+          <t>Rizzo, House, and Lirtzman (1970)</t>
+        </is>
+      </c>
+      <c r="AN52" t="inlineStr">
+        <is>
+          <t>For role ambiguity and role conflict, a 6-item scale (3 items each) from Rizzo, House, and Lirtzman (1970) was employed.</t>
+        </is>
+      </c>
+      <c r="AO52" t="inlineStr">
+        <is>
+          <t>Service Delivery</t>
+        </is>
+      </c>
+      <c r="AP52" t="n">
+        <v>5.81</v>
+      </c>
+      <c r="AQ52" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="AR52" t="n">
+        <v>0.876</v>
+      </c>
+      <c r="AS52" t="inlineStr">
+        <is>
+          <t>Role Ambiguity</t>
+        </is>
+      </c>
+      <c r="AT52" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="AU52" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="AV52" t="n">
+        <v>0.777</v>
+      </c>
+      <c r="AW52" t="n">
+        <v>-0.374</v>
+      </c>
+      <c r="AX52" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 28), Row: SD, Col: RA, Raw: − 0.374** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>94</v>
+      </c>
+      <c r="D53" t="n">
+        <v>11</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V53" t="n">
+        <v>382</v>
+      </c>
+      <c r="W53" t="n">
+        <v>999</v>
+      </c>
+      <c r="X53" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="Y53" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>Hotel frontline service employees</t>
+        </is>
+      </c>
+      <c r="AA53" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB53" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC53" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD53" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF53" t="inlineStr">
+        <is>
+          <t>Bettencourt et al. (2005)</t>
+        </is>
+      </c>
+      <c r="AG53" t="inlineStr">
+        <is>
+          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+        </is>
+      </c>
+      <c r="AH53" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI53" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ53" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK53" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM53" t="inlineStr">
+        <is>
+          <t>Seibert, Kraimer, and Crant (2001)</t>
+        </is>
+      </c>
+      <c r="AN53" t="inlineStr">
+        <is>
+          <t>A 3-item scale from Seibert, Kraimer, and Crant (2001) was utilized to assess proactive personality.</t>
+        </is>
+      </c>
+      <c r="AO53" t="inlineStr">
+        <is>
+          <t>Service Delivery</t>
+        </is>
+      </c>
+      <c r="AP53" t="n">
+        <v>5.81</v>
+      </c>
+      <c r="AQ53" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="AR53" t="n">
+        <v>0.876</v>
+      </c>
+      <c r="AS53" t="inlineStr">
+        <is>
+          <t>Proactive Personality</t>
+        </is>
+      </c>
+      <c r="AT53" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="AU53" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AV53" t="n">
+        <v>0.894</v>
+      </c>
+      <c r="AW53" t="n">
+        <v>-0.174</v>
+      </c>
+      <c r="AX53" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 28), Row: SD, Col: PP, Raw: − 0.174** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>94</v>
+      </c>
+      <c r="D54" t="n">
+        <v>12</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V54" t="n">
+        <v>382</v>
+      </c>
+      <c r="W54" t="n">
+        <v>999</v>
+      </c>
+      <c r="X54" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="Y54" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z54" t="inlineStr">
+        <is>
+          <t>Hotel frontline service employees</t>
+        </is>
+      </c>
+      <c r="AA54" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC54" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF54" t="inlineStr">
+        <is>
+          <t>Bettencourt et al. (2005)</t>
+        </is>
+      </c>
+      <c r="AG54" t="inlineStr">
+        <is>
+          <t>For the measure of COBSB, this research used a 9-item scale from Bettencourt et al. (2005); internal influence, external representation, and service delivery were assessed with 3 items each.</t>
+        </is>
+      </c>
+      <c r="AH54" t="n">
+        <v>4</v>
+      </c>
+      <c r="AI54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ54" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK54" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM54" t="inlineStr">
+        <is>
+          <t>Zhou and George’s (2001) 4-item scale</t>
+        </is>
+      </c>
+      <c r="AN54" t="inlineStr">
+        <is>
+          <t>For the measure of employee creativity, Zhou and George’s (2001) 4-item scale from was employed.</t>
+        </is>
+      </c>
+      <c r="AO54" t="inlineStr">
+        <is>
+          <t>Service Delivery</t>
+        </is>
+      </c>
+      <c r="AP54" t="n">
+        <v>5.81</v>
+      </c>
+      <c r="AQ54" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="AR54" t="n">
+        <v>0.876</v>
+      </c>
+      <c r="AS54" t="inlineStr">
+        <is>
+          <t>Employee Creativity</t>
+        </is>
+      </c>
+      <c r="AT54" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="AU54" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AV54" t="n">
+        <v>0.839</v>
+      </c>
+      <c r="AW54" t="n">
+        <v>0.669</v>
+      </c>
+      <c r="AX54" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 28), Row: SD, Col: EC, Raw: 0.669** | Latent correlation: [Table 2 Note] "Inter-construct correlations is shown off the diagonal; square root of average variance extracted (AVE) is shown on the diagonal of the matrix"</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
         <v>109</v>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E55" t="inlineStr">
         <is>
           <t>0 = exclude</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>

</xml_diff>